<commit_message>
Latest inventory updates & sales
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Apr26.xlsx
+++ b/docs/Chiraath-Summary-Apr26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6E7E765-A03C-B54F-A60B-47A125D6EE15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC2697E5-5F0F-7C47-A0F5-3F91032FF39D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2028" uniqueCount="815">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2043" uniqueCount="821">
   <si>
     <t>Notes:</t>
   </si>
@@ -2037,12 +2037,6 @@
     <t>⁠Viscose Chokda</t>
   </si>
   <si>
-    <t>Sreeja -Green:1250</t>
-  </si>
-  <si>
-    <t>Rust orange, burned orange (lotus)</t>
-  </si>
-  <si>
     <t>CHR-136</t>
   </si>
   <si>
@@ -2451,15 +2445,6 @@
     <t>CHR-169</t>
   </si>
   <si>
-    <t>Matka Silk Saree collections</t>
-  </si>
-  <si>
-    <t>Light Lavender/Dark Violet, Bottle Green/Golden Yellow, Maroon/Navy Blue, Navy Blue/Maroon, Purple/Green, Grey/Blue, Peacok Blue/Maroon, Black/Golden Yellow, Navy Blue/Bottle Green</t>
-  </si>
-  <si>
-    <t>Rani Pink, Jet Black, Maroon, Dark Green, navy Blue (2), Off white</t>
-  </si>
-  <si>
     <t>Dark biege with bottle green, Biege Maroon combination, Green</t>
   </si>
   <si>
@@ -2469,9 +2454,6 @@
     <t>Shinoob - 1100, Sruthi - 1100</t>
   </si>
   <si>
-    <t>Blue/bottle green - Saranya Hyd, Blue/red - Jothika, Mustard - Vineetha, Swapna (Thrissur)-1200</t>
-  </si>
-  <si>
     <t>Green Cotton Silk (CHR-88)</t>
   </si>
   <si>
@@ -2481,9 +2463,6 @@
     <t>Yellow Green (CHR-146)</t>
   </si>
   <si>
-    <t>Banarasi Sarees (New design)</t>
-  </si>
-  <si>
     <t>CHR-170</t>
   </si>
   <si>
@@ -2503,6 +2482,52 @@
   </si>
   <si>
     <t>CHR-173</t>
+  </si>
+  <si>
+    <t>Sungudi Saree (Alice Christy inspired)</t>
+  </si>
+  <si>
+    <t>Rani Pink(1), Jet Black(2), Maroon(3), Dark Green(1), navy Blue (2), Off white (1)</t>
+  </si>
+  <si>
+    <t>Matka Silk Saree collections - old design</t>
+  </si>
+  <si>
+    <t>CHR-174</t>
+  </si>
+  <si>
+    <t>Matka Silk Saree collections - new design</t>
+  </si>
+  <si>
+    <t>Blue/bottle green - Saranya Hyd, Blue/red - Jothika, Mustard - Vineetha, Bottle Green/Golden Yellow - Swapna (Thrissur)-1200</t>
+  </si>
+  <si>
+    <t>Bottle Green/Golden Yellow - 2 
+Black/Golden Yellow - 2
+Navy Blue/Bottle Green - 2</t>
+  </si>
+  <si>
+    <t>Peacok Blue/Maroon - 3
+Purple/Green - 1
+Navy Blue/Maroon - 3
+Maroon/Navy Blue - 1
+Lavender/Violet - 1
+Grey/Blue - 1</t>
+  </si>
+  <si>
+    <t>Banarasi Sarees with Paisley motifs</t>
+  </si>
+  <si>
+    <t>Chokda Rust Orange, Dolla</t>
+  </si>
+  <si>
+    <t>Ranju(1000)</t>
+  </si>
+  <si>
+    <t>burned orange (lotus)</t>
+  </si>
+  <si>
+    <t>Sreeja -Green:1250, Ranju - rust orange:1000</t>
   </si>
 </sst>
 </file>
@@ -2514,7 +2539,7 @@
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="166" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2723,6 +2748,12 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Trebuchet MS"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
@@ -3407,7 +3438,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>133</c:v>
+                  <c:v>135</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>76</c:v>
@@ -3510,7 +3541,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>74</c:v>
+                  <c:v>84</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>68</c:v>
@@ -3851,7 +3882,7 @@
                   <c:v>69946</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>55713.23333333333</c:v>
+                  <c:v>61570.593333333331</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1829</c:v>
@@ -4335,7 +4366,7 @@
                   <c:v>16548</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>18170</c:v>
+                  <c:v>20170</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4775,7 +4806,7 @@
                   <c:v>-5624</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-21226</c:v>
+                  <c:v>-19226</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -5248,10 +5279,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>211</c:v>
+                  <c:v>213</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>147</c:v>
+                  <c:v>157</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6438,7 +6469,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>260752</v>
+        <v>262752</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -6455,7 +6486,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>265282</v>
+        <v>267282</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -6472,7 +6503,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-57935</v>
+        <v>-55935</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -6684,15 +6715,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>239803</v>
+        <v>241803</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>86934.716799999995</v>
+        <v>87601.516799999998</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>152868.28320000001</v>
+        <v>154201.48320000002</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -6700,11 +6731,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>15558.257199999993</v>
+        <v>16891.457200000004</v>
       </c>
       <c r="G26" s="19" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹15,558</v>
+        <v>Pay ₹16,891</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -6718,11 +6749,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>86882.566399999996</v>
+        <v>87548.966400000005</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-78463.566399999996</v>
+        <v>-79129.966400000005</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -6730,11 +6761,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-6876.5243999999948</v>
+        <v>-7542.9244000000035</v>
       </c>
       <c r="G27" s="20" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹6,877</v>
+        <v>Receive ₹7,543</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -6748,11 +6779,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>86934.716799999995</v>
+        <v>87601.516799999998</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-74404.716799999995</v>
+        <v>-75071.516799999998</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -6760,11 +6791,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-8681.7327999999834</v>
+        <v>-9348.5327999999863</v>
       </c>
       <c r="G28" s="17" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹8,682</v>
+        <v>Receive ₹9,349</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -6892,7 +6923,7 @@
       </c>
       <c r="E5" s="23">
         <f>Summary!B4</f>
-        <v>260752</v>
+        <v>262752</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -6901,14 +6932,14 @@
       </c>
       <c r="B6" s="23">
         <f>Summary!B6</f>
-        <v>-57935</v>
+        <v>-55935</v>
       </c>
       <c r="D6" s="21" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="23">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>126408.23333333332</v>
+        <v>132265.59333333332</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -6960,7 +6991,7 @@
       </c>
       <c r="G10" s="23">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -6984,7 +7015,7 @@
       </c>
       <c r="G11" s="29">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>147</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -7014,11 +7045,11 @@
       </c>
       <c r="C13" s="29">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$997,"MMM")=$A13)*(YEAR(Sales!$A$2:$A$997)=$B$7)*Sales!$C$2:$C$997),0)</f>
-        <v>18170</v>
+        <v>20170</v>
       </c>
       <c r="D13" s="29">
         <f t="shared" si="0"/>
-        <v>-21226</v>
+        <v>-19226</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1">
@@ -7180,11 +7211,11 @@
       </c>
       <c r="G47" s="32">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H47" s="32">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="J47" s="32" t="s">
         <v>96</v>
@@ -7211,7 +7242,7 @@
       </c>
       <c r="K48" s="33">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>55713.23333333333</v>
+        <v>61570.593333333331</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -8158,7 +8189,7 @@
         <v>1000</v>
       </c>
       <c r="D61" s="41" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="15" customHeight="1">
@@ -13709,7 +13740,7 @@
       <c r="F131" s="50"/>
       <c r="G131" s="50"/>
       <c r="H131" s="52" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="I131" s="50" t="s">
         <v>139</v>
@@ -13920,7 +13951,7 @@
         <v>46113</v>
       </c>
       <c r="B140" s="54" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="C140" s="55">
         <v>3000</v>
@@ -13934,7 +13965,7 @@
       <c r="F140" s="57"/>
       <c r="G140" s="57"/>
       <c r="H140" s="58" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="I140" s="54" t="s">
         <v>139</v>
@@ -13959,7 +13990,7 @@
       <c r="F141" s="50"/>
       <c r="G141" s="50"/>
       <c r="H141" s="52" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="I141" s="50" t="s">
         <v>139</v>
@@ -13970,7 +14001,7 @@
         <v>46119</v>
       </c>
       <c r="B142" s="54" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="C142" s="55">
         <v>1200</v>
@@ -13984,7 +14015,7 @@
       <c r="F142" s="57"/>
       <c r="G142" s="57"/>
       <c r="H142" s="58" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="I142" s="54" t="s">
         <v>139</v>
@@ -13995,7 +14026,7 @@
         <v>46120</v>
       </c>
       <c r="B143" s="50" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="C143" s="51">
         <v>1200</v>
@@ -14009,7 +14040,7 @@
       <c r="F143" s="50"/>
       <c r="G143" s="50"/>
       <c r="H143" s="52" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="I143" s="50" t="s">
         <v>139</v>
@@ -14020,7 +14051,7 @@
         <v>46120</v>
       </c>
       <c r="B144" s="54" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="C144" s="55">
         <v>1500</v>
@@ -14034,7 +14065,7 @@
       <c r="F144" s="57"/>
       <c r="G144" s="57"/>
       <c r="H144" s="58" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="I144" s="54" t="s">
         <v>139</v>
@@ -14059,7 +14090,7 @@
       <c r="F145" s="50"/>
       <c r="G145" s="50"/>
       <c r="H145" s="52" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="I145" s="50" t="s">
         <v>139</v>
@@ -14082,7 +14113,7 @@
       <c r="F146" s="57"/>
       <c r="G146" s="57"/>
       <c r="H146" s="58" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="I146" s="54" t="s">
         <v>311</v>
@@ -14093,7 +14124,7 @@
         <v>46122</v>
       </c>
       <c r="B147" s="50" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
       <c r="C147" s="51">
         <v>650</v>
@@ -14107,7 +14138,7 @@
       <c r="F147" s="50"/>
       <c r="G147" s="50"/>
       <c r="H147" s="52" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
       <c r="I147" s="50" t="s">
         <v>139</v>
@@ -14118,7 +14149,7 @@
         <v>46122</v>
       </c>
       <c r="B148" s="54" t="s">
-        <v>794</v>
+        <v>792</v>
       </c>
       <c r="C148" s="55">
         <v>500</v>
@@ -14132,7 +14163,7 @@
       <c r="F148" s="57"/>
       <c r="G148" s="57"/>
       <c r="H148" s="58" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="I148" s="54" t="s">
         <v>139</v>
@@ -14155,7 +14186,7 @@
       <c r="F149" s="50"/>
       <c r="G149" s="50"/>
       <c r="H149" s="52" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="I149" s="50" t="s">
         <v>311</v>
@@ -14180,7 +14211,7 @@
       <c r="F150" s="57"/>
       <c r="G150" s="57"/>
       <c r="H150" s="58" t="s">
-        <v>804</v>
+        <v>798</v>
       </c>
       <c r="I150" s="54" t="s">
         <v>139</v>
@@ -14191,7 +14222,7 @@
         <v>46125</v>
       </c>
       <c r="B151" s="50" t="s">
-        <v>805</v>
+        <v>799</v>
       </c>
       <c r="C151" s="51">
         <v>1200</v>
@@ -14205,7 +14236,7 @@
       <c r="F151" s="50"/>
       <c r="G151" s="50"/>
       <c r="H151" s="52" t="s">
-        <v>806</v>
+        <v>800</v>
       </c>
       <c r="I151" s="50" t="s">
         <v>139</v>
@@ -14230,7 +14261,7 @@
       <c r="F152" s="57"/>
       <c r="G152" s="57"/>
       <c r="H152" s="58" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="I152" s="54" t="s">
         <v>139</v>
@@ -14255,22 +14286,36 @@
       <c r="F153" s="50"/>
       <c r="G153" s="50"/>
       <c r="H153" s="52" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="I153" s="50" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="154" spans="1:9">
-      <c r="A154" s="53"/>
-      <c r="B154" s="54"/>
-      <c r="C154" s="55"/>
-      <c r="D154" s="54"/>
-      <c r="E154" s="54"/>
+    <row r="154" spans="1:9" ht="16">
+      <c r="A154" s="53">
+        <v>46126</v>
+      </c>
+      <c r="B154" s="54" t="s">
+        <v>190</v>
+      </c>
+      <c r="C154" s="55">
+        <v>2000</v>
+      </c>
+      <c r="D154" s="54" t="s">
+        <v>141</v>
+      </c>
+      <c r="E154" s="54" t="s">
+        <v>49</v>
+      </c>
       <c r="F154" s="57"/>
       <c r="G154" s="57"/>
-      <c r="H154" s="58"/>
-      <c r="I154" s="54"/>
+      <c r="H154" s="58" t="s">
+        <v>817</v>
+      </c>
+      <c r="I154" s="54" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="155" spans="1:9">
       <c r="A155" s="49"/>
@@ -22546,7 +22591,7 @@
         <v>685</v>
       </c>
       <c r="L68" s="83" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="M68" s="83"/>
       <c r="N68" s="83" t="s">
@@ -22704,7 +22749,7 @@
         <v>0</v>
       </c>
       <c r="L71" s="78" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
       <c r="M71" s="78" t="s">
         <v>49</v>
@@ -22714,7 +22759,7 @@
       </c>
       <c r="O71" s="78"/>
       <c r="P71" s="78" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="Q71" s="78"/>
       <c r="R71" s="78"/>
@@ -23666,7 +23711,7 @@
         <v>0</v>
       </c>
       <c r="L89" s="78" t="s">
-        <v>802</v>
+        <v>797</v>
       </c>
       <c r="M89" s="78"/>
       <c r="N89" s="78" t="s">
@@ -25046,7 +25091,7 @@
         <v>0</v>
       </c>
       <c r="L115" s="78" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="M115" s="78"/>
       <c r="N115" s="78" t="s">
@@ -25291,11 +25336,11 @@
         <v>3</v>
       </c>
       <c r="G120" s="84">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H120" s="83">
         <f t="shared" si="9"/>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I120" s="83">
         <f>IF(D120&lt;&gt;"",D120,IFERROR(E120/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -25307,7 +25352,7 @@
       </c>
       <c r="K120" s="83">
         <f t="shared" si="11"/>
-        <v>2932.6733333333309</v>
+        <v>4189.5333333333301</v>
       </c>
       <c r="L120" s="83" t="s">
         <v>613</v>
@@ -25320,7 +25365,7 @@
       </c>
       <c r="O120" s="83"/>
       <c r="P120" s="83" t="s">
-        <v>799</v>
+        <v>809</v>
       </c>
       <c r="Q120" s="83"/>
       <c r="R120" s="83"/>
@@ -26500,10 +26545,10 @@
         <v>1550</v>
       </c>
       <c r="F130" s="92">
+        <v>1</v>
+      </c>
+      <c r="G130" s="92">
         <v>0</v>
-      </c>
-      <c r="G130" s="92">
-        <v>1</v>
       </c>
       <c r="H130" s="91">
         <f t="shared" ref="H130:H161" si="12">F130+IF(LEN(G130)=0,0,G130)</f>
@@ -26515,16 +26560,18 @@
       </c>
       <c r="J130" s="91">
         <f t="shared" ref="J130:J161" si="13">F130*I130</f>
-        <v>0</v>
+        <v>755</v>
       </c>
       <c r="K130" s="91">
         <f t="shared" ref="K130:K163" si="14">IF(LEN(G130)=0,0,G130)*I130</f>
-        <v>755</v>
-      </c>
-      <c r="L130" s="83"/>
+        <v>0</v>
+      </c>
+      <c r="L130" s="83" t="s">
+        <v>818</v>
+      </c>
       <c r="M130" s="83"/>
       <c r="N130" s="83" t="s">
-        <v>506</v>
+        <v>337</v>
       </c>
       <c r="O130" s="83"/>
       <c r="P130" s="83"/>
@@ -26804,10 +26851,10 @@
         <v>1250</v>
       </c>
       <c r="F136" s="92">
+        <v>2</v>
+      </c>
+      <c r="G136" s="92">
         <v>1</v>
-      </c>
-      <c r="G136" s="92">
-        <v>2</v>
       </c>
       <c r="H136" s="91">
         <f t="shared" si="12"/>
@@ -26819,14 +26866,14 @@
       </c>
       <c r="J136" s="91">
         <f t="shared" si="13"/>
-        <v>908</v>
+        <v>1816</v>
       </c>
       <c r="K136" s="91">
         <f t="shared" si="14"/>
-        <v>1816</v>
+        <v>908</v>
       </c>
       <c r="L136" s="83" t="s">
-        <v>659</v>
+        <v>820</v>
       </c>
       <c r="M136" s="83"/>
       <c r="N136" s="83" t="s">
@@ -26834,7 +26881,7 @@
       </c>
       <c r="O136" s="83"/>
       <c r="P136" s="83" t="s">
-        <v>660</v>
+        <v>819</v>
       </c>
       <c r="Q136" s="83"/>
       <c r="R136" s="83"/>
@@ -26843,10 +26890,10 @@
     </row>
     <row r="137" spans="1:20" ht="15">
       <c r="A137" s="89" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="B137" s="78" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="C137" s="78" t="s">
         <v>95</v>
@@ -26895,10 +26942,10 @@
     </row>
     <row r="138" spans="1:20" ht="15">
       <c r="A138" s="91" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="B138" s="83" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="C138" s="83" t="s">
         <v>95</v>
@@ -26945,10 +26992,10 @@
     </row>
     <row r="139" spans="1:20" ht="15">
       <c r="A139" s="89" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="B139" s="78" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="C139" s="78" t="s">
         <v>95</v>
@@ -26997,10 +27044,10 @@
     </row>
     <row r="140" spans="1:20" ht="15">
       <c r="A140" s="91" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="B140" s="83" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="C140" s="83" t="s">
         <v>95</v>
@@ -27034,7 +27081,7 @@
         <v>699</v>
       </c>
       <c r="L140" s="83" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="M140" s="83"/>
       <c r="N140" s="83" t="s">
@@ -27049,10 +27096,10 @@
     </row>
     <row r="141" spans="1:20" ht="15">
       <c r="A141" s="89" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="B141" s="78" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="C141" s="78" t="s">
         <v>95</v>
@@ -27099,10 +27146,10 @@
     </row>
     <row r="142" spans="1:20" ht="15">
       <c r="A142" s="83" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="B142" s="83" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="C142" s="83" t="s">
         <v>95</v>
@@ -27136,7 +27183,7 @@
         <v>600</v>
       </c>
       <c r="L142" s="83" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="M142" s="83"/>
       <c r="N142" s="83" t="s">
@@ -27153,10 +27200,10 @@
     </row>
     <row r="143" spans="1:20" ht="15">
       <c r="A143" s="78" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="B143" s="78" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="C143" s="78" t="s">
         <v>95</v>
@@ -27203,10 +27250,10 @@
     </row>
     <row r="144" spans="1:20" ht="15">
       <c r="A144" s="83" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="B144" s="83" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="C144" s="83" t="s">
         <v>95</v>
@@ -27253,7 +27300,7 @@
     </row>
     <row r="145" spans="1:20" ht="15">
       <c r="A145" s="78" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="B145" s="78" t="s">
         <v>293</v>
@@ -27305,10 +27352,10 @@
     </row>
     <row r="146" spans="1:20" ht="15">
       <c r="A146" s="83" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="B146" s="83" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="C146" s="83" t="s">
         <v>95</v>
@@ -27342,7 +27389,7 @@
         <v>1522</v>
       </c>
       <c r="L146" s="83" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="M146" s="83"/>
       <c r="N146" s="83" t="s">
@@ -27355,12 +27402,12 @@
       <c r="S146" s="83"/>
       <c r="T146" s="83"/>
     </row>
-    <row r="147" spans="1:20" ht="75">
+    <row r="147" spans="1:20" ht="45">
       <c r="A147" s="78" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="B147" s="78" t="s">
-        <v>797</v>
+        <v>810</v>
       </c>
       <c r="C147" s="78" t="s">
         <v>95</v>
@@ -27375,11 +27422,11 @@
         <v>4</v>
       </c>
       <c r="G147" s="90">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H147" s="89">
         <f t="shared" si="12"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I147" s="89">
         <f>IF(D147&lt;&gt;"",D147,IFERROR(E147/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -27391,10 +27438,10 @@
       </c>
       <c r="K147" s="89">
         <f t="shared" si="14"/>
-        <v>5752</v>
+        <v>5033</v>
       </c>
       <c r="L147" s="78" t="s">
-        <v>803</v>
+        <v>813</v>
       </c>
       <c r="M147" s="78"/>
       <c r="N147" s="78" t="s">
@@ -27402,7 +27449,7 @@
       </c>
       <c r="O147" s="78"/>
       <c r="P147" s="78" t="s">
-        <v>798</v>
+        <v>814</v>
       </c>
       <c r="Q147" s="78"/>
       <c r="R147" s="78"/>
@@ -27411,10 +27458,10 @@
     </row>
     <row r="148" spans="1:20" ht="15">
       <c r="A148" s="83" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B148" s="83" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="C148" s="83" t="s">
         <v>95</v>
@@ -27448,7 +27495,7 @@
         <v>502</v>
       </c>
       <c r="L148" s="83" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="M148" s="83"/>
       <c r="N148" s="83" t="s">
@@ -27463,10 +27510,10 @@
     </row>
     <row r="149" spans="1:20" ht="15">
       <c r="A149" s="78" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="B149" s="78" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="C149" s="78" t="s">
         <v>95</v>
@@ -27500,7 +27547,7 @@
         <v>2048</v>
       </c>
       <c r="L149" s="78" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="M149" s="78"/>
       <c r="N149" s="78" t="s">
@@ -27515,10 +27562,10 @@
     </row>
     <row r="150" spans="1:20" ht="15">
       <c r="A150" s="83" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="B150" s="83" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="C150" s="83" t="s">
         <v>95</v>
@@ -27565,10 +27612,10 @@
     </row>
     <row r="151" spans="1:20" ht="15">
       <c r="A151" s="78" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="B151" s="78" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="C151" s="78" t="s">
         <v>96</v>
@@ -27602,17 +27649,17 @@
         <v>1290</v>
       </c>
       <c r="L151" s="78" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="M151" s="78"/>
       <c r="N151" s="78" t="s">
         <v>422</v>
       </c>
       <c r="O151" s="78" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="P151" s="78" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="Q151" s="78"/>
       <c r="R151" s="78"/>
@@ -27621,10 +27668,10 @@
     </row>
     <row r="152" spans="1:20" ht="15">
       <c r="A152" s="83" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="B152" s="83" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="C152" s="83" t="s">
         <v>97</v>
@@ -27658,17 +27705,17 @@
         <v>885</v>
       </c>
       <c r="L152" s="83" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="M152" s="83"/>
       <c r="N152" s="83" t="s">
         <v>422</v>
       </c>
       <c r="O152" s="83" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="P152" s="83" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="Q152" s="83"/>
       <c r="R152" s="83"/>
@@ -27677,10 +27724,10 @@
     </row>
     <row r="153" spans="1:20" ht="15">
       <c r="A153" s="78" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="B153" s="78" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="C153" s="78" t="s">
         <v>95</v>
@@ -27714,7 +27761,7 @@
         <v>891.5</v>
       </c>
       <c r="L153" s="78" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="M153" s="78"/>
       <c r="N153" s="78" t="s">
@@ -27722,7 +27769,7 @@
       </c>
       <c r="O153" s="78"/>
       <c r="P153" s="78" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="Q153" s="78"/>
       <c r="R153" s="78"/>
@@ -27731,10 +27778,10 @@
     </row>
     <row r="154" spans="1:20" ht="15">
       <c r="A154" s="83" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="B154" s="83" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="C154" s="83" t="s">
         <v>96</v>
@@ -27773,7 +27820,7 @@
         <v>506</v>
       </c>
       <c r="O154" s="83" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="P154" s="83"/>
       <c r="Q154" s="83"/>
@@ -27783,10 +27830,10 @@
     </row>
     <row r="155" spans="1:20" ht="15">
       <c r="A155" s="78" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="B155" s="78" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="C155" s="78" t="s">
         <v>96</v>
@@ -27825,7 +27872,7 @@
         <v>506</v>
       </c>
       <c r="O155" s="78" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="P155" s="78"/>
       <c r="Q155" s="78"/>
@@ -27835,10 +27882,10 @@
     </row>
     <row r="156" spans="1:20" ht="15">
       <c r="A156" s="83" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="B156" s="83" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="C156" s="83" t="s">
         <v>96</v>
@@ -27877,7 +27924,7 @@
         <v>506</v>
       </c>
       <c r="O156" s="83" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="P156" s="83"/>
       <c r="Q156" s="83"/>
@@ -27887,10 +27934,10 @@
     </row>
     <row r="157" spans="1:20" ht="15">
       <c r="A157" s="78" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="B157" s="78" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="C157" s="78" t="s">
         <v>96</v>
@@ -27924,7 +27971,7 @@
         <v>1575</v>
       </c>
       <c r="L157" s="78" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="M157" s="78"/>
       <c r="N157" s="78" t="s">
@@ -27941,10 +27988,10 @@
     </row>
     <row r="158" spans="1:20" ht="15">
       <c r="A158" s="83" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="B158" s="83" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="C158" s="83" t="s">
         <v>96</v>
@@ -27983,7 +28030,7 @@
         <v>506</v>
       </c>
       <c r="O158" s="83" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="P158" s="83"/>
       <c r="Q158" s="83"/>
@@ -27993,10 +28040,10 @@
     </row>
     <row r="159" spans="1:20" ht="15">
       <c r="A159" s="78" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="B159" s="78" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="C159" s="78" t="s">
         <v>96</v>
@@ -28035,7 +28082,7 @@
         <v>506</v>
       </c>
       <c r="O159" s="78" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="P159" s="78"/>
       <c r="Q159" s="78"/>
@@ -28045,10 +28092,10 @@
     </row>
     <row r="160" spans="1:20" ht="15">
       <c r="A160" s="83" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="B160" s="83" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="C160" s="83" t="s">
         <v>95</v>
@@ -28097,10 +28144,10 @@
     </row>
     <row r="161" spans="1:20" ht="15">
       <c r="A161" s="78" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="B161" s="78" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="C161" s="78" t="s">
         <v>95</v>
@@ -28149,10 +28196,10 @@
     </row>
     <row r="162" spans="1:20" ht="15">
       <c r="A162" s="83" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="B162" s="83" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="C162" s="83" t="s">
         <v>95</v>
@@ -28199,10 +28246,10 @@
     </row>
     <row r="163" spans="1:20" ht="15">
       <c r="A163" s="78" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="B163" s="78" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="C163" s="78" t="s">
         <v>95</v>
@@ -28249,10 +28296,10 @@
     </row>
     <row r="164" spans="1:20" ht="60">
       <c r="A164" s="83" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="B164" s="83" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="C164" s="83" t="s">
         <v>95</v>
@@ -28292,7 +28339,7 @@
       </c>
       <c r="O164" s="83"/>
       <c r="P164" s="83" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="Q164" s="83"/>
       <c r="R164" s="83"/>
@@ -28301,10 +28348,10 @@
     </row>
     <row r="165" spans="1:20" ht="15">
       <c r="A165" s="78" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="B165" s="78" t="s">
-        <v>771</v>
+        <v>808</v>
       </c>
       <c r="C165" s="78" t="s">
         <v>95</v>
@@ -28346,7 +28393,7 @@
       </c>
       <c r="O165" s="78"/>
       <c r="P165" s="78" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="Q165" s="78"/>
       <c r="R165" s="78"/>
@@ -28355,10 +28402,10 @@
     </row>
     <row r="166" spans="1:20" ht="15">
       <c r="A166" s="83" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="B166" s="83" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="C166" s="83" t="s">
         <v>95</v>
@@ -28398,7 +28445,7 @@
       </c>
       <c r="O166" s="83"/>
       <c r="P166" s="83" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="Q166" s="83"/>
       <c r="R166" s="83"/>
@@ -28407,10 +28454,10 @@
     </row>
     <row r="167" spans="1:20" ht="15">
       <c r="A167" s="78" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="B167" s="78" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="C167" s="78" t="s">
         <v>95</v>
@@ -28444,7 +28491,7 @@
         <v>2220</v>
       </c>
       <c r="L167" s="78" t="s">
-        <v>801</v>
+        <v>796</v>
       </c>
       <c r="M167" s="78"/>
       <c r="N167" s="78" t="s">
@@ -28452,7 +28499,7 @@
       </c>
       <c r="O167" s="78"/>
       <c r="P167" s="78" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="Q167" s="78"/>
       <c r="R167" s="78"/>
@@ -28461,10 +28508,10 @@
     </row>
     <row r="168" spans="1:20" ht="15">
       <c r="A168" s="83" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B168" s="83" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
       <c r="C168" s="83" t="s">
         <v>95</v>
@@ -28504,7 +28551,7 @@
       </c>
       <c r="O168" s="83"/>
       <c r="P168" s="83" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="Q168" s="83"/>
       <c r="R168" s="83"/>
@@ -28513,10 +28560,10 @@
     </row>
     <row r="169" spans="1:20" ht="15">
       <c r="A169" s="78" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="B169" s="78" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="C169" s="78" t="s">
         <v>95</v>
@@ -28556,7 +28603,7 @@
       </c>
       <c r="O169" s="78"/>
       <c r="P169" s="78" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
       <c r="Q169" s="78"/>
       <c r="R169" s="78"/>
@@ -28565,10 +28612,10 @@
     </row>
     <row r="170" spans="1:20" ht="30">
       <c r="A170" s="83" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
       <c r="B170" s="83" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
       <c r="C170" s="83" t="s">
         <v>95</v>
@@ -28608,7 +28655,7 @@
       </c>
       <c r="O170" s="83"/>
       <c r="P170" s="83" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="Q170" s="83"/>
       <c r="R170" s="83"/>
@@ -28617,10 +28664,10 @@
     </row>
     <row r="171" spans="1:20" ht="15">
       <c r="A171" s="78" t="s">
-        <v>808</v>
+        <v>801</v>
       </c>
       <c r="B171" s="83" t="s">
-        <v>807</v>
+        <v>816</v>
       </c>
       <c r="C171" s="78" t="s">
         <v>95</v>
@@ -28655,7 +28702,9 @@
       </c>
       <c r="L171" s="78"/>
       <c r="M171" s="78"/>
-      <c r="N171" s="78"/>
+      <c r="N171" s="78" t="s">
+        <v>506</v>
+      </c>
       <c r="O171" s="78"/>
       <c r="P171" s="78"/>
       <c r="Q171" s="78"/>
@@ -28665,10 +28714,10 @@
     </row>
     <row r="172" spans="1:20" ht="15">
       <c r="A172" s="83" t="s">
-        <v>810</v>
+        <v>803</v>
       </c>
       <c r="B172" s="83" t="s">
-        <v>809</v>
+        <v>802</v>
       </c>
       <c r="C172" s="83" t="s">
         <v>95</v>
@@ -28703,7 +28752,9 @@
       </c>
       <c r="L172" s="83"/>
       <c r="M172" s="83"/>
-      <c r="N172" s="83"/>
+      <c r="N172" s="83" t="s">
+        <v>506</v>
+      </c>
       <c r="O172" s="83"/>
       <c r="P172" s="83"/>
       <c r="Q172" s="83"/>
@@ -28713,16 +28764,16 @@
     </row>
     <row r="173" spans="1:20" ht="15">
       <c r="A173" s="78" t="s">
-        <v>813</v>
+        <v>806</v>
       </c>
       <c r="B173" s="78" t="s">
-        <v>811</v>
+        <v>804</v>
       </c>
       <c r="C173" s="78" t="s">
         <v>95</v>
       </c>
       <c r="D173" s="85">
-        <v>791.7</v>
+        <v>803.26</v>
       </c>
       <c r="E173" s="85">
         <v>1250</v>
@@ -28739,7 +28790,7 @@
       </c>
       <c r="I173" s="89">
         <f>IF(D173&lt;&gt;"",D173,IFERROR(E173/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>791.7</v>
+        <v>803.26</v>
       </c>
       <c r="J173" s="89">
         <f t="shared" si="27"/>
@@ -28747,11 +28798,13 @@
       </c>
       <c r="K173" s="89">
         <f t="shared" si="28"/>
-        <v>791.7</v>
+        <v>803.26</v>
       </c>
       <c r="L173" s="78"/>
       <c r="M173" s="78"/>
-      <c r="N173" s="78"/>
+      <c r="N173" s="78" t="s">
+        <v>506</v>
+      </c>
       <c r="O173" s="78"/>
       <c r="P173" s="78"/>
       <c r="Q173" s="78"/>
@@ -28761,16 +28814,16 @@
     </row>
     <row r="174" spans="1:20" ht="15">
       <c r="A174" s="83" t="s">
-        <v>814</v>
+        <v>807</v>
       </c>
       <c r="B174" s="83" t="s">
-        <v>812</v>
+        <v>805</v>
       </c>
       <c r="C174" s="83" t="s">
         <v>95</v>
       </c>
       <c r="D174" s="84">
-        <v>803.26</v>
+        <v>791.7</v>
       </c>
       <c r="E174" s="84">
         <v>1250</v>
@@ -28787,7 +28840,7 @@
       </c>
       <c r="I174" s="91">
         <f>IF(D174&lt;&gt;"",D174,IFERROR(E174/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>803.26</v>
+        <v>791.7</v>
       </c>
       <c r="J174" s="91">
         <f t="shared" si="27"/>
@@ -28795,11 +28848,13 @@
       </c>
       <c r="K174" s="91">
         <f t="shared" si="28"/>
-        <v>803.26</v>
+        <v>791.7</v>
       </c>
       <c r="L174" s="83"/>
       <c r="M174" s="83"/>
-      <c r="N174" s="83"/>
+      <c r="N174" s="83" t="s">
+        <v>506</v>
+      </c>
       <c r="O174" s="83"/>
       <c r="P174" s="83"/>
       <c r="Q174" s="83"/>
@@ -28807,75 +28862,375 @@
       <c r="S174" s="83"/>
       <c r="T174" s="83"/>
     </row>
-    <row r="175" spans="1:20">
-      <c r="S175" s="62"/>
-      <c r="T175" s="62"/>
-    </row>
-    <row r="176" spans="1:20">
-      <c r="S176" s="62"/>
-      <c r="T176" s="62"/>
-    </row>
-    <row r="177" spans="19:20">
-      <c r="S177" s="62"/>
-      <c r="T177" s="62"/>
-    </row>
-    <row r="178" spans="19:20">
-      <c r="S178" s="62"/>
-      <c r="T178" s="62"/>
-    </row>
-    <row r="179" spans="19:20">
-      <c r="S179" s="62"/>
-      <c r="T179" s="62"/>
-    </row>
-    <row r="180" spans="19:20">
-      <c r="S180" s="62"/>
-      <c r="T180" s="62"/>
-    </row>
-    <row r="181" spans="19:20">
-      <c r="S181" s="62"/>
-      <c r="T181" s="62"/>
-    </row>
-    <row r="182" spans="19:20">
-      <c r="S182" s="62"/>
-      <c r="T182" s="62"/>
-    </row>
-    <row r="183" spans="19:20">
-      <c r="S183" s="62"/>
-      <c r="T183" s="62"/>
-    </row>
-    <row r="184" spans="19:20">
-      <c r="S184" s="62"/>
-      <c r="T184" s="62"/>
-    </row>
-    <row r="185" spans="19:20">
-      <c r="S185" s="62"/>
-      <c r="T185" s="62"/>
-    </row>
-    <row r="186" spans="19:20">
-      <c r="S186" s="62"/>
-      <c r="T186" s="62"/>
-    </row>
-    <row r="187" spans="19:20">
-      <c r="S187" s="62"/>
-      <c r="T187" s="62"/>
-    </row>
-    <row r="188" spans="19:20">
-      <c r="S188" s="62"/>
-      <c r="T188" s="62"/>
-    </row>
-    <row r="189" spans="19:20">
-      <c r="S189" s="62"/>
-      <c r="T189" s="62"/>
-    </row>
-    <row r="190" spans="19:20">
+    <row r="175" spans="1:20" ht="90">
+      <c r="A175" s="78" t="s">
+        <v>811</v>
+      </c>
+      <c r="B175" s="78" t="s">
+        <v>812</v>
+      </c>
+      <c r="C175" s="78" t="s">
+        <v>95</v>
+      </c>
+      <c r="D175" s="85">
+        <v>698.25</v>
+      </c>
+      <c r="E175" s="85">
+        <v>1250</v>
+      </c>
+      <c r="F175" s="90">
+        <v>0</v>
+      </c>
+      <c r="G175" s="90">
+        <v>10</v>
+      </c>
+      <c r="H175" s="89">
+        <f t="shared" ref="H175" si="29">F175+IF(LEN(G175)=0,0,G175)</f>
+        <v>10</v>
+      </c>
+      <c r="I175" s="89">
+        <f>IF(D175&lt;&gt;"",D175,IFERROR(E175/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
+        <v>698.25</v>
+      </c>
+      <c r="J175" s="89">
+        <f t="shared" ref="J175" si="30">F175*I175</f>
+        <v>0</v>
+      </c>
+      <c r="K175" s="89">
+        <f t="shared" ref="K175" si="31">IF(LEN(G175)=0,0,G175)*I175</f>
+        <v>6982.5</v>
+      </c>
+      <c r="L175" s="78"/>
+      <c r="M175" s="78"/>
+      <c r="N175" s="78" t="s">
+        <v>506</v>
+      </c>
+      <c r="O175" s="78"/>
+      <c r="P175" s="78" t="s">
+        <v>815</v>
+      </c>
+      <c r="Q175" s="78"/>
+      <c r="R175" s="78"/>
+      <c r="S175" s="78"/>
+      <c r="T175" s="78"/>
+    </row>
+    <row r="176" spans="1:20" ht="15">
+      <c r="A176" s="83"/>
+      <c r="B176" s="83"/>
+      <c r="C176" s="83"/>
+      <c r="D176" s="84"/>
+      <c r="E176" s="84"/>
+      <c r="F176" s="92"/>
+      <c r="G176" s="92"/>
+      <c r="H176" s="91"/>
+      <c r="I176" s="91"/>
+      <c r="J176" s="91"/>
+      <c r="K176" s="91"/>
+      <c r="L176" s="83"/>
+      <c r="M176" s="83"/>
+      <c r="N176" s="83"/>
+      <c r="O176" s="83"/>
+      <c r="P176" s="83"/>
+      <c r="Q176" s="83"/>
+      <c r="R176" s="83"/>
+      <c r="S176" s="83"/>
+      <c r="T176" s="83"/>
+    </row>
+    <row r="177" spans="1:20" ht="15">
+      <c r="A177" s="78"/>
+      <c r="B177" s="78"/>
+      <c r="C177" s="78"/>
+      <c r="D177" s="85"/>
+      <c r="E177" s="85"/>
+      <c r="F177" s="90"/>
+      <c r="G177" s="90"/>
+      <c r="H177" s="89"/>
+      <c r="I177" s="89"/>
+      <c r="J177" s="89"/>
+      <c r="K177" s="89"/>
+      <c r="L177" s="78"/>
+      <c r="M177" s="78"/>
+      <c r="N177" s="78"/>
+      <c r="O177" s="78"/>
+      <c r="P177" s="78"/>
+      <c r="Q177" s="78"/>
+      <c r="R177" s="78"/>
+      <c r="S177" s="78"/>
+      <c r="T177" s="78"/>
+    </row>
+    <row r="178" spans="1:20" ht="15">
+      <c r="A178" s="83"/>
+      <c r="B178" s="83"/>
+      <c r="C178" s="83"/>
+      <c r="D178" s="84"/>
+      <c r="E178" s="84"/>
+      <c r="F178" s="92"/>
+      <c r="G178" s="92"/>
+      <c r="H178" s="91"/>
+      <c r="I178" s="91"/>
+      <c r="J178" s="91"/>
+      <c r="K178" s="91"/>
+      <c r="L178" s="83"/>
+      <c r="M178" s="83"/>
+      <c r="N178" s="83"/>
+      <c r="O178" s="83"/>
+      <c r="P178" s="83"/>
+      <c r="Q178" s="83"/>
+      <c r="R178" s="83"/>
+      <c r="S178" s="83"/>
+      <c r="T178" s="83"/>
+    </row>
+    <row r="179" spans="1:20" ht="15">
+      <c r="A179" s="78"/>
+      <c r="B179" s="78"/>
+      <c r="C179" s="78"/>
+      <c r="D179" s="85"/>
+      <c r="E179" s="85"/>
+      <c r="F179" s="90"/>
+      <c r="G179" s="90"/>
+      <c r="H179" s="89"/>
+      <c r="I179" s="89"/>
+      <c r="J179" s="89"/>
+      <c r="K179" s="89"/>
+      <c r="L179" s="78"/>
+      <c r="M179" s="78"/>
+      <c r="N179" s="78"/>
+      <c r="O179" s="78"/>
+      <c r="P179" s="78"/>
+      <c r="Q179" s="78"/>
+      <c r="R179" s="78"/>
+      <c r="S179" s="78"/>
+      <c r="T179" s="78"/>
+    </row>
+    <row r="180" spans="1:20" ht="15">
+      <c r="A180" s="83"/>
+      <c r="B180" s="83"/>
+      <c r="C180" s="83"/>
+      <c r="D180" s="84"/>
+      <c r="E180" s="84"/>
+      <c r="F180" s="92"/>
+      <c r="G180" s="92"/>
+      <c r="H180" s="91"/>
+      <c r="I180" s="91"/>
+      <c r="J180" s="91"/>
+      <c r="K180" s="91"/>
+      <c r="L180" s="83"/>
+      <c r="M180" s="83"/>
+      <c r="N180" s="83"/>
+      <c r="O180" s="83"/>
+      <c r="P180" s="83"/>
+      <c r="Q180" s="83"/>
+      <c r="R180" s="83"/>
+      <c r="S180" s="83"/>
+      <c r="T180" s="83"/>
+    </row>
+    <row r="181" spans="1:20" ht="15">
+      <c r="A181" s="78"/>
+      <c r="B181" s="78"/>
+      <c r="C181" s="78"/>
+      <c r="D181" s="85"/>
+      <c r="E181" s="85"/>
+      <c r="F181" s="90"/>
+      <c r="G181" s="90"/>
+      <c r="H181" s="89"/>
+      <c r="I181" s="89"/>
+      <c r="J181" s="89"/>
+      <c r="K181" s="89"/>
+      <c r="L181" s="78"/>
+      <c r="M181" s="78"/>
+      <c r="N181" s="78"/>
+      <c r="O181" s="78"/>
+      <c r="P181" s="78"/>
+      <c r="Q181" s="78"/>
+      <c r="R181" s="78"/>
+      <c r="S181" s="78"/>
+      <c r="T181" s="78"/>
+    </row>
+    <row r="182" spans="1:20" ht="15">
+      <c r="A182" s="83"/>
+      <c r="B182" s="83"/>
+      <c r="C182" s="83"/>
+      <c r="D182" s="84"/>
+      <c r="E182" s="84"/>
+      <c r="F182" s="92"/>
+      <c r="G182" s="92"/>
+      <c r="H182" s="91"/>
+      <c r="I182" s="91"/>
+      <c r="J182" s="91"/>
+      <c r="K182" s="91"/>
+      <c r="L182" s="83"/>
+      <c r="M182" s="83"/>
+      <c r="N182" s="83"/>
+      <c r="O182" s="83"/>
+      <c r="P182" s="83"/>
+      <c r="Q182" s="83"/>
+      <c r="R182" s="83"/>
+      <c r="S182" s="83"/>
+      <c r="T182" s="83"/>
+    </row>
+    <row r="183" spans="1:20" ht="15">
+      <c r="A183" s="78"/>
+      <c r="B183" s="78"/>
+      <c r="C183" s="78"/>
+      <c r="D183" s="85"/>
+      <c r="E183" s="85"/>
+      <c r="F183" s="90"/>
+      <c r="G183" s="90"/>
+      <c r="H183" s="89"/>
+      <c r="I183" s="89"/>
+      <c r="J183" s="89"/>
+      <c r="K183" s="89"/>
+      <c r="L183" s="78"/>
+      <c r="M183" s="78"/>
+      <c r="N183" s="78"/>
+      <c r="O183" s="78"/>
+      <c r="P183" s="78"/>
+      <c r="Q183" s="78"/>
+      <c r="R183" s="78"/>
+      <c r="S183" s="78"/>
+      <c r="T183" s="78"/>
+    </row>
+    <row r="184" spans="1:20" ht="15">
+      <c r="A184" s="83"/>
+      <c r="B184" s="83"/>
+      <c r="C184" s="83"/>
+      <c r="D184" s="84"/>
+      <c r="E184" s="84"/>
+      <c r="F184" s="92"/>
+      <c r="G184" s="92"/>
+      <c r="H184" s="91"/>
+      <c r="I184" s="91"/>
+      <c r="J184" s="91"/>
+      <c r="K184" s="91"/>
+      <c r="L184" s="83"/>
+      <c r="M184" s="83"/>
+      <c r="N184" s="83"/>
+      <c r="O184" s="83"/>
+      <c r="P184" s="83"/>
+      <c r="Q184" s="83"/>
+      <c r="R184" s="83"/>
+      <c r="S184" s="83"/>
+      <c r="T184" s="83"/>
+    </row>
+    <row r="185" spans="1:20" ht="15">
+      <c r="A185" s="78"/>
+      <c r="B185" s="78"/>
+      <c r="C185" s="78"/>
+      <c r="D185" s="85"/>
+      <c r="E185" s="85"/>
+      <c r="F185" s="90"/>
+      <c r="G185" s="90"/>
+      <c r="H185" s="89"/>
+      <c r="I185" s="89"/>
+      <c r="J185" s="89"/>
+      <c r="K185" s="89"/>
+      <c r="L185" s="78"/>
+      <c r="M185" s="78"/>
+      <c r="N185" s="78"/>
+      <c r="O185" s="78"/>
+      <c r="P185" s="78"/>
+      <c r="Q185" s="78"/>
+      <c r="R185" s="78"/>
+      <c r="S185" s="78"/>
+      <c r="T185" s="78"/>
+    </row>
+    <row r="186" spans="1:20" ht="15">
+      <c r="A186" s="83"/>
+      <c r="B186" s="83"/>
+      <c r="C186" s="83"/>
+      <c r="D186" s="84"/>
+      <c r="E186" s="84"/>
+      <c r="F186" s="92"/>
+      <c r="G186" s="92"/>
+      <c r="H186" s="91"/>
+      <c r="I186" s="91"/>
+      <c r="J186" s="91"/>
+      <c r="K186" s="91"/>
+      <c r="L186" s="83"/>
+      <c r="M186" s="83"/>
+      <c r="N186" s="83"/>
+      <c r="O186" s="83"/>
+      <c r="P186" s="83"/>
+      <c r="Q186" s="83"/>
+      <c r="R186" s="83"/>
+      <c r="S186" s="83"/>
+      <c r="T186" s="83"/>
+    </row>
+    <row r="187" spans="1:20" ht="15">
+      <c r="A187" s="78"/>
+      <c r="B187" s="78"/>
+      <c r="C187" s="78"/>
+      <c r="D187" s="85"/>
+      <c r="E187" s="85"/>
+      <c r="F187" s="90"/>
+      <c r="G187" s="90"/>
+      <c r="H187" s="89"/>
+      <c r="I187" s="89"/>
+      <c r="J187" s="89"/>
+      <c r="K187" s="89"/>
+      <c r="L187" s="78"/>
+      <c r="M187" s="78"/>
+      <c r="N187" s="78"/>
+      <c r="O187" s="78"/>
+      <c r="P187" s="78"/>
+      <c r="Q187" s="78"/>
+      <c r="R187" s="78"/>
+      <c r="S187" s="78"/>
+      <c r="T187" s="78"/>
+    </row>
+    <row r="188" spans="1:20" ht="15">
+      <c r="A188" s="83"/>
+      <c r="B188" s="83"/>
+      <c r="C188" s="83"/>
+      <c r="D188" s="84"/>
+      <c r="E188" s="84"/>
+      <c r="F188" s="92"/>
+      <c r="G188" s="92"/>
+      <c r="H188" s="91"/>
+      <c r="I188" s="91"/>
+      <c r="J188" s="91"/>
+      <c r="K188" s="91"/>
+      <c r="L188" s="83"/>
+      <c r="M188" s="83"/>
+      <c r="N188" s="83"/>
+      <c r="O188" s="83"/>
+      <c r="P188" s="83"/>
+      <c r="Q188" s="83"/>
+      <c r="R188" s="83"/>
+      <c r="S188" s="83"/>
+      <c r="T188" s="83"/>
+    </row>
+    <row r="189" spans="1:20" ht="15">
+      <c r="A189" s="78"/>
+      <c r="B189" s="78"/>
+      <c r="C189" s="78"/>
+      <c r="D189" s="85"/>
+      <c r="E189" s="85"/>
+      <c r="F189" s="90"/>
+      <c r="G189" s="90"/>
+      <c r="H189" s="89"/>
+      <c r="I189" s="89"/>
+      <c r="J189" s="89"/>
+      <c r="K189" s="89"/>
+      <c r="L189" s="78"/>
+      <c r="M189" s="78"/>
+      <c r="N189" s="78"/>
+      <c r="O189" s="78"/>
+      <c r="P189" s="78"/>
+      <c r="Q189" s="78"/>
+      <c r="R189" s="78"/>
+      <c r="S189" s="78"/>
+      <c r="T189" s="78"/>
+    </row>
+    <row r="190" spans="1:20">
       <c r="S190" s="62"/>
       <c r="T190" s="62"/>
     </row>
-    <row r="191" spans="19:20">
+    <row r="191" spans="1:20">
       <c r="S191" s="62"/>
       <c r="T191" s="62"/>
     </row>
-    <row r="192" spans="19:20">
+    <row r="192" spans="1:20">
       <c r="S192" s="62"/>
       <c r="T192" s="62"/>
     </row>
@@ -36096,6 +36451,7 @@
       <c r="T1996" s="62"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="29" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N988" xr:uid="{00000000-0002-0000-0500-000000000000}">
       <formula1>"Pending,Partially Sold,Sold Out,New,Reserved"</formula1>
@@ -36125,7 +36481,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1">
       <c r="A1" s="94" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="B1" s="94"/>
     </row>
@@ -36134,7 +36490,7 @@
         <v>42</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="13.5" customHeight="1">
@@ -36166,25 +36522,25 @@
         <v>42</v>
       </c>
       <c r="B7" s="72" t="s">
+        <v>728</v>
+      </c>
+      <c r="C7" s="72" t="s">
+        <v>729</v>
+      </c>
+      <c r="D7" s="72" t="s">
         <v>730</v>
       </c>
-      <c r="C7" s="72" t="s">
+      <c r="E7" s="72" t="s">
         <v>731</v>
       </c>
-      <c r="D7" s="72" t="s">
+      <c r="F7" s="72" t="s">
         <v>732</v>
       </c>
-      <c r="E7" s="72" t="s">
+      <c r="G7" s="72" t="s">
         <v>733</v>
       </c>
-      <c r="F7" s="72" t="s">
+      <c r="H7" s="72" t="s">
         <v>734</v>
-      </c>
-      <c r="G7" s="72" t="s">
-        <v>735</v>
-      </c>
-      <c r="H7" s="72" t="s">
-        <v>736</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="13.5" customHeight="1">
@@ -36288,7 +36644,7 @@
     </row>
     <row r="12" spans="1:8" s="74" customFormat="1" ht="15.75" customHeight="1">
       <c r="A12" s="95" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="B12" s="95"/>
       <c r="C12" s="95"/>
@@ -36301,13 +36657,13 @@
         <v>98</v>
       </c>
       <c r="B13" s="72" t="s">
+        <v>736</v>
+      </c>
+      <c r="C13" s="72" t="s">
+        <v>737</v>
+      </c>
+      <c r="D13" s="72" t="s">
         <v>738</v>
-      </c>
-      <c r="C13" s="72" t="s">
-        <v>739</v>
-      </c>
-      <c r="D13" s="72" t="s">
-        <v>740</v>
       </c>
       <c r="E13" s="72" t="s">
         <v>99</v>
@@ -36321,7 +36677,7 @@
         <v>45952</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>51</v>
@@ -36339,7 +36695,7 @@
         <v>45952</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>51</v>
@@ -36393,7 +36749,7 @@
         <v>45970</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>50</v>
@@ -36411,7 +36767,7 @@
         <v>45970</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>50</v>
@@ -36429,7 +36785,7 @@
         <v>45973</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>50</v>
@@ -36447,7 +36803,7 @@
         <v>45973</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>49</v>
@@ -36465,7 +36821,7 @@
         <v>46058</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>51</v>
@@ -36501,7 +36857,7 @@
         <v>46059</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>49</v>
@@ -36537,7 +36893,7 @@
         <v>46093</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>50</v>
@@ -36555,7 +36911,7 @@
         <v>46093</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>51</v>
@@ -36638,7 +36994,7 @@
     </row>
     <row r="58" spans="2:2" ht="13.5" customHeight="1">
       <c r="B58" s="6" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
     </row>
   </sheetData>
@@ -36668,7 +37024,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="13.5" customHeight="1">
       <c r="A1" s="77" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="73" customFormat="1" ht="13.5" customHeight="1">
@@ -36676,22 +37032,22 @@
         <v>42</v>
       </c>
       <c r="B3" s="72" t="s">
+        <v>742</v>
+      </c>
+      <c r="C3" s="72" t="s">
+        <v>727</v>
+      </c>
+      <c r="D3" s="72" t="s">
+        <v>743</v>
+      </c>
+      <c r="E3" s="72" t="s">
         <v>744</v>
       </c>
-      <c r="C3" s="72" t="s">
-        <v>729</v>
-      </c>
-      <c r="D3" s="72" t="s">
+      <c r="F3" s="72" t="s">
         <v>745</v>
       </c>
-      <c r="E3" s="72" t="s">
+      <c r="G3" s="72" t="s">
         <v>746</v>
-      </c>
-      <c r="F3" s="72" t="s">
-        <v>747</v>
-      </c>
-      <c r="G3" s="72" t="s">
-        <v>748</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="13.5" customHeight="1">
@@ -36700,7 +37056,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>239803</v>
+        <v>241803</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -36708,11 +37064,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>86934.716799999995</v>
+        <v>87601.516799999998</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>152868.28320000001</v>
+        <v>154201.48320000002</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -36720,7 +37076,7 @@
       </c>
       <c r="G4" s="16">
         <f>E4+F4</f>
-        <v>15558.257199999993</v>
+        <v>16891.457200000004</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -36737,11 +37093,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>86882.566399999996</v>
+        <v>87548.966400000005</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-78463.566399999996</v>
+        <v>-79129.966400000005</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -36749,7 +37105,7 @@
       </c>
       <c r="G5" s="18">
         <f>E5+F5</f>
-        <v>-6876.5243999999948</v>
+        <v>-7542.9244000000035</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -36766,11 +37122,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>86934.716799999995</v>
+        <v>87601.516799999998</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-74404.716799999995</v>
+        <v>-75071.516799999998</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -36778,7 +37134,7 @@
       </c>
       <c r="G6" s="16">
         <f>E6+F6</f>
-        <v>-8681.7327999999834</v>
+        <v>-9348.5327999999863</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">
@@ -36788,27 +37144,27 @@
     </row>
     <row r="10" spans="1:7" ht="13.5" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="13.5" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="13.5" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="13.5" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="13.5" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rust Orange Banarasi sales
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Apr26.xlsx
+++ b/docs/Chiraath-Summary-Apr26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC2697E5-5F0F-7C47-A0F5-3F91032FF39D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0877EBD5-9369-174C-9C54-C9FEB07C1797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2043" uniqueCount="821">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2047" uniqueCount="822">
   <si>
     <t>Notes:</t>
   </si>
@@ -1851,6 +1851,671 @@
   </si>
   <si>
     <t>Banarasi Silk</t>
+  </si>
+  <si>
+    <t>CHR-116</t>
+  </si>
+  <si>
+    <t>Banarasi Silk (Yellow design)</t>
+  </si>
+  <si>
+    <t>CHR-117</t>
+  </si>
+  <si>
+    <t>Chanderi Silk Tie &amp; Dye collection</t>
+  </si>
+  <si>
+    <t>Nalini - Pink (1400)</t>
+  </si>
+  <si>
+    <t>Blue - 1</t>
+  </si>
+  <si>
+    <t>CHR-118</t>
+  </si>
+  <si>
+    <t>Off-white block-printed silk saree</t>
+  </si>
+  <si>
+    <t>CHR-119</t>
+  </si>
+  <si>
+    <t>Chanderi Printed Silk Saree</t>
+  </si>
+  <si>
+    <t>Aruna - violet, Resmi - navy blue, Malini - Rani Pink</t>
+  </si>
+  <si>
+    <t>CHR-120</t>
+  </si>
+  <si>
+    <t>Kalyani cotton silk</t>
+  </si>
+  <si>
+    <t>Aruna - Yellow, Malu - Orange (Pending)</t>
+  </si>
+  <si>
+    <t>yellow green &amp; orange green</t>
+  </si>
+  <si>
+    <t>CHR-121</t>
+  </si>
+  <si>
+    <t>Roman Silk Salwar Set</t>
+  </si>
+  <si>
+    <t>Sushitha (XXL-1600)</t>
+  </si>
+  <si>
+    <t>M, L, XL</t>
+  </si>
+  <si>
+    <t>CHR-122</t>
+  </si>
+  <si>
+    <t>Banarasi Silk (Parrot Green)</t>
+  </si>
+  <si>
+    <t>Nisha Nair
+Shiji
+Priya Reji
+Raji
+Nisha Sajitha</t>
+  </si>
+  <si>
+    <t>CHR-123</t>
+  </si>
+  <si>
+    <t>Kalyani cotton silk (red)</t>
+  </si>
+  <si>
+    <t>Divya (Kollam), Ananya (TVM), Liji (Vadakara), Archana(Devagiri)-Ordered, Anu(Kottayam), Linu(Kottayam)</t>
+  </si>
+  <si>
+    <t>CHR-124</t>
+  </si>
+  <si>
+    <t>Viscose Chokda</t>
+  </si>
+  <si>
+    <t>Neethu(Pkd)-1450, Remya(Pkd)-1250</t>
+  </si>
+  <si>
+    <t>Blue, Green</t>
+  </si>
+  <si>
+    <t>CHR-125</t>
+  </si>
+  <si>
+    <t>Aanchal Maroon Salwar</t>
+  </si>
+  <si>
+    <t>Malu (1800)</t>
+  </si>
+  <si>
+    <t>XXXL</t>
+  </si>
+  <si>
+    <t>CHR-126</t>
+  </si>
+  <si>
+    <t>Aanchal maroon palzo kurta</t>
+  </si>
+  <si>
+    <t>CHR-127</t>
+  </si>
+  <si>
+    <t>⁠Rustic Geo Kota (Stairs) - Net Kota</t>
+  </si>
+  <si>
+    <t>CHR-128</t>
+  </si>
+  <si>
+    <t>⁠Grey Arrow Kota (Arrow) - Net kota</t>
+  </si>
+  <si>
+    <t>Chris (1250)</t>
+  </si>
+  <si>
+    <t>CHR-129</t>
+  </si>
+  <si>
+    <t>Dolla silk Olive Green</t>
+  </si>
+  <si>
+    <t>CHR-130</t>
+  </si>
+  <si>
+    <t>Chanderi Cotton (Golden Yellow)</t>
+  </si>
+  <si>
+    <t>CHR-131</t>
+  </si>
+  <si>
+    <t>⁠​Regal Black semi silk Brocade type</t>
+  </si>
+  <si>
+    <t>Saranya Gopalakrishnan(1300)</t>
+  </si>
+  <si>
+    <t>CHR-132</t>
+  </si>
+  <si>
+    <t>Kota Doria (Green with silver floral work)</t>
+  </si>
+  <si>
+    <t>CHR-133</t>
+  </si>
+  <si>
+    <t>Semi Silk (Peach)</t>
+  </si>
+  <si>
+    <t>CHR-134</t>
+  </si>
+  <si>
+    <t>Net kota saree - turquoise blue with floral design and maroon border</t>
+  </si>
+  <si>
+    <t>priya(hosur)</t>
+  </si>
+  <si>
+    <t>CHR-135</t>
+  </si>
+  <si>
+    <t>⁠Viscose Chokda</t>
+  </si>
+  <si>
+    <t>CHR-136</t>
+  </si>
+  <si>
+    <t>Banarasi silk (lavender)</t>
+  </si>
+  <si>
+    <t>CHR-137</t>
+  </si>
+  <si>
+    <t>⁠​Blue manipuri silk saree</t>
+  </si>
+  <si>
+    <t>CHR-138</t>
+  </si>
+  <si>
+    <t>⁠​Linen black saree</t>
+  </si>
+  <si>
+    <t>CHR-139</t>
+  </si>
+  <si>
+    <t xml:space="preserve">⁠​Maheswari cotton Silk saree </t>
+  </si>
+  <si>
+    <t>haris(ekm)</t>
+  </si>
+  <si>
+    <t>CHR-140</t>
+  </si>
+  <si>
+    <t>⁠​Ganga Jamuna kalyani Cotton Saree</t>
+  </si>
+  <si>
+    <t>CHR-141</t>
+  </si>
+  <si>
+    <t>Semi Silk</t>
+  </si>
+  <si>
+    <t>Annu (Light Violet Semi Silk), Susmi - Coffee, Navya - mustard</t>
+  </si>
+  <si>
+    <t>CHR-142</t>
+  </si>
+  <si>
+    <t>Semi Silk (Rose Pink)</t>
+  </si>
+  <si>
+    <t>CHR-143</t>
+  </si>
+  <si>
+    <t>Synthetic Net Kota Doria (Soft ivory/off-white - Muted Coral Pink &amp; Olive green floral motifs)</t>
+  </si>
+  <si>
+    <t>CHR-144</t>
+  </si>
+  <si>
+    <t>CHR-145</t>
+  </si>
+  <si>
+    <t>Linen Saree with Check (Maroon with golden checks, Rust Orange with golden checks)</t>
+  </si>
+  <si>
+    <t>Chris (1000 - Green)</t>
+  </si>
+  <si>
+    <t>CHR-146</t>
+  </si>
+  <si>
+    <t>CHR-147</t>
+  </si>
+  <si>
+    <t>Soft Cotton Saree (with butterfly design on Pallu)</t>
+  </si>
+  <si>
+    <t>Latha(Yellow), Sari(Peach)</t>
+  </si>
+  <si>
+    <t>CHR-148</t>
+  </si>
+  <si>
+    <t>SAREES 5619 (Tissue Silk Saree Golden Color)</t>
+  </si>
+  <si>
+    <t>CHR-149</t>
+  </si>
+  <si>
+    <t>SAREE TISSUE EMB (Lavender (light &amp; dark), Red)</t>
+  </si>
+  <si>
+    <t>CHR-150</t>
+  </si>
+  <si>
+    <t>CHIKKANKARI SALWAR</t>
+  </si>
+  <si>
+    <t>Praneetha (L), Rameez Cousin (M)</t>
+  </si>
+  <si>
+    <t>XL, XXL</t>
+  </si>
+  <si>
+    <t>Purple</t>
+  </si>
+  <si>
+    <t>CHR-151</t>
+  </si>
+  <si>
+    <t>Short Kurta</t>
+  </si>
+  <si>
+    <t>Rinsha(M)</t>
+  </si>
+  <si>
+    <t>L,XL,XXL</t>
+  </si>
+  <si>
+    <t>Light Brown colr</t>
+  </si>
+  <si>
+    <t>CHR-152</t>
+  </si>
+  <si>
+    <t>Banarasi (Yellow/Green)</t>
+  </si>
+  <si>
+    <t>Yellow Green</t>
+  </si>
+  <si>
+    <t>CHR-153</t>
+  </si>
+  <si>
+    <t>Ivory &amp; black printed cotton 3-piece salwar set</t>
+  </si>
+  <si>
+    <t>M, XL, XXL</t>
+  </si>
+  <si>
+    <t>CHR-154</t>
+  </si>
+  <si>
+    <t>Dark brown embroidered cotton 3-piece salwar set</t>
+  </si>
+  <si>
+    <t>CHR-155</t>
+  </si>
+  <si>
+    <t>Black cotton 3-piece salwar set with printed dupatta</t>
+  </si>
+  <si>
+    <t>M, L, XL, XXL</t>
+  </si>
+  <si>
+    <t>CHR-156</t>
+  </si>
+  <si>
+    <t>Off-white cotton 2-piece set with blue floral prints</t>
+  </si>
+  <si>
+    <t>Prema(XXL)</t>
+  </si>
+  <si>
+    <t>CHR-157</t>
+  </si>
+  <si>
+    <t>Off-white printed 2-piece kurti set with multicolor pattern</t>
+  </si>
+  <si>
+    <t>M, L, XL, XXL, XXXL</t>
+  </si>
+  <si>
+    <t>CHR-158</t>
+  </si>
+  <si>
+    <t>Olive green cotton 2-piece kurti set with floral prints</t>
+  </si>
+  <si>
+    <t>CHR-159</t>
+  </si>
+  <si>
+    <t>Khadee Saree - Navy Blue and Olive Green</t>
+  </si>
+  <si>
+    <t>CHR-160</t>
+  </si>
+  <si>
+    <t>Khadee Saree - Brown &amp; Black</t>
+  </si>
+  <si>
+    <t>CHR-161</t>
+  </si>
+  <si>
+    <t>Black &amp; Beige Leaf Print Cotton Silk Saree</t>
+  </si>
+  <si>
+    <t>CHR-162</t>
+  </si>
+  <si>
+    <t>Teal &amp; Coral Abstract Print Cotton Silk Saree</t>
+  </si>
+  <si>
+    <t>Partner Settings</t>
+  </si>
+  <si>
+    <t>Share %</t>
+  </si>
+  <si>
+    <t>Total Purchases (Contributions)</t>
+  </si>
+  <si>
+    <t>Target Contributions (by %)</t>
+  </si>
+  <si>
+    <t>Contribution Over/(Under)</t>
+  </si>
+  <si>
+    <t>Profit Share (Completed Only)</t>
+  </si>
+  <si>
+    <t>Net Before Settlements</t>
+  </si>
+  <si>
+    <t>Net Settlements (Received - Paid)</t>
+  </si>
+  <si>
+    <t>Net Position After Settlements</t>
+  </si>
+  <si>
+    <t>Global Settlements Log (used for Contributions, Cash Pool &amp; Profit)</t>
+  </si>
+  <si>
+    <t>Type (Contribution/Cash/Profit)</t>
+  </si>
+  <si>
+    <t>From Partner</t>
+  </si>
+  <si>
+    <t>To Partner</t>
+  </si>
+  <si>
+    <t>Contribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Cash Pool Overview (Completed Sales Only)</t>
+  </si>
+  <si>
+    <t>Cash Collected (Completed Sales)</t>
+  </si>
+  <si>
+    <t>Target Cash Based on %</t>
+  </si>
+  <si>
+    <t>Over/(Under) Collection</t>
+  </si>
+  <si>
+    <t>Net Cash Settlements (Received - Paid)</t>
+  </si>
+  <si>
+    <t>Cash Position After Settlements</t>
+  </si>
+  <si>
+    <t>1. Cash Collected only counts sales with Status = "Completed".</t>
+  </si>
+  <si>
+    <t>2. Target Cash is based on the same partner percentages as profit sharing.</t>
+  </si>
+  <si>
+    <t>3. Over/(Under) is the raw difference before any cash settlements.</t>
+  </si>
+  <si>
+    <t>4. Net Cash Settlements reads Type = "Cash" rows from PartnerShares Settlements Log.</t>
+  </si>
+  <si>
+    <t>5. Cash Position After Settlements = Over/(Under) + Net Cash Settlements.</t>
+  </si>
+  <si>
+    <t>Shinoob</t>
+  </si>
+  <si>
+    <t>Banarasi Yello &amp; Green, Tussar Silk Teal Blue, Green Cotton Silk</t>
+  </si>
+  <si>
+    <t>Green</t>
+  </si>
+  <si>
+    <t>Shinoob (1200)</t>
+  </si>
+  <si>
+    <t>Chris (Goldern with flowers)</t>
+  </si>
+  <si>
+    <t>Matka silk - Blue/Green</t>
+  </si>
+  <si>
+    <t>Golden color tissue with flowers</t>
+  </si>
+  <si>
+    <t>Jothika(Pkd)</t>
+  </si>
+  <si>
+    <t>Matka silk - Blue/red</t>
+  </si>
+  <si>
+    <t>Vineetha(Kottayam)</t>
+  </si>
+  <si>
+    <t>Matka Silk - mustard</t>
+  </si>
+  <si>
+    <t>Amalu(black/maroon), Lethy(Thiruvalla):1550, Vineet(Maroon): 1550, Chris(Yellow) - 1250, Geemol (Black/Violet) - 1500</t>
+  </si>
+  <si>
+    <t>Geemol Mathew (Kottayam)</t>
+  </si>
+  <si>
+    <t>Viscose georgette - Black/Violet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grey-Black/Red, Maroon-Yellow/Bottle Green, Purple-Yellow/Bottle Green, Bottle Green-Yellow/Red, Peacock Blue-Purple/Golden Yellow  </t>
+  </si>
+  <si>
+    <t>CHR-163</t>
+  </si>
+  <si>
+    <t>Sungudi  (Alice Christy inspired)</t>
+  </si>
+  <si>
+    <t>CHR-164</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Red &amp; Navy Blue </t>
+  </si>
+  <si>
+    <t>CHR-165</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Violet, Chocolate Brown, Bottle Green  </t>
+  </si>
+  <si>
+    <t>Tant Mix (Bank)</t>
+  </si>
+  <si>
+    <t>CHR-166</t>
+  </si>
+  <si>
+    <t>Tant mix bank - peacock blue</t>
+  </si>
+  <si>
+    <t>Peacock blue with rany pink</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yellow, Dark Green, Violet  </t>
+  </si>
+  <si>
+    <t>CHR-167</t>
+  </si>
+  <si>
+    <t>CHR-168</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bengal Cotton (Light Orange Floral)  </t>
+  </si>
+  <si>
+    <t>Orange floral</t>
+  </si>
+  <si>
+    <t>March boosting</t>
+  </si>
+  <si>
+    <t>Susmi. Shinoob (Teal blue), Sarany Hyd -980</t>
+  </si>
+  <si>
+    <t>Tussar silk Green(CHR-70) - 500 advance, Tissue silk non floral(CHR-148)</t>
+  </si>
+  <si>
+    <t>Cotton blend saree yellow - CHR-67</t>
+  </si>
+  <si>
+    <t>Jitha Joy</t>
+  </si>
+  <si>
+    <t>Jitha Joy - 650</t>
+  </si>
+  <si>
+    <t>Mulmul cotton black - CHR-65</t>
+  </si>
+  <si>
+    <t>Deepa Rajan</t>
+  </si>
+  <si>
+    <t>Banarasi Sarees (New Collection)</t>
+  </si>
+  <si>
+    <t>CHR-169</t>
+  </si>
+  <si>
+    <t>Dark biege with bottle green, Biege Maroon combination, Green</t>
+  </si>
+  <si>
+    <t>Rajna - 740, Malini - 980, Baby Khadeeja - 980</t>
+  </si>
+  <si>
+    <t>Shinoob - 1100, Sruthi - 1100</t>
+  </si>
+  <si>
+    <t>Green Cotton Silk (CHR-88)</t>
+  </si>
+  <si>
+    <t>Swapna Binu(Thrisurr)</t>
+  </si>
+  <si>
+    <t>Yellow Green (CHR-146)</t>
+  </si>
+  <si>
+    <t>CHR-170</t>
+  </si>
+  <si>
+    <t>Kerala Saree Temple design</t>
+  </si>
+  <si>
+    <t>CHR-171</t>
+  </si>
+  <si>
+    <t>Kerala Saree Kathakali</t>
+  </si>
+  <si>
+    <t>Kerala Saree floral embroidery</t>
+  </si>
+  <si>
+    <t>CHR-172</t>
+  </si>
+  <si>
+    <t>CHR-173</t>
+  </si>
+  <si>
+    <t>Sungudi Saree (Alice Christy inspired)</t>
+  </si>
+  <si>
+    <t>Rani Pink(1), Jet Black(2), Maroon(3), Dark Green(1), navy Blue (2), Off white (1)</t>
+  </si>
+  <si>
+    <t>Matka Silk Saree collections - old design</t>
+  </si>
+  <si>
+    <t>CHR-174</t>
+  </si>
+  <si>
+    <t>Matka Silk Saree collections - new design</t>
+  </si>
+  <si>
+    <t>Blue/bottle green - Saranya Hyd, Blue/red - Jothika, Mustard - Vineetha, Bottle Green/Golden Yellow - Swapna (Thrissur)-1200</t>
+  </si>
+  <si>
+    <t>Bottle Green/Golden Yellow - 2 
+Black/Golden Yellow - 2
+Navy Blue/Bottle Green - 2</t>
+  </si>
+  <si>
+    <t>Peacok Blue/Maroon - 3
+Purple/Green - 1
+Navy Blue/Maroon - 3
+Maroon/Navy Blue - 1
+Lavender/Violet - 1
+Grey/Blue - 1</t>
+  </si>
+  <si>
+    <t>Banarasi Sarees with Paisley motifs</t>
+  </si>
+  <si>
+    <t>Chokda Rust Orange, Dolla</t>
+  </si>
+  <si>
+    <t>Ranju(1000)</t>
+  </si>
+  <si>
+    <t>burned orange (lotus)</t>
+  </si>
+  <si>
+    <t>Sreeja -Green:1250, Ranju - rust orange:1000</t>
+  </si>
+  <si>
+    <t>Jute Silk Checked Saree</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khadi Cotton Saree (Jar Border)  </t>
+  </si>
+  <si>
+    <t>Narayanpet sarees</t>
   </si>
   <si>
     <t>Biscuit - Aruna, Silpa, Malini, Aswathi,  Resmi(Thrissur), Asha(Navaikulam), Ambika Preman (Pazhanji), Anitha(Pathanamthitta),salini(kottayam) vinod(kottayam), Laks Pillai
@@ -1859,675 +2524,14 @@
 Blue blue - Aruna
 Golden yellow - Malu 
 Golden Yellow - Vijina, Preethi Thomas
-Pink - Ambika Preman (Pazhanji)</t>
-  </si>
-  <si>
-    <t>Rust orange - 1</t>
-  </si>
-  <si>
-    <t>CHR-116</t>
-  </si>
-  <si>
-    <t>Banarasi Silk (Yellow design)</t>
-  </si>
-  <si>
-    <t>CHR-117</t>
-  </si>
-  <si>
-    <t>Chanderi Silk Tie &amp; Dye collection</t>
-  </si>
-  <si>
-    <t>Nalini - Pink (1400)</t>
-  </si>
-  <si>
-    <t>Blue - 1</t>
-  </si>
-  <si>
-    <t>CHR-118</t>
-  </si>
-  <si>
-    <t>Off-white block-printed silk saree</t>
-  </si>
-  <si>
-    <t>CHR-119</t>
-  </si>
-  <si>
-    <t>Chanderi Printed Silk Saree</t>
-  </si>
-  <si>
-    <t>Aruna - violet, Resmi - navy blue, Malini - Rani Pink</t>
-  </si>
-  <si>
-    <t>CHR-120</t>
-  </si>
-  <si>
-    <t>Kalyani cotton silk</t>
-  </si>
-  <si>
-    <t>Aruna - Yellow, Malu - Orange (Pending)</t>
-  </si>
-  <si>
-    <t>yellow green &amp; orange green</t>
-  </si>
-  <si>
-    <t>CHR-121</t>
-  </si>
-  <si>
-    <t>Roman Silk Salwar Set</t>
-  </si>
-  <si>
-    <t>Sushitha (XXL-1600)</t>
-  </si>
-  <si>
-    <t>M, L, XL</t>
-  </si>
-  <si>
-    <t>CHR-122</t>
-  </si>
-  <si>
-    <t>Banarasi Silk (Parrot Green)</t>
-  </si>
-  <si>
-    <t>Nisha Nair
-Shiji
-Priya Reji
-Raji
-Nisha Sajitha</t>
-  </si>
-  <si>
-    <t>CHR-123</t>
-  </si>
-  <si>
-    <t>Kalyani cotton silk (red)</t>
-  </si>
-  <si>
-    <t>Divya (Kollam), Ananya (TVM), Liji (Vadakara), Archana(Devagiri)-Ordered, Anu(Kottayam), Linu(Kottayam)</t>
-  </si>
-  <si>
-    <t>CHR-124</t>
-  </si>
-  <si>
-    <t>Viscose Chokda</t>
-  </si>
-  <si>
-    <t>Neethu(Pkd)-1450, Remya(Pkd)-1250</t>
-  </si>
-  <si>
-    <t>Blue, Green</t>
-  </si>
-  <si>
-    <t>CHR-125</t>
-  </si>
-  <si>
-    <t>Aanchal Maroon Salwar</t>
-  </si>
-  <si>
-    <t>Malu (1800)</t>
-  </si>
-  <si>
-    <t>XXXL</t>
-  </si>
-  <si>
-    <t>CHR-126</t>
-  </si>
-  <si>
-    <t>Aanchal maroon palzo kurta</t>
-  </si>
-  <si>
-    <t>CHR-127</t>
-  </si>
-  <si>
-    <t>⁠Rustic Geo Kota (Stairs) - Net Kota</t>
-  </si>
-  <si>
-    <t>CHR-128</t>
-  </si>
-  <si>
-    <t>⁠Grey Arrow Kota (Arrow) - Net kota</t>
-  </si>
-  <si>
-    <t>Chris (1250)</t>
-  </si>
-  <si>
-    <t>CHR-129</t>
-  </si>
-  <si>
-    <t>Dolla silk Olive Green</t>
-  </si>
-  <si>
-    <t>CHR-130</t>
-  </si>
-  <si>
-    <t>Chanderi Cotton (Golden Yellow)</t>
-  </si>
-  <si>
-    <t>CHR-131</t>
-  </si>
-  <si>
-    <t>⁠​Regal Black semi silk Brocade type</t>
-  </si>
-  <si>
-    <t>Saranya Gopalakrishnan(1300)</t>
-  </si>
-  <si>
-    <t>CHR-132</t>
-  </si>
-  <si>
-    <t>Kota Doria (Green with silver floral work)</t>
-  </si>
-  <si>
-    <t>CHR-133</t>
-  </si>
-  <si>
-    <t>Semi Silk (Peach)</t>
-  </si>
-  <si>
-    <t>CHR-134</t>
-  </si>
-  <si>
-    <t>Net kota saree - turquoise blue with floral design and maroon border</t>
-  </si>
-  <si>
-    <t>priya(hosur)</t>
-  </si>
-  <si>
-    <t>CHR-135</t>
-  </si>
-  <si>
-    <t>⁠Viscose Chokda</t>
-  </si>
-  <si>
-    <t>CHR-136</t>
-  </si>
-  <si>
-    <t>Banarasi silk (lavender)</t>
-  </si>
-  <si>
-    <t>CHR-137</t>
-  </si>
-  <si>
-    <t>⁠​Blue manipuri silk saree</t>
-  </si>
-  <si>
-    <t>CHR-138</t>
-  </si>
-  <si>
-    <t>⁠​Linen black saree</t>
-  </si>
-  <si>
-    <t>CHR-139</t>
-  </si>
-  <si>
-    <t xml:space="preserve">⁠​Maheswari cotton Silk saree </t>
-  </si>
-  <si>
-    <t>haris(ekm)</t>
-  </si>
-  <si>
-    <t>CHR-140</t>
-  </si>
-  <si>
-    <t>⁠​Ganga Jamuna kalyani Cotton Saree</t>
-  </si>
-  <si>
-    <t>CHR-141</t>
-  </si>
-  <si>
-    <t>Semi Silk</t>
-  </si>
-  <si>
-    <t>Annu (Light Violet Semi Silk), Susmi - Coffee, Navya - mustard</t>
-  </si>
-  <si>
-    <t>CHR-142</t>
-  </si>
-  <si>
-    <t>Semi Silk (Rose Pink)</t>
-  </si>
-  <si>
-    <t>CHR-143</t>
-  </si>
-  <si>
-    <t>Synthetic Net Kota Doria (Soft ivory/off-white - Muted Coral Pink &amp; Olive green floral motifs)</t>
-  </si>
-  <si>
-    <t>CHR-144</t>
-  </si>
-  <si>
-    <t>CHR-145</t>
-  </si>
-  <si>
-    <t>Linen Saree with Check (Maroon with golden checks, Rust Orange with golden checks)</t>
-  </si>
-  <si>
-    <t>Chris (1000 - Green)</t>
-  </si>
-  <si>
-    <t>CHR-146</t>
-  </si>
-  <si>
-    <t>CHR-147</t>
-  </si>
-  <si>
-    <t>Soft Cotton Saree (with butterfly design on Pallu)</t>
-  </si>
-  <si>
-    <t>Latha(Yellow), Sari(Peach)</t>
-  </si>
-  <si>
-    <t>CHR-148</t>
-  </si>
-  <si>
-    <t>SAREES 5619 (Tissue Silk Saree Golden Color)</t>
-  </si>
-  <si>
-    <t>CHR-149</t>
-  </si>
-  <si>
-    <t>SAREE TISSUE EMB (Lavender (light &amp; dark), Red)</t>
-  </si>
-  <si>
-    <t>CHR-150</t>
-  </si>
-  <si>
-    <t>CHIKKANKARI SALWAR</t>
-  </si>
-  <si>
-    <t>Praneetha (L), Rameez Cousin (M)</t>
-  </si>
-  <si>
-    <t>XL, XXL</t>
-  </si>
-  <si>
-    <t>Purple</t>
-  </si>
-  <si>
-    <t>CHR-151</t>
-  </si>
-  <si>
-    <t>Short Kurta</t>
-  </si>
-  <si>
-    <t>Rinsha(M)</t>
-  </si>
-  <si>
-    <t>L,XL,XXL</t>
-  </si>
-  <si>
-    <t>Light Brown colr</t>
-  </si>
-  <si>
-    <t>CHR-152</t>
-  </si>
-  <si>
-    <t>Banarasi (Yellow/Green)</t>
-  </si>
-  <si>
-    <t>Yellow Green</t>
-  </si>
-  <si>
-    <t>CHR-153</t>
-  </si>
-  <si>
-    <t>Ivory &amp; black printed cotton 3-piece salwar set</t>
-  </si>
-  <si>
-    <t>M, XL, XXL</t>
-  </si>
-  <si>
-    <t>CHR-154</t>
-  </si>
-  <si>
-    <t>Dark brown embroidered cotton 3-piece salwar set</t>
-  </si>
-  <si>
-    <t>CHR-155</t>
-  </si>
-  <si>
-    <t>Black cotton 3-piece salwar set with printed dupatta</t>
-  </si>
-  <si>
-    <t>M, L, XL, XXL</t>
-  </si>
-  <si>
-    <t>CHR-156</t>
-  </si>
-  <si>
-    <t>Off-white cotton 2-piece set with blue floral prints</t>
-  </si>
-  <si>
-    <t>Prema(XXL)</t>
-  </si>
-  <si>
-    <t>CHR-157</t>
-  </si>
-  <si>
-    <t>Off-white printed 2-piece kurti set with multicolor pattern</t>
-  </si>
-  <si>
-    <t>M, L, XL, XXL, XXXL</t>
-  </si>
-  <si>
-    <t>CHR-158</t>
-  </si>
-  <si>
-    <t>Olive green cotton 2-piece kurti set with floral prints</t>
-  </si>
-  <si>
-    <t>CHR-159</t>
-  </si>
-  <si>
-    <t>Khadee Saree - Navy Blue and Olive Green</t>
-  </si>
-  <si>
-    <t>CHR-160</t>
-  </si>
-  <si>
-    <t>Khadee Saree - Brown &amp; Black</t>
-  </si>
-  <si>
-    <t>CHR-161</t>
-  </si>
-  <si>
-    <t>Black &amp; Beige Leaf Print Cotton Silk Saree</t>
-  </si>
-  <si>
-    <t>CHR-162</t>
-  </si>
-  <si>
-    <t>Teal &amp; Coral Abstract Print Cotton Silk Saree</t>
-  </si>
-  <si>
-    <t>Partner Settings</t>
-  </si>
-  <si>
-    <t>Share %</t>
-  </si>
-  <si>
-    <t>Total Purchases (Contributions)</t>
-  </si>
-  <si>
-    <t>Target Contributions (by %)</t>
-  </si>
-  <si>
-    <t>Contribution Over/(Under)</t>
-  </si>
-  <si>
-    <t>Profit Share (Completed Only)</t>
-  </si>
-  <si>
-    <t>Net Before Settlements</t>
-  </si>
-  <si>
-    <t>Net Settlements (Received - Paid)</t>
-  </si>
-  <si>
-    <t>Net Position After Settlements</t>
-  </si>
-  <si>
-    <t>Global Settlements Log (used for Contributions, Cash Pool &amp; Profit)</t>
-  </si>
-  <si>
-    <t>Type (Contribution/Cash/Profit)</t>
-  </si>
-  <si>
-    <t>From Partner</t>
-  </si>
-  <si>
-    <t>To Partner</t>
-  </si>
-  <si>
-    <t>Contribution</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>Cash Pool Overview (Completed Sales Only)</t>
-  </si>
-  <si>
-    <t>Cash Collected (Completed Sales)</t>
-  </si>
-  <si>
-    <t>Target Cash Based on %</t>
-  </si>
-  <si>
-    <t>Over/(Under) Collection</t>
-  </si>
-  <si>
-    <t>Net Cash Settlements (Received - Paid)</t>
-  </si>
-  <si>
-    <t>Cash Position After Settlements</t>
-  </si>
-  <si>
-    <t>1. Cash Collected only counts sales with Status = "Completed".</t>
-  </si>
-  <si>
-    <t>2. Target Cash is based on the same partner percentages as profit sharing.</t>
-  </si>
-  <si>
-    <t>3. Over/(Under) is the raw difference before any cash settlements.</t>
-  </si>
-  <si>
-    <t>4. Net Cash Settlements reads Type = "Cash" rows from PartnerShares Settlements Log.</t>
-  </si>
-  <si>
-    <t>5. Cash Position After Settlements = Over/(Under) + Net Cash Settlements.</t>
-  </si>
-  <si>
-    <t>Shinoob</t>
-  </si>
-  <si>
-    <t>Banarasi Yello &amp; Green, Tussar Silk Teal Blue, Green Cotton Silk</t>
-  </si>
-  <si>
-    <t>Green</t>
-  </si>
-  <si>
-    <t>Shinoob (1200)</t>
-  </si>
-  <si>
-    <t>Chris (Goldern with flowers)</t>
-  </si>
-  <si>
-    <t>Matka silk - Blue/Green</t>
-  </si>
-  <si>
-    <t>Golden color tissue with flowers</t>
-  </si>
-  <si>
-    <t>Jothika(Pkd)</t>
-  </si>
-  <si>
-    <t>Matka silk - Blue/red</t>
-  </si>
-  <si>
-    <t>Vineetha(Kottayam)</t>
-  </si>
-  <si>
-    <t>Matka Silk - mustard</t>
-  </si>
-  <si>
-    <t>Amalu(black/maroon), Lethy(Thiruvalla):1550, Vineet(Maroon): 1550, Chris(Yellow) - 1250, Geemol (Black/Violet) - 1500</t>
-  </si>
-  <si>
-    <t>Geemol Mathew (Kottayam)</t>
-  </si>
-  <si>
-    <t>Viscose georgette - Black/Violet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Narayanpett (Ganga Jamuna Alpha) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grey-Black/Red, Maroon-Yellow/Bottle Green, Purple-Yellow/Bottle Green, Bottle Green-Yellow/Red, Peacock Blue-Purple/Golden Yellow  </t>
-  </si>
-  <si>
-    <t>CHR-163</t>
-  </si>
-  <si>
-    <t>Sungudi  (Alice Christy inspired)</t>
-  </si>
-  <si>
-    <t>CHR-164</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Red &amp; Navy Blue </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jute Silk Checked </t>
-  </si>
-  <si>
-    <t>CHR-165</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Violet, Chocolate Brown, Bottle Green  </t>
-  </si>
-  <si>
-    <t>Tant Mix (Bank)</t>
-  </si>
-  <si>
-    <t>CHR-166</t>
-  </si>
-  <si>
-    <t>Tant mix bank - peacock blue</t>
-  </si>
-  <si>
-    <t>Peacock blue with rany pink</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Khadi Cotton (Jar Border)  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yellow, Dark Green, Violet  </t>
-  </si>
-  <si>
-    <t>CHR-167</t>
-  </si>
-  <si>
-    <t>CHR-168</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bengal Cotton (Light Orange Floral)  </t>
-  </si>
-  <si>
-    <t>Orange floral</t>
-  </si>
-  <si>
-    <t>March boosting</t>
-  </si>
-  <si>
-    <t>Susmi. Shinoob (Teal blue), Sarany Hyd -980</t>
-  </si>
-  <si>
-    <t>Tussar silk Green(CHR-70) - 500 advance, Tissue silk non floral(CHR-148)</t>
-  </si>
-  <si>
-    <t>Cotton blend saree yellow - CHR-67</t>
-  </si>
-  <si>
-    <t>Jitha Joy</t>
-  </si>
-  <si>
-    <t>Jitha Joy - 650</t>
-  </si>
-  <si>
-    <t>Mulmul cotton black - CHR-65</t>
-  </si>
-  <si>
-    <t>Deepa Rajan</t>
-  </si>
-  <si>
-    <t>Banarasi Sarees (New Collection)</t>
-  </si>
-  <si>
-    <t>CHR-169</t>
-  </si>
-  <si>
-    <t>Dark biege with bottle green, Biege Maroon combination, Green</t>
-  </si>
-  <si>
-    <t>Rajna - 740, Malini - 980, Baby Khadeeja - 980</t>
-  </si>
-  <si>
-    <t>Shinoob - 1100, Sruthi - 1100</t>
-  </si>
-  <si>
-    <t>Green Cotton Silk (CHR-88)</t>
-  </si>
-  <si>
-    <t>Swapna Binu(Thrisurr)</t>
-  </si>
-  <si>
-    <t>Yellow Green (CHR-146)</t>
-  </si>
-  <si>
-    <t>CHR-170</t>
-  </si>
-  <si>
-    <t>Kerala Saree Temple design</t>
-  </si>
-  <si>
-    <t>CHR-171</t>
-  </si>
-  <si>
-    <t>Kerala Saree Kathakali</t>
-  </si>
-  <si>
-    <t>Kerala Saree floral embroidery</t>
-  </si>
-  <si>
-    <t>CHR-172</t>
-  </si>
-  <si>
-    <t>CHR-173</t>
-  </si>
-  <si>
-    <t>Sungudi Saree (Alice Christy inspired)</t>
-  </si>
-  <si>
-    <t>Rani Pink(1), Jet Black(2), Maroon(3), Dark Green(1), navy Blue (2), Off white (1)</t>
-  </si>
-  <si>
-    <t>Matka Silk Saree collections - old design</t>
-  </si>
-  <si>
-    <t>CHR-174</t>
-  </si>
-  <si>
-    <t>Matka Silk Saree collections - new design</t>
-  </si>
-  <si>
-    <t>Blue/bottle green - Saranya Hyd, Blue/red - Jothika, Mustard - Vineetha, Bottle Green/Golden Yellow - Swapna (Thrissur)-1200</t>
-  </si>
-  <si>
-    <t>Bottle Green/Golden Yellow - 2 
-Black/Golden Yellow - 2
-Navy Blue/Bottle Green - 2</t>
-  </si>
-  <si>
-    <t>Peacok Blue/Maroon - 3
-Purple/Green - 1
-Navy Blue/Maroon - 3
-Maroon/Navy Blue - 1
-Lavender/Violet - 1
-Grey/Blue - 1</t>
-  </si>
-  <si>
-    <t>Banarasi Sarees with Paisley motifs</t>
-  </si>
-  <si>
-    <t>Chokda Rust Orange, Dolla</t>
-  </si>
-  <si>
-    <t>Ranju(1000)</t>
-  </si>
-  <si>
-    <t>burned orange (lotus)</t>
-  </si>
-  <si>
-    <t>Sreeja -Green:1250, Ranju - rust orange:1000</t>
+Pink - Ambika Preman (Pazhanji)
+Rust Orange - Rasha Suresh (Palakkad) - 1299</t>
+  </si>
+  <si>
+    <t>Rasha Suresh (PKD)</t>
+  </si>
+  <si>
+    <t>Banarasi Rust Orange</t>
   </si>
 </sst>
 </file>
@@ -3438,7 +3442,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>135</c:v>
+                  <c:v>136</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>76</c:v>
@@ -3541,7 +3545,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>84</c:v>
+                  <c:v>83</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>68</c:v>
@@ -3882,7 +3886,7 @@
                   <c:v>69946</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>61570.593333333331</c:v>
+                  <c:v>60679.093333333331</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1829</c:v>
@@ -4366,7 +4370,7 @@
                   <c:v>16548</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>20170</c:v>
+                  <c:v>21469</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4806,7 +4810,7 @@
                   <c:v>-5624</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-19226</c:v>
+                  <c:v>-17927</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -5279,10 +5283,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>213</c:v>
+                  <c:v>214</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>157</c:v>
+                  <c:v>156</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6469,7 +6473,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>262752</v>
+        <v>264051</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -6486,7 +6490,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>267282</v>
+        <v>268581</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -6503,7 +6507,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-55935</v>
+        <v>-54636</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -6715,15 +6719,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>241803</v>
+        <v>243102</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>87601.516799999998</v>
+        <v>88034.603399999993</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>154201.48320000002</v>
+        <v>155067.39660000001</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -6731,11 +6735,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>16891.457200000004</v>
+        <v>17757.370599999995</v>
       </c>
       <c r="G26" s="19" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹16,891</v>
+        <v>Pay ₹17,757</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -6749,11 +6753,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>87548.966400000005</v>
+        <v>87981.7932</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-79129.966400000005</v>
+        <v>-79562.7932</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -6761,11 +6765,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-7542.9244000000035</v>
+        <v>-7975.7511999999988</v>
       </c>
       <c r="G27" s="20" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹7,543</v>
+        <v>Receive ₹7,976</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -6779,11 +6783,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>87601.516799999998</v>
+        <v>88034.603399999993</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-75071.516799999998</v>
+        <v>-75504.603399999993</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -6791,11 +6795,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-9348.5327999999863</v>
+        <v>-9781.6193999999814</v>
       </c>
       <c r="G28" s="17" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹9,349</v>
+        <v>Receive ₹9,782</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -6907,7 +6911,7 @@
       </c>
       <c r="B3" s="22">
         <f ca="1">TODAY()</f>
-        <v>46126</v>
+        <v>46127</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -6923,7 +6927,7 @@
       </c>
       <c r="E5" s="23">
         <f>Summary!B4</f>
-        <v>262752</v>
+        <v>264051</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -6932,14 +6936,14 @@
       </c>
       <c r="B6" s="23">
         <f>Summary!B6</f>
-        <v>-55935</v>
+        <v>-54636</v>
       </c>
       <c r="D6" s="21" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="23">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>132265.59333333332</v>
+        <v>131374.09333333332</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -6991,7 +6995,7 @@
       </c>
       <c r="G10" s="23">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -7015,7 +7019,7 @@
       </c>
       <c r="G11" s="29">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -7045,11 +7049,11 @@
       </c>
       <c r="C13" s="29">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$997,"MMM")=$A13)*(YEAR(Sales!$A$2:$A$997)=$B$7)*Sales!$C$2:$C$997),0)</f>
-        <v>20170</v>
+        <v>21469</v>
       </c>
       <c r="D13" s="29">
         <f t="shared" si="0"/>
-        <v>-19226</v>
+        <v>-17927</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1">
@@ -7211,11 +7215,11 @@
       </c>
       <c r="G47" s="32">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H47" s="32">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J47" s="32" t="s">
         <v>96</v>
@@ -7242,7 +7246,7 @@
       </c>
       <c r="K48" s="33">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>61570.593333333331</v>
+        <v>60679.093333333331</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -8189,7 +8193,7 @@
         <v>1000</v>
       </c>
       <c r="D61" s="41" t="s">
-        <v>785</v>
+        <v>780</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="15" customHeight="1">
@@ -13740,7 +13744,7 @@
       <c r="F131" s="50"/>
       <c r="G131" s="50"/>
       <c r="H131" s="52" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="I131" s="50" t="s">
         <v>139</v>
@@ -13951,7 +13955,7 @@
         <v>46113</v>
       </c>
       <c r="B140" s="54" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="C140" s="55">
         <v>3000</v>
@@ -13965,7 +13969,7 @@
       <c r="F140" s="57"/>
       <c r="G140" s="57"/>
       <c r="H140" s="58" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="I140" s="54" t="s">
         <v>139</v>
@@ -13990,7 +13994,7 @@
       <c r="F141" s="50"/>
       <c r="G141" s="50"/>
       <c r="H141" s="52" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="I141" s="50" t="s">
         <v>139</v>
@@ -14001,7 +14005,7 @@
         <v>46119</v>
       </c>
       <c r="B142" s="54" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="C142" s="55">
         <v>1200</v>
@@ -14015,7 +14019,7 @@
       <c r="F142" s="57"/>
       <c r="G142" s="57"/>
       <c r="H142" s="58" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="I142" s="54" t="s">
         <v>139</v>
@@ -14026,7 +14030,7 @@
         <v>46120</v>
       </c>
       <c r="B143" s="50" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="C143" s="51">
         <v>1200</v>
@@ -14040,7 +14044,7 @@
       <c r="F143" s="50"/>
       <c r="G143" s="50"/>
       <c r="H143" s="52" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="I143" s="50" t="s">
         <v>139</v>
@@ -14051,7 +14055,7 @@
         <v>46120</v>
       </c>
       <c r="B144" s="54" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="C144" s="55">
         <v>1500</v>
@@ -14065,7 +14069,7 @@
       <c r="F144" s="57"/>
       <c r="G144" s="57"/>
       <c r="H144" s="58" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="I144" s="54" t="s">
         <v>139</v>
@@ -14090,7 +14094,7 @@
       <c r="F145" s="50"/>
       <c r="G145" s="50"/>
       <c r="H145" s="52" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="I145" s="50" t="s">
         <v>139</v>
@@ -14113,7 +14117,7 @@
       <c r="F146" s="57"/>
       <c r="G146" s="57"/>
       <c r="H146" s="58" t="s">
-        <v>787</v>
+        <v>782</v>
       </c>
       <c r="I146" s="54" t="s">
         <v>311</v>
@@ -14124,7 +14128,7 @@
         <v>46122</v>
       </c>
       <c r="B147" s="50" t="s">
-        <v>789</v>
+        <v>784</v>
       </c>
       <c r="C147" s="51">
         <v>650</v>
@@ -14138,7 +14142,7 @@
       <c r="F147" s="50"/>
       <c r="G147" s="50"/>
       <c r="H147" s="52" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="I147" s="50" t="s">
         <v>139</v>
@@ -14149,7 +14153,7 @@
         <v>46122</v>
       </c>
       <c r="B148" s="54" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="C148" s="55">
         <v>500</v>
@@ -14163,7 +14167,7 @@
       <c r="F148" s="57"/>
       <c r="G148" s="57"/>
       <c r="H148" s="58" t="s">
-        <v>791</v>
+        <v>786</v>
       </c>
       <c r="I148" s="54" t="s">
         <v>139</v>
@@ -14186,7 +14190,7 @@
       <c r="F149" s="50"/>
       <c r="G149" s="50"/>
       <c r="H149" s="52" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
       <c r="I149" s="50" t="s">
         <v>311</v>
@@ -14211,7 +14215,7 @@
       <c r="F150" s="57"/>
       <c r="G150" s="57"/>
       <c r="H150" s="58" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="I150" s="54" t="s">
         <v>139</v>
@@ -14222,7 +14226,7 @@
         <v>46125</v>
       </c>
       <c r="B151" s="50" t="s">
-        <v>799</v>
+        <v>794</v>
       </c>
       <c r="C151" s="51">
         <v>1200</v>
@@ -14236,7 +14240,7 @@
       <c r="F151" s="50"/>
       <c r="G151" s="50"/>
       <c r="H151" s="52" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="I151" s="50" t="s">
         <v>139</v>
@@ -14261,7 +14265,7 @@
       <c r="F152" s="57"/>
       <c r="G152" s="57"/>
       <c r="H152" s="58" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="I152" s="54" t="s">
         <v>139</v>
@@ -14286,7 +14290,7 @@
       <c r="F153" s="50"/>
       <c r="G153" s="50"/>
       <c r="H153" s="52" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="I153" s="50" t="s">
         <v>139</v>
@@ -14311,22 +14315,36 @@
       <c r="F154" s="57"/>
       <c r="G154" s="57"/>
       <c r="H154" s="58" t="s">
-        <v>817</v>
+        <v>812</v>
       </c>
       <c r="I154" s="54" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="155" spans="1:9">
-      <c r="A155" s="49"/>
-      <c r="B155" s="50"/>
-      <c r="C155" s="51"/>
-      <c r="D155" s="50"/>
-      <c r="E155" s="50"/>
+      <c r="A155" s="49">
+        <v>46127</v>
+      </c>
+      <c r="B155" s="50" t="s">
+        <v>820</v>
+      </c>
+      <c r="C155" s="51">
+        <v>1299</v>
+      </c>
+      <c r="D155" s="50" t="s">
+        <v>153</v>
+      </c>
+      <c r="E155" s="50" t="s">
+        <v>49</v>
+      </c>
       <c r="F155" s="50"/>
       <c r="G155" s="50"/>
-      <c r="H155" s="52"/>
-      <c r="I155" s="50"/>
+      <c r="H155" s="52" t="s">
+        <v>821</v>
+      </c>
+      <c r="I155" s="50" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="156" spans="1:9">
       <c r="A156" s="53"/>
@@ -22591,7 +22609,7 @@
         <v>685</v>
       </c>
       <c r="L68" s="83" t="s">
-        <v>790</v>
+        <v>785</v>
       </c>
       <c r="M68" s="83"/>
       <c r="N68" s="83" t="s">
@@ -22749,7 +22767,7 @@
         <v>0</v>
       </c>
       <c r="L71" s="78" t="s">
-        <v>786</v>
+        <v>781</v>
       </c>
       <c r="M71" s="78" t="s">
         <v>49</v>
@@ -22759,7 +22777,7 @@
       </c>
       <c r="O71" s="78"/>
       <c r="P71" s="78" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="Q71" s="78"/>
       <c r="R71" s="78"/>
@@ -23711,7 +23729,7 @@
         <v>0</v>
       </c>
       <c r="L89" s="78" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="M89" s="78"/>
       <c r="N89" s="78" t="s">
@@ -25091,7 +25109,7 @@
         <v>0</v>
       </c>
       <c r="L115" s="78" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="M115" s="78"/>
       <c r="N115" s="78" t="s">
@@ -25104,7 +25122,7 @@
       <c r="S115" s="78"/>
       <c r="T115" s="78"/>
     </row>
-    <row r="116" spans="1:246" ht="135">
+    <row r="116" spans="1:246" ht="150">
       <c r="A116" s="83" t="s">
         <v>599</v>
       </c>
@@ -25121,10 +25139,10 @@
         <v>1400</v>
       </c>
       <c r="F116" s="84">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G116" s="84">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H116" s="83">
         <f t="shared" si="9"/>
@@ -25136,23 +25154,21 @@
       </c>
       <c r="J116" s="83">
         <f t="shared" si="10"/>
-        <v>17830</v>
+        <v>18721.5</v>
       </c>
       <c r="K116" s="83">
         <f t="shared" si="11"/>
-        <v>891.5</v>
+        <v>0</v>
       </c>
       <c r="L116" s="83" t="s">
-        <v>601</v>
+        <v>819</v>
       </c>
       <c r="M116" s="83"/>
       <c r="N116" s="83" t="s">
-        <v>422</v>
+        <v>337</v>
       </c>
       <c r="O116" s="83"/>
-      <c r="P116" s="83" t="s">
-        <v>602</v>
-      </c>
+      <c r="P116" s="83"/>
       <c r="Q116" s="83"/>
       <c r="R116" s="83"/>
       <c r="S116" s="83"/>
@@ -25160,10 +25176,10 @@
     </row>
     <row r="117" spans="1:246" ht="15">
       <c r="A117" s="78" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="B117" s="78" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="C117" s="78" t="s">
         <v>95</v>
@@ -25212,10 +25228,10 @@
     </row>
     <row r="118" spans="1:246" ht="15">
       <c r="A118" s="83" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="B118" s="83" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="C118" s="83" t="s">
         <v>95</v>
@@ -25249,7 +25265,7 @@
         <v>1047.9000000000001</v>
       </c>
       <c r="L118" s="83" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="M118" s="83"/>
       <c r="N118" s="83" t="s">
@@ -25257,7 +25273,7 @@
       </c>
       <c r="O118" s="83"/>
       <c r="P118" s="83" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="Q118" s="83"/>
       <c r="R118" s="83"/>
@@ -25266,10 +25282,10 @@
     </row>
     <row r="119" spans="1:246" ht="15">
       <c r="A119" s="78" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="B119" s="78" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="C119" s="78" t="s">
         <v>95</v>
@@ -25318,10 +25334,10 @@
     </row>
     <row r="120" spans="1:246" ht="30">
       <c r="A120" s="83" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="B120" s="83" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="C120" s="83" t="s">
         <v>95</v>
@@ -25355,7 +25371,7 @@
         <v>4189.5333333333301</v>
       </c>
       <c r="L120" s="83" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="M120" s="83" t="s">
         <v>49</v>
@@ -25365,7 +25381,7 @@
       </c>
       <c r="O120" s="83"/>
       <c r="P120" s="83" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="Q120" s="83"/>
       <c r="R120" s="83"/>
@@ -25374,10 +25390,10 @@
     </row>
     <row r="121" spans="1:246" ht="15">
       <c r="A121" s="78" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="B121" s="78" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="C121" s="78" t="s">
         <v>95</v>
@@ -25411,7 +25427,7 @@
         <v>0</v>
       </c>
       <c r="L121" s="78" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="M121" s="78"/>
       <c r="N121" s="78" t="s">
@@ -25419,7 +25435,7 @@
       </c>
       <c r="O121" s="78"/>
       <c r="P121" s="78" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="Q121" s="78"/>
       <c r="R121" s="78"/>
@@ -25428,10 +25444,10 @@
     </row>
     <row r="122" spans="1:246" ht="15">
       <c r="A122" s="83" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="B122" s="83" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="C122" s="83" t="s">
         <v>96</v>
@@ -25465,14 +25481,14 @@
         <v>3525</v>
       </c>
       <c r="L122" s="83" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="M122" s="83"/>
       <c r="N122" s="83" t="s">
         <v>422</v>
       </c>
       <c r="O122" s="83" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="P122" s="83"/>
       <c r="Q122" s="83"/>
@@ -25482,10 +25498,10 @@
     </row>
     <row r="123" spans="1:246" s="67" customFormat="1" ht="75">
       <c r="A123" s="89" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="B123" s="89" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="C123" s="89" t="s">
         <v>95</v>
@@ -25519,7 +25535,7 @@
         <v>891.44</v>
       </c>
       <c r="L123" s="89" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="M123" s="89"/>
       <c r="N123" s="89" t="s">
@@ -25760,10 +25776,10 @@
     </row>
     <row r="124" spans="1:246" s="69" customFormat="1" ht="30">
       <c r="A124" s="91" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="B124" s="91" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="C124" s="91" t="s">
         <v>95</v>
@@ -25797,7 +25813,7 @@
         <v>0</v>
       </c>
       <c r="L124" s="91" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="M124" s="91"/>
       <c r="N124" s="91" t="s">
@@ -26040,10 +26056,10 @@
     </row>
     <row r="125" spans="1:246" s="67" customFormat="1" ht="15">
       <c r="A125" s="89" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B125" s="89" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="C125" s="89" t="s">
         <v>95</v>
@@ -26077,7 +26093,7 @@
         <v>0</v>
       </c>
       <c r="L125" s="89" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="M125" s="89"/>
       <c r="N125" s="89" t="s">
@@ -26085,7 +26101,7 @@
       </c>
       <c r="O125" s="89"/>
       <c r="P125" s="89" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="Q125" s="89"/>
       <c r="R125" s="89"/>
@@ -26320,10 +26336,10 @@
     </row>
     <row r="126" spans="1:246" ht="15">
       <c r="A126" s="91" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="B126" s="83" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="C126" s="83" t="s">
         <v>96</v>
@@ -26357,14 +26373,14 @@
         <v>0</v>
       </c>
       <c r="L126" s="83" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="M126" s="83"/>
       <c r="N126" s="83" t="s">
         <v>337</v>
       </c>
       <c r="O126" s="83" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="P126" s="83"/>
       <c r="Q126" s="83"/>
@@ -26374,10 +26390,10 @@
     </row>
     <row r="127" spans="1:246" ht="15">
       <c r="A127" s="89" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="B127" s="78" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="C127" s="78" t="s">
         <v>96</v>
@@ -26428,10 +26444,10 @@
     </row>
     <row r="128" spans="1:246" ht="15">
       <c r="A128" s="91" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="B128" s="83" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="C128" s="83" t="s">
         <v>95</v>
@@ -26478,10 +26494,10 @@
     </row>
     <row r="129" spans="1:20" ht="15">
       <c r="A129" s="89" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="B129" s="78" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="C129" s="78" t="s">
         <v>95</v>
@@ -26515,7 +26531,7 @@
         <v>0</v>
       </c>
       <c r="L129" s="78" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="M129" s="78"/>
       <c r="N129" s="78" t="s">
@@ -26530,10 +26546,10 @@
     </row>
     <row r="130" spans="1:20" ht="15">
       <c r="A130" s="91" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B130" s="83" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="C130" s="83" t="s">
         <v>95</v>
@@ -26567,7 +26583,7 @@
         <v>0</v>
       </c>
       <c r="L130" s="83" t="s">
-        <v>818</v>
+        <v>813</v>
       </c>
       <c r="M130" s="83"/>
       <c r="N130" s="83" t="s">
@@ -26582,10 +26598,10 @@
     </row>
     <row r="131" spans="1:20" ht="15">
       <c r="A131" s="89" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="B131" s="78" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="C131" s="78" t="s">
         <v>95</v>
@@ -26632,10 +26648,10 @@
     </row>
     <row r="132" spans="1:20" ht="15">
       <c r="A132" s="91" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="B132" s="83" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="C132" s="83" t="s">
         <v>95</v>
@@ -26669,7 +26685,7 @@
         <v>0</v>
       </c>
       <c r="L132" s="83" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="M132" s="83"/>
       <c r="N132" s="83" t="s">
@@ -26684,10 +26700,10 @@
     </row>
     <row r="133" spans="1:20" ht="15">
       <c r="A133" s="89" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="B133" s="78" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="C133" s="78" t="s">
         <v>95</v>
@@ -26734,10 +26750,10 @@
     </row>
     <row r="134" spans="1:20" ht="15">
       <c r="A134" s="91" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="B134" s="83" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="C134" s="83" t="s">
         <v>95</v>
@@ -26784,10 +26800,10 @@
     </row>
     <row r="135" spans="1:20" ht="15">
       <c r="A135" s="89" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="B135" s="78" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="C135" s="78" t="s">
         <v>95</v>
@@ -26821,7 +26837,7 @@
         <v>0</v>
       </c>
       <c r="L135" s="78" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="M135" s="78"/>
       <c r="N135" s="78" t="s">
@@ -26836,10 +26852,10 @@
     </row>
     <row r="136" spans="1:20" ht="15">
       <c r="A136" s="91" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="B136" s="83" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="C136" s="83" t="s">
         <v>95</v>
@@ -26873,7 +26889,7 @@
         <v>908</v>
       </c>
       <c r="L136" s="83" t="s">
-        <v>820</v>
+        <v>815</v>
       </c>
       <c r="M136" s="83"/>
       <c r="N136" s="83" t="s">
@@ -26881,7 +26897,7 @@
       </c>
       <c r="O136" s="83"/>
       <c r="P136" s="83" t="s">
-        <v>819</v>
+        <v>814</v>
       </c>
       <c r="Q136" s="83"/>
       <c r="R136" s="83"/>
@@ -26890,10 +26906,10 @@
     </row>
     <row r="137" spans="1:20" ht="15">
       <c r="A137" s="89" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="B137" s="78" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="C137" s="78" t="s">
         <v>95</v>
@@ -26942,10 +26958,10 @@
     </row>
     <row r="138" spans="1:20" ht="15">
       <c r="A138" s="91" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="B138" s="83" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="C138" s="83" t="s">
         <v>95</v>
@@ -26992,10 +27008,10 @@
     </row>
     <row r="139" spans="1:20" ht="15">
       <c r="A139" s="89" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="B139" s="78" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="C139" s="78" t="s">
         <v>95</v>
@@ -27044,10 +27060,10 @@
     </row>
     <row r="140" spans="1:20" ht="15">
       <c r="A140" s="91" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="B140" s="83" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="C140" s="83" t="s">
         <v>95</v>
@@ -27081,7 +27097,7 @@
         <v>699</v>
       </c>
       <c r="L140" s="83" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="M140" s="83"/>
       <c r="N140" s="83" t="s">
@@ -27096,10 +27112,10 @@
     </row>
     <row r="141" spans="1:20" ht="15">
       <c r="A141" s="89" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="B141" s="78" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="C141" s="78" t="s">
         <v>95</v>
@@ -27146,10 +27162,10 @@
     </row>
     <row r="142" spans="1:20" ht="15">
       <c r="A142" s="83" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="B142" s="83" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="C142" s="83" t="s">
         <v>95</v>
@@ -27183,7 +27199,7 @@
         <v>600</v>
       </c>
       <c r="L142" s="83" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="M142" s="83"/>
       <c r="N142" s="83" t="s">
@@ -27200,10 +27216,10 @@
     </row>
     <row r="143" spans="1:20" ht="15">
       <c r="A143" s="78" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B143" s="78" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="C143" s="78" t="s">
         <v>95</v>
@@ -27250,10 +27266,10 @@
     </row>
     <row r="144" spans="1:20" ht="15">
       <c r="A144" s="83" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="B144" s="83" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="C144" s="83" t="s">
         <v>95</v>
@@ -27300,7 +27316,7 @@
     </row>
     <row r="145" spans="1:20" ht="15">
       <c r="A145" s="78" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="B145" s="78" t="s">
         <v>293</v>
@@ -27352,10 +27368,10 @@
     </row>
     <row r="146" spans="1:20" ht="15">
       <c r="A146" s="83" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="B146" s="83" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="C146" s="83" t="s">
         <v>95</v>
@@ -27389,7 +27405,7 @@
         <v>1522</v>
       </c>
       <c r="L146" s="83" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="M146" s="83"/>
       <c r="N146" s="83" t="s">
@@ -27404,10 +27420,10 @@
     </row>
     <row r="147" spans="1:20" ht="45">
       <c r="A147" s="78" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="B147" s="78" t="s">
-        <v>810</v>
+        <v>805</v>
       </c>
       <c r="C147" s="78" t="s">
         <v>95</v>
@@ -27441,7 +27457,7 @@
         <v>5033</v>
       </c>
       <c r="L147" s="78" t="s">
-        <v>813</v>
+        <v>808</v>
       </c>
       <c r="M147" s="78"/>
       <c r="N147" s="78" t="s">
@@ -27449,7 +27465,7 @@
       </c>
       <c r="O147" s="78"/>
       <c r="P147" s="78" t="s">
-        <v>814</v>
+        <v>809</v>
       </c>
       <c r="Q147" s="78"/>
       <c r="R147" s="78"/>
@@ -27458,10 +27474,10 @@
     </row>
     <row r="148" spans="1:20" ht="15">
       <c r="A148" s="83" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="B148" s="83" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="C148" s="83" t="s">
         <v>95</v>
@@ -27495,7 +27511,7 @@
         <v>502</v>
       </c>
       <c r="L148" s="83" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="M148" s="83"/>
       <c r="N148" s="83" t="s">
@@ -27510,10 +27526,10 @@
     </row>
     <row r="149" spans="1:20" ht="15">
       <c r="A149" s="78" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="B149" s="78" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="C149" s="78" t="s">
         <v>95</v>
@@ -27547,7 +27563,7 @@
         <v>2048</v>
       </c>
       <c r="L149" s="78" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="M149" s="78"/>
       <c r="N149" s="78" t="s">
@@ -27562,10 +27578,10 @@
     </row>
     <row r="150" spans="1:20" ht="15">
       <c r="A150" s="83" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="B150" s="83" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="C150" s="83" t="s">
         <v>95</v>
@@ -27612,10 +27628,10 @@
     </row>
     <row r="151" spans="1:20" ht="15">
       <c r="A151" s="78" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="B151" s="78" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="C151" s="78" t="s">
         <v>96</v>
@@ -27649,17 +27665,17 @@
         <v>1290</v>
       </c>
       <c r="L151" s="78" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="M151" s="78"/>
       <c r="N151" s="78" t="s">
         <v>422</v>
       </c>
       <c r="O151" s="78" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="P151" s="78" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="Q151" s="78"/>
       <c r="R151" s="78"/>
@@ -27668,10 +27684,10 @@
     </row>
     <row r="152" spans="1:20" ht="15">
       <c r="A152" s="83" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="B152" s="83" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="C152" s="83" t="s">
         <v>97</v>
@@ -27705,17 +27721,17 @@
         <v>885</v>
       </c>
       <c r="L152" s="83" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="M152" s="83"/>
       <c r="N152" s="83" t="s">
         <v>422</v>
       </c>
       <c r="O152" s="83" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="P152" s="83" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="Q152" s="83"/>
       <c r="R152" s="83"/>
@@ -27724,10 +27740,10 @@
     </row>
     <row r="153" spans="1:20" ht="15">
       <c r="A153" s="78" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="B153" s="78" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="C153" s="78" t="s">
         <v>95</v>
@@ -27761,7 +27777,7 @@
         <v>891.5</v>
       </c>
       <c r="L153" s="78" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="M153" s="78"/>
       <c r="N153" s="78" t="s">
@@ -27769,7 +27785,7 @@
       </c>
       <c r="O153" s="78"/>
       <c r="P153" s="78" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="Q153" s="78"/>
       <c r="R153" s="78"/>
@@ -27778,10 +27794,10 @@
     </row>
     <row r="154" spans="1:20" ht="15">
       <c r="A154" s="83" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="B154" s="83" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="C154" s="83" t="s">
         <v>96</v>
@@ -27820,7 +27836,7 @@
         <v>506</v>
       </c>
       <c r="O154" s="83" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="P154" s="83"/>
       <c r="Q154" s="83"/>
@@ -27830,10 +27846,10 @@
     </row>
     <row r="155" spans="1:20" ht="15">
       <c r="A155" s="78" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="B155" s="78" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="C155" s="78" t="s">
         <v>96</v>
@@ -27872,7 +27888,7 @@
         <v>506</v>
       </c>
       <c r="O155" s="78" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="P155" s="78"/>
       <c r="Q155" s="78"/>
@@ -27882,10 +27898,10 @@
     </row>
     <row r="156" spans="1:20" ht="15">
       <c r="A156" s="83" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="B156" s="83" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="C156" s="83" t="s">
         <v>96</v>
@@ -27924,7 +27940,7 @@
         <v>506</v>
       </c>
       <c r="O156" s="83" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="P156" s="83"/>
       <c r="Q156" s="83"/>
@@ -27934,10 +27950,10 @@
     </row>
     <row r="157" spans="1:20" ht="15">
       <c r="A157" s="78" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="B157" s="78" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="C157" s="78" t="s">
         <v>96</v>
@@ -27971,14 +27987,14 @@
         <v>1575</v>
       </c>
       <c r="L157" s="78" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="M157" s="78"/>
       <c r="N157" s="78" t="s">
         <v>422</v>
       </c>
       <c r="O157" s="78" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="P157" s="78"/>
       <c r="Q157" s="78"/>
@@ -27988,10 +28004,10 @@
     </row>
     <row r="158" spans="1:20" ht="15">
       <c r="A158" s="83" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="B158" s="83" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="C158" s="83" t="s">
         <v>96</v>
@@ -28030,7 +28046,7 @@
         <v>506</v>
       </c>
       <c r="O158" s="83" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="P158" s="83"/>
       <c r="Q158" s="83"/>
@@ -28040,10 +28056,10 @@
     </row>
     <row r="159" spans="1:20" ht="15">
       <c r="A159" s="78" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="B159" s="78" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="C159" s="78" t="s">
         <v>96</v>
@@ -28082,7 +28098,7 @@
         <v>506</v>
       </c>
       <c r="O159" s="78" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="P159" s="78"/>
       <c r="Q159" s="78"/>
@@ -28092,10 +28108,10 @@
     </row>
     <row r="160" spans="1:20" ht="15">
       <c r="A160" s="83" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="B160" s="83" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="C160" s="83" t="s">
         <v>95</v>
@@ -28144,10 +28160,10 @@
     </row>
     <row r="161" spans="1:20" ht="15">
       <c r="A161" s="78" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="B161" s="78" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="C161" s="78" t="s">
         <v>95</v>
@@ -28196,10 +28212,10 @@
     </row>
     <row r="162" spans="1:20" ht="15">
       <c r="A162" s="83" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="B162" s="83" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="C162" s="83" t="s">
         <v>95</v>
@@ -28246,10 +28262,10 @@
     </row>
     <row r="163" spans="1:20" ht="15">
       <c r="A163" s="78" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="B163" s="78" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="C163" s="78" t="s">
         <v>95</v>
@@ -28296,10 +28312,10 @@
     </row>
     <row r="164" spans="1:20" ht="60">
       <c r="A164" s="83" t="s">
-        <v>768</v>
+        <v>765</v>
       </c>
       <c r="B164" s="83" t="s">
-        <v>766</v>
+        <v>818</v>
       </c>
       <c r="C164" s="83" t="s">
         <v>95</v>
@@ -28339,7 +28355,7 @@
       </c>
       <c r="O164" s="83"/>
       <c r="P164" s="83" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
       <c r="Q164" s="83"/>
       <c r="R164" s="83"/>
@@ -28348,10 +28364,10 @@
     </row>
     <row r="165" spans="1:20" ht="15">
       <c r="A165" s="78" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
       <c r="B165" s="78" t="s">
-        <v>808</v>
+        <v>803</v>
       </c>
       <c r="C165" s="78" t="s">
         <v>95</v>
@@ -28393,7 +28409,7 @@
       </c>
       <c r="O165" s="78"/>
       <c r="P165" s="78" t="s">
-        <v>771</v>
+        <v>768</v>
       </c>
       <c r="Q165" s="78"/>
       <c r="R165" s="78"/>
@@ -28402,10 +28418,10 @@
     </row>
     <row r="166" spans="1:20" ht="15">
       <c r="A166" s="83" t="s">
-        <v>773</v>
+        <v>769</v>
       </c>
       <c r="B166" s="83" t="s">
-        <v>772</v>
+        <v>816</v>
       </c>
       <c r="C166" s="83" t="s">
         <v>95</v>
@@ -28445,7 +28461,7 @@
       </c>
       <c r="O166" s="83"/>
       <c r="P166" s="83" t="s">
-        <v>774</v>
+        <v>770</v>
       </c>
       <c r="Q166" s="83"/>
       <c r="R166" s="83"/>
@@ -28454,10 +28470,10 @@
     </row>
     <row r="167" spans="1:20" ht="15">
       <c r="A167" s="78" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="B167" s="78" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
       <c r="C167" s="78" t="s">
         <v>95</v>
@@ -28491,7 +28507,7 @@
         <v>2220</v>
       </c>
       <c r="L167" s="78" t="s">
-        <v>796</v>
+        <v>791</v>
       </c>
       <c r="M167" s="78"/>
       <c r="N167" s="78" t="s">
@@ -28499,7 +28515,7 @@
       </c>
       <c r="O167" s="78"/>
       <c r="P167" s="78" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="Q167" s="78"/>
       <c r="R167" s="78"/>
@@ -28508,10 +28524,10 @@
     </row>
     <row r="168" spans="1:20" ht="15">
       <c r="A168" s="83" t="s">
-        <v>781</v>
+        <v>776</v>
       </c>
       <c r="B168" s="83" t="s">
-        <v>779</v>
+        <v>817</v>
       </c>
       <c r="C168" s="83" t="s">
         <v>95</v>
@@ -28551,7 +28567,7 @@
       </c>
       <c r="O168" s="83"/>
       <c r="P168" s="83" t="s">
-        <v>780</v>
+        <v>775</v>
       </c>
       <c r="Q168" s="83"/>
       <c r="R168" s="83"/>
@@ -28560,10 +28576,10 @@
     </row>
     <row r="169" spans="1:20" ht="15">
       <c r="A169" s="78" t="s">
-        <v>782</v>
+        <v>777</v>
       </c>
       <c r="B169" s="78" t="s">
-        <v>783</v>
+        <v>778</v>
       </c>
       <c r="C169" s="78" t="s">
         <v>95</v>
@@ -28603,7 +28619,7 @@
       </c>
       <c r="O169" s="78"/>
       <c r="P169" s="78" t="s">
-        <v>784</v>
+        <v>779</v>
       </c>
       <c r="Q169" s="78"/>
       <c r="R169" s="78"/>
@@ -28612,10 +28628,10 @@
     </row>
     <row r="170" spans="1:20" ht="30">
       <c r="A170" s="83" t="s">
-        <v>794</v>
+        <v>789</v>
       </c>
       <c r="B170" s="83" t="s">
-        <v>793</v>
+        <v>788</v>
       </c>
       <c r="C170" s="83" t="s">
         <v>95</v>
@@ -28655,7 +28671,7 @@
       </c>
       <c r="O170" s="83"/>
       <c r="P170" s="83" t="s">
-        <v>795</v>
+        <v>790</v>
       </c>
       <c r="Q170" s="83"/>
       <c r="R170" s="83"/>
@@ -28664,10 +28680,10 @@
     </row>
     <row r="171" spans="1:20" ht="15">
       <c r="A171" s="78" t="s">
-        <v>801</v>
+        <v>796</v>
       </c>
       <c r="B171" s="83" t="s">
-        <v>816</v>
+        <v>811</v>
       </c>
       <c r="C171" s="78" t="s">
         <v>95</v>
@@ -28714,10 +28730,10 @@
     </row>
     <row r="172" spans="1:20" ht="15">
       <c r="A172" s="83" t="s">
-        <v>803</v>
+        <v>798</v>
       </c>
       <c r="B172" s="83" t="s">
-        <v>802</v>
+        <v>797</v>
       </c>
       <c r="C172" s="83" t="s">
         <v>95</v>
@@ -28764,10 +28780,10 @@
     </row>
     <row r="173" spans="1:20" ht="15">
       <c r="A173" s="78" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="B173" s="78" t="s">
-        <v>804</v>
+        <v>799</v>
       </c>
       <c r="C173" s="78" t="s">
         <v>95</v>
@@ -28814,10 +28830,10 @@
     </row>
     <row r="174" spans="1:20" ht="15">
       <c r="A174" s="83" t="s">
-        <v>807</v>
+        <v>802</v>
       </c>
       <c r="B174" s="83" t="s">
-        <v>805</v>
+        <v>800</v>
       </c>
       <c r="C174" s="83" t="s">
         <v>95</v>
@@ -28864,10 +28880,10 @@
     </row>
     <row r="175" spans="1:20" ht="90">
       <c r="A175" s="78" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="B175" s="78" t="s">
-        <v>812</v>
+        <v>807</v>
       </c>
       <c r="C175" s="78" t="s">
         <v>95</v>
@@ -28907,14 +28923,14 @@
       </c>
       <c r="O175" s="78"/>
       <c r="P175" s="78" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="Q175" s="78"/>
       <c r="R175" s="78"/>
       <c r="S175" s="78"/>
       <c r="T175" s="78"/>
     </row>
-    <row r="176" spans="1:20" ht="15">
+    <row r="176" spans="1:20">
       <c r="A176" s="83"/>
       <c r="B176" s="83"/>
       <c r="C176" s="83"/>
@@ -28936,7 +28952,7 @@
       <c r="S176" s="83"/>
       <c r="T176" s="83"/>
     </row>
-    <row r="177" spans="1:20" ht="15">
+    <row r="177" spans="1:20">
       <c r="A177" s="78"/>
       <c r="B177" s="78"/>
       <c r="C177" s="78"/>
@@ -28958,7 +28974,7 @@
       <c r="S177" s="78"/>
       <c r="T177" s="78"/>
     </row>
-    <row r="178" spans="1:20" ht="15">
+    <row r="178" spans="1:20">
       <c r="A178" s="83"/>
       <c r="B178" s="83"/>
       <c r="C178" s="83"/>
@@ -28980,7 +28996,7 @@
       <c r="S178" s="83"/>
       <c r="T178" s="83"/>
     </row>
-    <row r="179" spans="1:20" ht="15">
+    <row r="179" spans="1:20">
       <c r="A179" s="78"/>
       <c r="B179" s="78"/>
       <c r="C179" s="78"/>
@@ -29002,7 +29018,7 @@
       <c r="S179" s="78"/>
       <c r="T179" s="78"/>
     </row>
-    <row r="180" spans="1:20" ht="15">
+    <row r="180" spans="1:20">
       <c r="A180" s="83"/>
       <c r="B180" s="83"/>
       <c r="C180" s="83"/>
@@ -29024,7 +29040,7 @@
       <c r="S180" s="83"/>
       <c r="T180" s="83"/>
     </row>
-    <row r="181" spans="1:20" ht="15">
+    <row r="181" spans="1:20">
       <c r="A181" s="78"/>
       <c r="B181" s="78"/>
       <c r="C181" s="78"/>
@@ -29046,7 +29062,7 @@
       <c r="S181" s="78"/>
       <c r="T181" s="78"/>
     </row>
-    <row r="182" spans="1:20" ht="15">
+    <row r="182" spans="1:20">
       <c r="A182" s="83"/>
       <c r="B182" s="83"/>
       <c r="C182" s="83"/>
@@ -29068,7 +29084,7 @@
       <c r="S182" s="83"/>
       <c r="T182" s="83"/>
     </row>
-    <row r="183" spans="1:20" ht="15">
+    <row r="183" spans="1:20">
       <c r="A183" s="78"/>
       <c r="B183" s="78"/>
       <c r="C183" s="78"/>
@@ -29090,7 +29106,7 @@
       <c r="S183" s="78"/>
       <c r="T183" s="78"/>
     </row>
-    <row r="184" spans="1:20" ht="15">
+    <row r="184" spans="1:20">
       <c r="A184" s="83"/>
       <c r="B184" s="83"/>
       <c r="C184" s="83"/>
@@ -29112,7 +29128,7 @@
       <c r="S184" s="83"/>
       <c r="T184" s="83"/>
     </row>
-    <row r="185" spans="1:20" ht="15">
+    <row r="185" spans="1:20">
       <c r="A185" s="78"/>
       <c r="B185" s="78"/>
       <c r="C185" s="78"/>
@@ -29134,7 +29150,7 @@
       <c r="S185" s="78"/>
       <c r="T185" s="78"/>
     </row>
-    <row r="186" spans="1:20" ht="15">
+    <row r="186" spans="1:20">
       <c r="A186" s="83"/>
       <c r="B186" s="83"/>
       <c r="C186" s="83"/>
@@ -29156,7 +29172,7 @@
       <c r="S186" s="83"/>
       <c r="T186" s="83"/>
     </row>
-    <row r="187" spans="1:20" ht="15">
+    <row r="187" spans="1:20">
       <c r="A187" s="78"/>
       <c r="B187" s="78"/>
       <c r="C187" s="78"/>
@@ -29178,7 +29194,7 @@
       <c r="S187" s="78"/>
       <c r="T187" s="78"/>
     </row>
-    <row r="188" spans="1:20" ht="15">
+    <row r="188" spans="1:20">
       <c r="A188" s="83"/>
       <c r="B188" s="83"/>
       <c r="C188" s="83"/>
@@ -29200,7 +29216,7 @@
       <c r="S188" s="83"/>
       <c r="T188" s="83"/>
     </row>
-    <row r="189" spans="1:20" ht="15">
+    <row r="189" spans="1:20">
       <c r="A189" s="78"/>
       <c r="B189" s="78"/>
       <c r="C189" s="78"/>
@@ -36481,7 +36497,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1">
       <c r="A1" s="94" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="B1" s="94"/>
     </row>
@@ -36490,7 +36506,7 @@
         <v>42</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="13.5" customHeight="1">
@@ -36522,25 +36538,25 @@
         <v>42</v>
       </c>
       <c r="B7" s="72" t="s">
+        <v>726</v>
+      </c>
+      <c r="C7" s="72" t="s">
+        <v>727</v>
+      </c>
+      <c r="D7" s="72" t="s">
         <v>728</v>
       </c>
-      <c r="C7" s="72" t="s">
+      <c r="E7" s="72" t="s">
         <v>729</v>
       </c>
-      <c r="D7" s="72" t="s">
+      <c r="F7" s="72" t="s">
         <v>730</v>
       </c>
-      <c r="E7" s="72" t="s">
+      <c r="G7" s="72" t="s">
         <v>731</v>
       </c>
-      <c r="F7" s="72" t="s">
+      <c r="H7" s="72" t="s">
         <v>732</v>
-      </c>
-      <c r="G7" s="72" t="s">
-        <v>733</v>
-      </c>
-      <c r="H7" s="72" t="s">
-        <v>734</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="13.5" customHeight="1">
@@ -36644,7 +36660,7 @@
     </row>
     <row r="12" spans="1:8" s="74" customFormat="1" ht="15.75" customHeight="1">
       <c r="A12" s="95" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="B12" s="95"/>
       <c r="C12" s="95"/>
@@ -36657,13 +36673,13 @@
         <v>98</v>
       </c>
       <c r="B13" s="72" t="s">
+        <v>734</v>
+      </c>
+      <c r="C13" s="72" t="s">
+        <v>735</v>
+      </c>
+      <c r="D13" s="72" t="s">
         <v>736</v>
-      </c>
-      <c r="C13" s="72" t="s">
-        <v>737</v>
-      </c>
-      <c r="D13" s="72" t="s">
-        <v>738</v>
       </c>
       <c r="E13" s="72" t="s">
         <v>99</v>
@@ -36677,7 +36693,7 @@
         <v>45952</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>51</v>
@@ -36695,7 +36711,7 @@
         <v>45952</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>51</v>
@@ -36749,7 +36765,7 @@
         <v>45970</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>50</v>
@@ -36767,7 +36783,7 @@
         <v>45970</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>50</v>
@@ -36785,7 +36801,7 @@
         <v>45973</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>50</v>
@@ -36803,7 +36819,7 @@
         <v>45973</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>49</v>
@@ -36821,7 +36837,7 @@
         <v>46058</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>51</v>
@@ -36857,7 +36873,7 @@
         <v>46059</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>49</v>
@@ -36893,7 +36909,7 @@
         <v>46093</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>50</v>
@@ -36911,7 +36927,7 @@
         <v>46093</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>51</v>
@@ -36994,7 +37010,7 @@
     </row>
     <row r="58" spans="2:2" ht="13.5" customHeight="1">
       <c r="B58" s="6" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
     </row>
   </sheetData>
@@ -37024,7 +37040,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="13.5" customHeight="1">
       <c r="A1" s="77" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="73" customFormat="1" ht="13.5" customHeight="1">
@@ -37032,22 +37048,22 @@
         <v>42</v>
       </c>
       <c r="B3" s="72" t="s">
+        <v>740</v>
+      </c>
+      <c r="C3" s="72" t="s">
+        <v>725</v>
+      </c>
+      <c r="D3" s="72" t="s">
+        <v>741</v>
+      </c>
+      <c r="E3" s="72" t="s">
         <v>742</v>
       </c>
-      <c r="C3" s="72" t="s">
-        <v>727</v>
-      </c>
-      <c r="D3" s="72" t="s">
+      <c r="F3" s="72" t="s">
         <v>743</v>
       </c>
-      <c r="E3" s="72" t="s">
+      <c r="G3" s="72" t="s">
         <v>744</v>
-      </c>
-      <c r="F3" s="72" t="s">
-        <v>745</v>
-      </c>
-      <c r="G3" s="72" t="s">
-        <v>746</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="13.5" customHeight="1">
@@ -37056,7 +37072,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>241803</v>
+        <v>243102</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -37064,11 +37080,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>87601.516799999998</v>
+        <v>88034.603399999993</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>154201.48320000002</v>
+        <v>155067.39660000001</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -37076,7 +37092,7 @@
       </c>
       <c r="G4" s="16">
         <f>E4+F4</f>
-        <v>16891.457200000004</v>
+        <v>17757.370599999995</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -37093,11 +37109,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>87548.966400000005</v>
+        <v>87981.7932</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-79129.966400000005</v>
+        <v>-79562.7932</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -37105,7 +37121,7 @@
       </c>
       <c r="G5" s="18">
         <f>E5+F5</f>
-        <v>-7542.9244000000035</v>
+        <v>-7975.7511999999988</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -37122,11 +37138,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>87601.516799999998</v>
+        <v>88034.603399999993</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-75071.516799999998</v>
+        <v>-75504.603399999993</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -37134,7 +37150,7 @@
       </c>
       <c r="G6" s="16">
         <f>E6+F6</f>
-        <v>-9348.5327999999863</v>
+        <v>-9781.6193999999814</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">
@@ -37144,27 +37160,27 @@
     </row>
     <row r="10" spans="1:7" ht="13.5" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="13.5" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="13.5" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="13.5" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="13.5" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Jute Kurti and Manipuri sales update
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Apr26.xlsx
+++ b/docs/Chiraath-Summary-Apr26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4B309B2-16EC-9E4C-872B-B77A0164A203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3EA06F4-4E1B-7841-9022-4A0D7B3DE4D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2065" uniqueCount="826">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2075" uniqueCount="830">
   <si>
     <t>Notes:</t>
   </si>
@@ -1704,12 +1704,6 @@
   </si>
   <si>
     <t>Kurti blue Jute</t>
-  </si>
-  <si>
-    <t>Sourabhya (XL - 580)</t>
-  </si>
-  <si>
-    <t>L, XXL</t>
   </si>
   <si>
     <t>CHR-93</t>
@@ -2544,6 +2538,24 @@
   </si>
   <si>
     <t>CHR-117 - Tie &amp; Dye blue</t>
+  </si>
+  <si>
+    <t>Shini</t>
+  </si>
+  <si>
+    <t>Sourabhya (XL - 580), Shini (L-450)</t>
+  </si>
+  <si>
+    <t>Jute Kurti(L)?</t>
+  </si>
+  <si>
+    <t>Shanta Priya</t>
+  </si>
+  <si>
+    <t>Shantha Priya</t>
+  </si>
+  <si>
+    <t>Manipuri Silk</t>
   </si>
 </sst>
 </file>
@@ -3454,13 +3466,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>135</c:v>
+                  <c:v>136</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>76</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3557,13 +3569,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>84</c:v>
+                  <c:v>83</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>68</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3898,10 +3910,10 @@
                   <c:v>69946</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>61726.993333333332</c:v>
+                  <c:v>60912.993333333332</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1829</c:v>
+                  <c:v>1357</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4382,7 +4394,7 @@
                   <c:v>16248</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>25689</c:v>
+                  <c:v>27239</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4822,7 +4834,7 @@
                   <c:v>-5924</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-13707</c:v>
+                  <c:v>-12157</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -5295,10 +5307,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>213</c:v>
+                  <c:v>215</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>157</c:v>
+                  <c:v>155</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6485,7 +6497,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>266861</v>
+        <v>267961</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -6502,7 +6514,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>272501</v>
+        <v>274051</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -6519,7 +6531,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-51826</v>
+        <v>-50726</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -6731,15 +6743,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>245912</v>
+        <v>247012</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>88971.457399999999</v>
+        <v>89338.19739999999</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>156940.54259999999</v>
+        <v>157673.8026</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -6747,11 +6759,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>19630.516599999974</v>
+        <v>20363.776599999983</v>
       </c>
       <c r="G26" s="19" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹19,631</v>
+        <v>Pay ₹20,364</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -6765,11 +6777,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>88918.085200000001</v>
+        <v>89284.605200000005</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-80499.085200000001</v>
+        <v>-80865.605200000005</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -6777,11 +6789,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-8912.0432000000001</v>
+        <v>-9278.5632000000041</v>
       </c>
       <c r="G27" s="20" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹8,912</v>
+        <v>Receive ₹9,279</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -6795,11 +6807,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>88971.457399999999</v>
+        <v>89338.19739999999</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-76441.457399999999</v>
+        <v>-76808.19739999999</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -6807,11 +6819,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-10718.473399999988</v>
+        <v>-11085.213399999979</v>
       </c>
       <c r="G28" s="17" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹10,718</v>
+        <v>Receive ₹11,085</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -6923,7 +6935,7 @@
       </c>
       <c r="B3" s="22">
         <f ca="1">TODAY()</f>
-        <v>46131</v>
+        <v>46132</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -6939,7 +6951,7 @@
       </c>
       <c r="E5" s="23">
         <f>Summary!B4</f>
-        <v>266861</v>
+        <v>267961</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -6948,14 +6960,14 @@
       </c>
       <c r="B6" s="23">
         <f>Summary!B6</f>
-        <v>-51826</v>
+        <v>-50726</v>
       </c>
       <c r="D6" s="21" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="23">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>130326.19333333331</v>
+        <v>129040.19333333331</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -7007,7 +7019,7 @@
       </c>
       <c r="G10" s="23">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -7031,7 +7043,7 @@
       </c>
       <c r="G11" s="29">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -7061,11 +7073,11 @@
       </c>
       <c r="C13" s="29">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$997,"MMM")=$A13)*(YEAR(Sales!$A$2:$A$997)=$B$7)*Sales!$C$2:$C$997),0)</f>
-        <v>25689</v>
+        <v>27239</v>
       </c>
       <c r="D13" s="29">
         <f t="shared" si="0"/>
-        <v>-13707</v>
+        <v>-12157</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1">
@@ -7227,11 +7239,11 @@
       </c>
       <c r="G47" s="32">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H47" s="32">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J47" s="32" t="s">
         <v>96</v>
@@ -7258,7 +7270,7 @@
       </c>
       <c r="K48" s="33">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>61726.993333333332</v>
+        <v>60912.993333333332</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -7267,18 +7279,18 @@
       </c>
       <c r="G49" s="32">
         <f>SUMIF(INVENTORY!C:C, F49, INVENTORY!F:F)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H49" s="32">
         <f>SUMIF(INVENTORY!C:C, F49, INVENTORY!G:G)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J49" s="32" t="s">
         <v>97</v>
       </c>
       <c r="K49" s="33">
         <f t="array" ref="K49">SUMPRODUCT((INVENTORY!$C$2:$C$477=J49)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>1829</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="55" spans="5:12" ht="15" customHeight="1">
@@ -8205,7 +8217,7 @@
         <v>1000</v>
       </c>
       <c r="D61" s="41" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="15" customHeight="1">
@@ -13756,7 +13768,7 @@
       <c r="F131" s="50"/>
       <c r="G131" s="50"/>
       <c r="H131" s="52" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="I131" s="50" t="s">
         <v>139</v>
@@ -13967,7 +13979,7 @@
         <v>46113</v>
       </c>
       <c r="B140" s="54" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="C140" s="55">
         <v>3000</v>
@@ -13981,7 +13993,7 @@
       <c r="F140" s="57"/>
       <c r="G140" s="57"/>
       <c r="H140" s="58" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="I140" s="54" t="s">
         <v>139</v>
@@ -14006,7 +14018,7 @@
       <c r="F141" s="50"/>
       <c r="G141" s="50"/>
       <c r="H141" s="52" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="I141" s="50" t="s">
         <v>139</v>
@@ -14017,7 +14029,7 @@
         <v>46119</v>
       </c>
       <c r="B142" s="54" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="C142" s="55">
         <v>1200</v>
@@ -14031,7 +14043,7 @@
       <c r="F142" s="57"/>
       <c r="G142" s="57"/>
       <c r="H142" s="58" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="I142" s="54" t="s">
         <v>139</v>
@@ -14042,7 +14054,7 @@
         <v>46120</v>
       </c>
       <c r="B143" s="50" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="C143" s="51">
         <v>1200</v>
@@ -14056,7 +14068,7 @@
       <c r="F143" s="50"/>
       <c r="G143" s="50"/>
       <c r="H143" s="52" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="I143" s="50" t="s">
         <v>139</v>
@@ -14067,7 +14079,7 @@
         <v>46120</v>
       </c>
       <c r="B144" s="54" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="C144" s="55">
         <v>1500</v>
@@ -14081,7 +14093,7 @@
       <c r="F144" s="57"/>
       <c r="G144" s="57"/>
       <c r="H144" s="58" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="I144" s="54" t="s">
         <v>139</v>
@@ -14106,7 +14118,7 @@
       <c r="F145" s="50"/>
       <c r="G145" s="50"/>
       <c r="H145" s="52" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="I145" s="50" t="s">
         <v>139</v>
@@ -14129,7 +14141,7 @@
       <c r="F146" s="57"/>
       <c r="G146" s="57"/>
       <c r="H146" s="58" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="I146" s="54" t="s">
         <v>311</v>
@@ -14140,7 +14152,7 @@
         <v>46122</v>
       </c>
       <c r="B147" s="50" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="C147" s="51">
         <v>650</v>
@@ -14154,7 +14166,7 @@
       <c r="F147" s="50"/>
       <c r="G147" s="50"/>
       <c r="H147" s="52" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
       <c r="I147" s="50" t="s">
         <v>139</v>
@@ -14165,7 +14177,7 @@
         <v>46122</v>
       </c>
       <c r="B148" s="54" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="C148" s="55">
         <v>500</v>
@@ -14179,7 +14191,7 @@
       <c r="F148" s="57"/>
       <c r="G148" s="57"/>
       <c r="H148" s="58" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="I148" s="54" t="s">
         <v>139</v>
@@ -14202,7 +14214,7 @@
       <c r="F149" s="50"/>
       <c r="G149" s="50"/>
       <c r="H149" s="52" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="I149" s="50" t="s">
         <v>311</v>
@@ -14227,7 +14239,7 @@
       <c r="F150" s="57"/>
       <c r="G150" s="57"/>
       <c r="H150" s="58" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
       <c r="I150" s="54" t="s">
         <v>139</v>
@@ -14238,7 +14250,7 @@
         <v>46125</v>
       </c>
       <c r="B151" s="50" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="C151" s="51">
         <v>1200</v>
@@ -14252,7 +14264,7 @@
       <c r="F151" s="50"/>
       <c r="G151" s="50"/>
       <c r="H151" s="52" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="I151" s="50" t="s">
         <v>139</v>
@@ -14277,7 +14289,7 @@
       <c r="F152" s="57"/>
       <c r="G152" s="57"/>
       <c r="H152" s="58" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="I152" s="54" t="s">
         <v>139</v>
@@ -14302,7 +14314,7 @@
       <c r="F153" s="50"/>
       <c r="G153" s="50"/>
       <c r="H153" s="52" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="I153" s="50" t="s">
         <v>139</v>
@@ -14327,7 +14339,7 @@
       <c r="F154" s="57"/>
       <c r="G154" s="57"/>
       <c r="H154" s="58" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="I154" s="54" t="s">
         <v>139</v>
@@ -14338,7 +14350,7 @@
         <v>46127</v>
       </c>
       <c r="B155" s="50" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
       <c r="C155" s="51">
         <v>1299</v>
@@ -14352,7 +14364,7 @@
       <c r="F155" s="50"/>
       <c r="G155" s="50"/>
       <c r="H155" s="52" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="I155" s="50" t="s">
         <v>139</v>
@@ -14363,7 +14375,7 @@
         <v>46129</v>
       </c>
       <c r="B156" s="54" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="C156" s="55">
         <v>980</v>
@@ -14377,7 +14389,7 @@
       <c r="F156" s="57"/>
       <c r="G156" s="57"/>
       <c r="H156" s="58" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="I156" s="54" t="s">
         <v>139</v>
@@ -14388,7 +14400,7 @@
         <v>46129</v>
       </c>
       <c r="B157" s="50" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
       <c r="C157" s="51">
         <v>980</v>
@@ -14400,7 +14412,7 @@
       <c r="F157" s="50"/>
       <c r="G157" s="50"/>
       <c r="H157" s="52" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="I157" s="50" t="s">
         <v>311</v>
@@ -14423,7 +14435,7 @@
       <c r="F158" s="57"/>
       <c r="G158" s="57"/>
       <c r="H158" s="58" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="I158" s="54" t="s">
         <v>311</v>
@@ -14434,7 +14446,7 @@
         <v>46130</v>
       </c>
       <c r="B159" s="50" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
       <c r="C159" s="51">
         <v>1280</v>
@@ -14448,33 +14460,59 @@
       <c r="F159" s="50"/>
       <c r="G159" s="50"/>
       <c r="H159" s="52" t="s">
-        <v>825</v>
+        <v>823</v>
       </c>
       <c r="I159" s="50" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="160" spans="1:9">
-      <c r="A160" s="53"/>
-      <c r="B160" s="54"/>
-      <c r="C160" s="55"/>
+    <row r="160" spans="1:9" ht="16">
+      <c r="A160" s="53">
+        <v>46131</v>
+      </c>
+      <c r="B160" s="54" t="s">
+        <v>824</v>
+      </c>
+      <c r="C160" s="55">
+        <v>450</v>
+      </c>
       <c r="D160" s="54"/>
-      <c r="E160" s="54"/>
+      <c r="E160" s="54" t="s">
+        <v>49</v>
+      </c>
       <c r="F160" s="57"/>
       <c r="G160" s="57"/>
-      <c r="H160" s="58"/>
-      <c r="I160" s="54"/>
+      <c r="H160" s="58" t="s">
+        <v>826</v>
+      </c>
+      <c r="I160" s="54" t="s">
+        <v>311</v>
+      </c>
     </row>
     <row r="161" spans="1:9">
-      <c r="A161" s="49"/>
-      <c r="B161" s="50"/>
-      <c r="C161" s="51"/>
-      <c r="D161" s="50"/>
-      <c r="E161" s="50"/>
+      <c r="A161" s="49">
+        <v>46132</v>
+      </c>
+      <c r="B161" s="50" t="s">
+        <v>827</v>
+      </c>
+      <c r="C161" s="51">
+        <v>1100</v>
+      </c>
+      <c r="D161" s="50" t="s">
+        <v>153</v>
+      </c>
+      <c r="E161" s="50" t="s">
+        <v>49</v>
+      </c>
       <c r="F161" s="50"/>
       <c r="G161" s="50"/>
-      <c r="H161" s="52"/>
-      <c r="I161" s="50"/>
+      <c r="H161" s="52" t="s">
+        <v>829</v>
+      </c>
+      <c r="I161" s="50" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="162" spans="1:9">
       <c r="A162" s="53"/>
@@ -22673,7 +22711,7 @@
         <v>685</v>
       </c>
       <c r="L68" s="83" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="M68" s="83"/>
       <c r="N68" s="83" t="s">
@@ -22831,7 +22869,7 @@
         <v>0</v>
       </c>
       <c r="L71" s="78" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="M71" s="78" t="s">
         <v>49</v>
@@ -22841,7 +22879,7 @@
       </c>
       <c r="O71" s="78"/>
       <c r="P71" s="78" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="Q71" s="78"/>
       <c r="R71" s="78"/>
@@ -23793,7 +23831,7 @@
         <v>0</v>
       </c>
       <c r="L89" s="78" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
       <c r="M89" s="78"/>
       <c r="N89" s="78" t="s">
@@ -23979,10 +24017,10 @@
         <v>650</v>
       </c>
       <c r="F93" s="85">
+        <v>2</v>
+      </c>
+      <c r="G93" s="85">
         <v>1</v>
-      </c>
-      <c r="G93" s="85">
-        <v>2</v>
       </c>
       <c r="H93" s="78">
         <f t="shared" si="6"/>
@@ -23994,21 +24032,21 @@
       </c>
       <c r="J93" s="78">
         <f t="shared" si="7"/>
-        <v>472</v>
+        <v>944</v>
       </c>
       <c r="K93" s="78">
         <f t="shared" si="8"/>
-        <v>944</v>
+        <v>472</v>
       </c>
       <c r="L93" s="78" t="s">
-        <v>552</v>
+        <v>825</v>
       </c>
       <c r="M93" s="78"/>
       <c r="N93" s="83" t="s">
         <v>422</v>
       </c>
       <c r="O93" s="78" t="s">
-        <v>553</v>
+        <v>207</v>
       </c>
       <c r="P93" s="78"/>
       <c r="Q93" s="78"/>
@@ -24018,10 +24056,10 @@
     </row>
     <row r="94" spans="1:20" ht="15">
       <c r="A94" s="83" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B94" s="83" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="C94" s="83" t="s">
         <v>95</v>
@@ -24070,10 +24108,10 @@
     </row>
     <row r="95" spans="1:20" ht="15">
       <c r="A95" s="78" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="B95" s="78" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="C95" s="78" t="s">
         <v>95</v>
@@ -24107,7 +24145,7 @@
         <v>0</v>
       </c>
       <c r="L95" s="78" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="M95" s="78"/>
       <c r="N95" s="78" t="s">
@@ -24122,10 +24160,10 @@
     </row>
     <row r="96" spans="1:20" ht="15">
       <c r="A96" s="83" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="B96" s="83" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="C96" s="83" t="s">
         <v>95</v>
@@ -24172,10 +24210,10 @@
     </row>
     <row r="97" spans="1:20" ht="15">
       <c r="A97" s="78" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="B97" s="78" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C97" s="78" t="s">
         <v>95</v>
@@ -24224,10 +24262,10 @@
     </row>
     <row r="98" spans="1:20" ht="15">
       <c r="A98" s="83" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="B98" s="83" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="C98" s="83" t="s">
         <v>96</v>
@@ -24278,10 +24316,10 @@
     </row>
     <row r="99" spans="1:20" ht="15">
       <c r="A99" s="78" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="B99" s="78" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="C99" s="78" t="s">
         <v>96</v>
@@ -24332,10 +24370,10 @@
     </row>
     <row r="100" spans="1:20" ht="15">
       <c r="A100" s="83" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="B100" s="83" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="C100" s="83" t="s">
         <v>96</v>
@@ -24386,10 +24424,10 @@
     </row>
     <row r="101" spans="1:20" ht="15">
       <c r="A101" s="78" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="B101" s="78" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="C101" s="78" t="s">
         <v>96</v>
@@ -24440,10 +24478,10 @@
     </row>
     <row r="102" spans="1:20" ht="15">
       <c r="A102" s="83" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="B102" s="83" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="C102" s="83" t="s">
         <v>96</v>
@@ -24494,10 +24532,10 @@
     </row>
     <row r="103" spans="1:20" ht="15">
       <c r="A103" s="78" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="B103" s="78" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="C103" s="78" t="s">
         <v>96</v>
@@ -24548,10 +24586,10 @@
     </row>
     <row r="104" spans="1:20" ht="15">
       <c r="A104" s="83" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="B104" s="83" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="C104" s="83" t="s">
         <v>96</v>
@@ -24602,10 +24640,10 @@
     </row>
     <row r="105" spans="1:20" ht="15">
       <c r="A105" s="78" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="B105" s="78" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="C105" s="78" t="s">
         <v>96</v>
@@ -24656,10 +24694,10 @@
     </row>
     <row r="106" spans="1:20" ht="15">
       <c r="A106" s="83" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="B106" s="83" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="C106" s="83" t="s">
         <v>96</v>
@@ -24708,10 +24746,10 @@
     </row>
     <row r="107" spans="1:20" ht="15">
       <c r="A107" s="78" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="B107" s="78" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="C107" s="78" t="s">
         <v>96</v>
@@ -24762,10 +24800,10 @@
     </row>
     <row r="108" spans="1:20" ht="15">
       <c r="A108" s="83" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B108" s="83" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="C108" s="83" t="s">
         <v>96</v>
@@ -24816,10 +24854,10 @@
     </row>
     <row r="109" spans="1:20" ht="15">
       <c r="A109" s="78" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="B109" s="78" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="C109" s="78" t="s">
         <v>96</v>
@@ -24870,10 +24908,10 @@
     </row>
     <row r="110" spans="1:20" ht="15">
       <c r="A110" s="83" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="B110" s="83" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="C110" s="83" t="s">
         <v>96</v>
@@ -24924,10 +24962,10 @@
     </row>
     <row r="111" spans="1:20" ht="15">
       <c r="A111" s="78" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="B111" s="78" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="C111" s="78" t="s">
         <v>96</v>
@@ -24978,10 +25016,10 @@
     </row>
     <row r="112" spans="1:20" ht="15">
       <c r="A112" s="83" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="B112" s="83" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="C112" s="83" t="s">
         <v>96</v>
@@ -25030,10 +25068,10 @@
     </row>
     <row r="113" spans="1:246" ht="15">
       <c r="A113" s="78" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B113" s="78" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="C113" s="78" t="s">
         <v>96</v>
@@ -25084,10 +25122,10 @@
     </row>
     <row r="114" spans="1:246" ht="15">
       <c r="A114" s="83" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="B114" s="83" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="C114" s="83" t="s">
         <v>95</v>
@@ -25136,10 +25174,10 @@
     </row>
     <row r="115" spans="1:246" ht="30">
       <c r="A115" s="78" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B115" s="78" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="C115" s="78" t="s">
         <v>95</v>
@@ -25173,7 +25211,7 @@
         <v>0</v>
       </c>
       <c r="L115" s="78" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="M115" s="78"/>
       <c r="N115" s="78" t="s">
@@ -25188,10 +25226,10 @@
     </row>
     <row r="116" spans="1:246" ht="150">
       <c r="A116" s="83" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="B116" s="83" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="C116" s="83" t="s">
         <v>95</v>
@@ -25225,7 +25263,7 @@
         <v>0</v>
       </c>
       <c r="L116" s="83" t="s">
-        <v>817</v>
+        <v>815</v>
       </c>
       <c r="M116" s="83"/>
       <c r="N116" s="83" t="s">
@@ -25240,10 +25278,10 @@
     </row>
     <row r="117" spans="1:246" ht="15">
       <c r="A117" s="78" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="B117" s="78" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="C117" s="78" t="s">
         <v>95</v>
@@ -25292,10 +25330,10 @@
     </row>
     <row r="118" spans="1:246" ht="15">
       <c r="A118" s="83" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="B118" s="83" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="C118" s="83" t="s">
         <v>95</v>
@@ -25329,7 +25367,7 @@
         <v>2095.8000000000002</v>
       </c>
       <c r="L118" s="83" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
       <c r="M118" s="83"/>
       <c r="N118" s="83" t="s">
@@ -25337,7 +25375,7 @@
       </c>
       <c r="O118" s="83"/>
       <c r="P118" s="83" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="Q118" s="83"/>
       <c r="R118" s="83"/>
@@ -25346,10 +25384,10 @@
     </row>
     <row r="119" spans="1:246" ht="15">
       <c r="A119" s="78" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="B119" s="78" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="C119" s="78" t="s">
         <v>95</v>
@@ -25398,10 +25436,10 @@
     </row>
     <row r="120" spans="1:246" ht="30">
       <c r="A120" s="83" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="B120" s="83" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="C120" s="83" t="s">
         <v>95</v>
@@ -25435,7 +25473,7 @@
         <v>4189.5333333333301</v>
       </c>
       <c r="L120" s="83" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="M120" s="83" t="s">
         <v>49</v>
@@ -25445,7 +25483,7 @@
       </c>
       <c r="O120" s="83"/>
       <c r="P120" s="83" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="Q120" s="83"/>
       <c r="R120" s="83"/>
@@ -25454,10 +25492,10 @@
     </row>
     <row r="121" spans="1:246" ht="15">
       <c r="A121" s="78" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="B121" s="78" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="C121" s="78" t="s">
         <v>95</v>
@@ -25491,7 +25529,7 @@
         <v>0</v>
       </c>
       <c r="L121" s="78" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="M121" s="78"/>
       <c r="N121" s="78" t="s">
@@ -25499,7 +25537,7 @@
       </c>
       <c r="O121" s="78"/>
       <c r="P121" s="78" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="Q121" s="78"/>
       <c r="R121" s="78"/>
@@ -25508,10 +25546,10 @@
     </row>
     <row r="122" spans="1:246" ht="15">
       <c r="A122" s="83" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="B122" s="83" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="C122" s="83" t="s">
         <v>96</v>
@@ -25545,14 +25583,14 @@
         <v>3525</v>
       </c>
       <c r="L122" s="83" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="M122" s="83"/>
       <c r="N122" s="83" t="s">
         <v>422</v>
       </c>
       <c r="O122" s="83" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="P122" s="83"/>
       <c r="Q122" s="83"/>
@@ -25562,10 +25600,10 @@
     </row>
     <row r="123" spans="1:246" s="67" customFormat="1" ht="75">
       <c r="A123" s="89" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="B123" s="89" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="C123" s="89" t="s">
         <v>95</v>
@@ -25599,7 +25637,7 @@
         <v>891.44</v>
       </c>
       <c r="L123" s="89" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="M123" s="89"/>
       <c r="N123" s="89" t="s">
@@ -25840,10 +25878,10 @@
     </row>
     <row r="124" spans="1:246" s="69" customFormat="1" ht="30">
       <c r="A124" s="91" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="B124" s="91" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="C124" s="91" t="s">
         <v>95</v>
@@ -25877,7 +25915,7 @@
         <v>0</v>
       </c>
       <c r="L124" s="91" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="M124" s="91"/>
       <c r="N124" s="91" t="s">
@@ -26120,10 +26158,10 @@
     </row>
     <row r="125" spans="1:246" s="67" customFormat="1" ht="15">
       <c r="A125" s="89" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="B125" s="89" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="C125" s="89" t="s">
         <v>95</v>
@@ -26157,7 +26195,7 @@
         <v>0</v>
       </c>
       <c r="L125" s="89" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="M125" s="89"/>
       <c r="N125" s="89" t="s">
@@ -26165,7 +26203,7 @@
       </c>
       <c r="O125" s="89"/>
       <c r="P125" s="89" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="Q125" s="89"/>
       <c r="R125" s="89"/>
@@ -26400,10 +26438,10 @@
     </row>
     <row r="126" spans="1:246" ht="15">
       <c r="A126" s="91" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="B126" s="83" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="C126" s="83" t="s">
         <v>96</v>
@@ -26437,14 +26475,14 @@
         <v>0</v>
       </c>
       <c r="L126" s="83" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="M126" s="83"/>
       <c r="N126" s="83" t="s">
         <v>337</v>
       </c>
       <c r="O126" s="83" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="P126" s="83"/>
       <c r="Q126" s="83"/>
@@ -26454,10 +26492,10 @@
     </row>
     <row r="127" spans="1:246" ht="15">
       <c r="A127" s="89" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="B127" s="78" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="C127" s="78" t="s">
         <v>96</v>
@@ -26508,10 +26546,10 @@
     </row>
     <row r="128" spans="1:246" ht="15">
       <c r="A128" s="91" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="B128" s="83" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="C128" s="83" t="s">
         <v>95</v>
@@ -26558,10 +26596,10 @@
     </row>
     <row r="129" spans="1:20" ht="15">
       <c r="A129" s="89" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="B129" s="78" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="C129" s="78" t="s">
         <v>95</v>
@@ -26595,7 +26633,7 @@
         <v>0</v>
       </c>
       <c r="L129" s="78" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="M129" s="78"/>
       <c r="N129" s="78" t="s">
@@ -26610,10 +26648,10 @@
     </row>
     <row r="130" spans="1:20" ht="15">
       <c r="A130" s="91" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="B130" s="83" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="C130" s="83" t="s">
         <v>95</v>
@@ -26647,7 +26685,7 @@
         <v>0</v>
       </c>
       <c r="L130" s="83" t="s">
-        <v>811</v>
+        <v>809</v>
       </c>
       <c r="M130" s="83"/>
       <c r="N130" s="83" t="s">
@@ -26662,10 +26700,10 @@
     </row>
     <row r="131" spans="1:20" ht="15">
       <c r="A131" s="89" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="B131" s="78" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="C131" s="78" t="s">
         <v>95</v>
@@ -26712,10 +26750,10 @@
     </row>
     <row r="132" spans="1:20" ht="15">
       <c r="A132" s="91" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="B132" s="83" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="C132" s="83" t="s">
         <v>95</v>
@@ -26749,7 +26787,7 @@
         <v>0</v>
       </c>
       <c r="L132" s="83" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="M132" s="83"/>
       <c r="N132" s="83" t="s">
@@ -26764,10 +26802,10 @@
     </row>
     <row r="133" spans="1:20" ht="15">
       <c r="A133" s="89" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="B133" s="78" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="C133" s="78" t="s">
         <v>95</v>
@@ -26814,10 +26852,10 @@
     </row>
     <row r="134" spans="1:20" ht="15">
       <c r="A134" s="91" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="B134" s="83" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C134" s="83" t="s">
         <v>95</v>
@@ -26864,10 +26902,10 @@
     </row>
     <row r="135" spans="1:20" ht="15">
       <c r="A135" s="89" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="B135" s="78" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="C135" s="78" t="s">
         <v>95</v>
@@ -26901,7 +26939,7 @@
         <v>0</v>
       </c>
       <c r="L135" s="78" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="M135" s="78"/>
       <c r="N135" s="78" t="s">
@@ -26916,10 +26954,10 @@
     </row>
     <row r="136" spans="1:20" ht="15">
       <c r="A136" s="91" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="B136" s="83" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="C136" s="83" t="s">
         <v>95</v>
@@ -26953,7 +26991,7 @@
         <v>908</v>
       </c>
       <c r="L136" s="83" t="s">
-        <v>813</v>
+        <v>811</v>
       </c>
       <c r="M136" s="83"/>
       <c r="N136" s="83" t="s">
@@ -26961,7 +26999,7 @@
       </c>
       <c r="O136" s="83"/>
       <c r="P136" s="83" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
       <c r="Q136" s="83"/>
       <c r="R136" s="83"/>
@@ -26970,10 +27008,10 @@
     </row>
     <row r="137" spans="1:20" ht="15">
       <c r="A137" s="89" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="B137" s="78" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="C137" s="78" t="s">
         <v>95</v>
@@ -27022,10 +27060,10 @@
     </row>
     <row r="138" spans="1:20" ht="15">
       <c r="A138" s="91" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="B138" s="83" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="C138" s="83" t="s">
         <v>95</v>
@@ -27037,10 +27075,10 @@
         <v>1100</v>
       </c>
       <c r="F138" s="92">
+        <v>1</v>
+      </c>
+      <c r="G138" s="92">
         <v>0</v>
-      </c>
-      <c r="G138" s="92">
-        <v>1</v>
       </c>
       <c r="H138" s="91">
         <f t="shared" si="12"/>
@@ -27052,16 +27090,18 @@
       </c>
       <c r="J138" s="91">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>814</v>
       </c>
       <c r="K138" s="91">
         <f t="shared" si="14"/>
-        <v>814</v>
-      </c>
-      <c r="L138" s="83"/>
+        <v>0</v>
+      </c>
+      <c r="L138" s="83" t="s">
+        <v>828</v>
+      </c>
       <c r="M138" s="83"/>
       <c r="N138" s="83" t="s">
-        <v>506</v>
+        <v>337</v>
       </c>
       <c r="O138" s="83"/>
       <c r="P138" s="83"/>
@@ -27072,10 +27112,10 @@
     </row>
     <row r="139" spans="1:20" ht="15">
       <c r="A139" s="89" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="B139" s="78" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="C139" s="78" t="s">
         <v>95</v>
@@ -27124,10 +27164,10 @@
     </row>
     <row r="140" spans="1:20" ht="15">
       <c r="A140" s="91" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="B140" s="83" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="C140" s="83" t="s">
         <v>95</v>
@@ -27161,7 +27201,7 @@
         <v>699</v>
       </c>
       <c r="L140" s="83" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="M140" s="83"/>
       <c r="N140" s="83" t="s">
@@ -27176,10 +27216,10 @@
     </row>
     <row r="141" spans="1:20" ht="15">
       <c r="A141" s="89" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="B141" s="78" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="C141" s="78" t="s">
         <v>95</v>
@@ -27226,10 +27266,10 @@
     </row>
     <row r="142" spans="1:20" ht="15">
       <c r="A142" s="83" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="B142" s="83" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="C142" s="83" t="s">
         <v>95</v>
@@ -27263,7 +27303,7 @@
         <v>600</v>
       </c>
       <c r="L142" s="83" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="M142" s="83"/>
       <c r="N142" s="83" t="s">
@@ -27280,10 +27320,10 @@
     </row>
     <row r="143" spans="1:20" ht="15">
       <c r="A143" s="78" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="B143" s="78" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="C143" s="78" t="s">
         <v>95</v>
@@ -27330,10 +27370,10 @@
     </row>
     <row r="144" spans="1:20" ht="15">
       <c r="A144" s="83" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="B144" s="83" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="C144" s="83" t="s">
         <v>95</v>
@@ -27380,7 +27420,7 @@
     </row>
     <row r="145" spans="1:20" ht="15">
       <c r="A145" s="78" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="B145" s="78" t="s">
         <v>293</v>
@@ -27432,10 +27472,10 @@
     </row>
     <row r="146" spans="1:20" ht="15">
       <c r="A146" s="83" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="B146" s="83" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="C146" s="83" t="s">
         <v>95</v>
@@ -27469,7 +27509,7 @@
         <v>1522</v>
       </c>
       <c r="L146" s="83" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="M146" s="83"/>
       <c r="N146" s="83" t="s">
@@ -27484,10 +27524,10 @@
     </row>
     <row r="147" spans="1:20" ht="45">
       <c r="A147" s="78" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="B147" s="78" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="C147" s="78" t="s">
         <v>95</v>
@@ -27521,7 +27561,7 @@
         <v>5033</v>
       </c>
       <c r="L147" s="78" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
       <c r="M147" s="78"/>
       <c r="N147" s="78" t="s">
@@ -27529,7 +27569,7 @@
       </c>
       <c r="O147" s="78"/>
       <c r="P147" s="78" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="Q147" s="78"/>
       <c r="R147" s="78"/>
@@ -27538,10 +27578,10 @@
     </row>
     <row r="148" spans="1:20" ht="15">
       <c r="A148" s="83" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="B148" s="83" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="C148" s="83" t="s">
         <v>95</v>
@@ -27575,7 +27615,7 @@
         <v>502</v>
       </c>
       <c r="L148" s="83" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="M148" s="83"/>
       <c r="N148" s="83" t="s">
@@ -27590,10 +27630,10 @@
     </row>
     <row r="149" spans="1:20" ht="15">
       <c r="A149" s="78" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="B149" s="78" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="C149" s="78" t="s">
         <v>95</v>
@@ -27627,7 +27667,7 @@
         <v>2048</v>
       </c>
       <c r="L149" s="78" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="M149" s="78"/>
       <c r="N149" s="78" t="s">
@@ -27642,10 +27682,10 @@
     </row>
     <row r="150" spans="1:20" ht="15">
       <c r="A150" s="83" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B150" s="83" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="C150" s="83" t="s">
         <v>95</v>
@@ -27692,10 +27732,10 @@
     </row>
     <row r="151" spans="1:20" ht="15">
       <c r="A151" s="78" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="B151" s="78" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="C151" s="78" t="s">
         <v>96</v>
@@ -27729,17 +27769,17 @@
         <v>1290</v>
       </c>
       <c r="L151" s="78" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="M151" s="78"/>
       <c r="N151" s="78" t="s">
         <v>422</v>
       </c>
       <c r="O151" s="78" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="P151" s="78" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="Q151" s="78"/>
       <c r="R151" s="78"/>
@@ -27748,10 +27788,10 @@
     </row>
     <row r="152" spans="1:20" ht="15">
       <c r="A152" s="83" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="B152" s="83" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="C152" s="83" t="s">
         <v>97</v>
@@ -27785,17 +27825,17 @@
         <v>885</v>
       </c>
       <c r="L152" s="83" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="M152" s="83"/>
       <c r="N152" s="83" t="s">
         <v>422</v>
       </c>
       <c r="O152" s="83" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="P152" s="83" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="Q152" s="83"/>
       <c r="R152" s="83"/>
@@ -27804,10 +27844,10 @@
     </row>
     <row r="153" spans="1:20" ht="15">
       <c r="A153" s="78" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="B153" s="78" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="C153" s="78" t="s">
         <v>95</v>
@@ -27841,7 +27881,7 @@
         <v>891.5</v>
       </c>
       <c r="L153" s="78" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="M153" s="78"/>
       <c r="N153" s="78" t="s">
@@ -27849,7 +27889,7 @@
       </c>
       <c r="O153" s="78"/>
       <c r="P153" s="78" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="Q153" s="78"/>
       <c r="R153" s="78"/>
@@ -27858,10 +27898,10 @@
     </row>
     <row r="154" spans="1:20" ht="15">
       <c r="A154" s="83" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="B154" s="83" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="C154" s="83" t="s">
         <v>96</v>
@@ -27900,7 +27940,7 @@
         <v>506</v>
       </c>
       <c r="O154" s="83" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="P154" s="83"/>
       <c r="Q154" s="83"/>
@@ -27910,10 +27950,10 @@
     </row>
     <row r="155" spans="1:20" ht="15">
       <c r="A155" s="78" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="B155" s="78" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="C155" s="78" t="s">
         <v>96</v>
@@ -27952,7 +27992,7 @@
         <v>506</v>
       </c>
       <c r="O155" s="78" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="P155" s="78"/>
       <c r="Q155" s="78"/>
@@ -27962,10 +28002,10 @@
     </row>
     <row r="156" spans="1:20" ht="15">
       <c r="A156" s="83" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="B156" s="83" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="C156" s="83" t="s">
         <v>96</v>
@@ -28004,7 +28044,7 @@
         <v>506</v>
       </c>
       <c r="O156" s="83" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="P156" s="83"/>
       <c r="Q156" s="83"/>
@@ -28014,10 +28054,10 @@
     </row>
     <row r="157" spans="1:20" ht="15">
       <c r="A157" s="78" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="B157" s="78" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="C157" s="78" t="s">
         <v>96</v>
@@ -28051,14 +28091,14 @@
         <v>1575</v>
       </c>
       <c r="L157" s="78" t="s">
-        <v>822</v>
+        <v>820</v>
       </c>
       <c r="M157" s="78"/>
       <c r="N157" s="78" t="s">
         <v>422</v>
       </c>
       <c r="O157" s="78" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="P157" s="78"/>
       <c r="Q157" s="78"/>
@@ -28068,10 +28108,10 @@
     </row>
     <row r="158" spans="1:20" ht="15">
       <c r="A158" s="83" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="B158" s="83" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="C158" s="83" t="s">
         <v>96</v>
@@ -28110,7 +28150,7 @@
         <v>506</v>
       </c>
       <c r="O158" s="83" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="P158" s="83"/>
       <c r="Q158" s="83"/>
@@ -28120,10 +28160,10 @@
     </row>
     <row r="159" spans="1:20" ht="15">
       <c r="A159" s="78" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="B159" s="78" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="C159" s="78" t="s">
         <v>96</v>
@@ -28162,7 +28202,7 @@
         <v>506</v>
       </c>
       <c r="O159" s="78" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="P159" s="78"/>
       <c r="Q159" s="78"/>
@@ -28172,10 +28212,10 @@
     </row>
     <row r="160" spans="1:20" ht="15">
       <c r="A160" s="83" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="B160" s="83" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="C160" s="83" t="s">
         <v>95</v>
@@ -28224,10 +28264,10 @@
     </row>
     <row r="161" spans="1:20" ht="15">
       <c r="A161" s="78" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="B161" s="78" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="C161" s="78" t="s">
         <v>95</v>
@@ -28276,10 +28316,10 @@
     </row>
     <row r="162" spans="1:20" ht="15">
       <c r="A162" s="83" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="B162" s="83" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="C162" s="83" t="s">
         <v>95</v>
@@ -28326,10 +28366,10 @@
     </row>
     <row r="163" spans="1:20" ht="15">
       <c r="A163" s="78" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="B163" s="78" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="C163" s="78" t="s">
         <v>95</v>
@@ -28376,10 +28416,10 @@
     </row>
     <row r="164" spans="1:20" ht="60">
       <c r="A164" s="83" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="B164" s="83" t="s">
-        <v>816</v>
+        <v>814</v>
       </c>
       <c r="C164" s="83" t="s">
         <v>95</v>
@@ -28419,7 +28459,7 @@
       </c>
       <c r="O164" s="83"/>
       <c r="P164" s="83" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="Q164" s="83"/>
       <c r="R164" s="83"/>
@@ -28428,10 +28468,10 @@
     </row>
     <row r="165" spans="1:20" ht="15">
       <c r="A165" s="78" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="B165" s="78" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="C165" s="78" t="s">
         <v>95</v>
@@ -28473,7 +28513,7 @@
       </c>
       <c r="O165" s="78"/>
       <c r="P165" s="78" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="Q165" s="78"/>
       <c r="R165" s="78"/>
@@ -28482,10 +28522,10 @@
     </row>
     <row r="166" spans="1:20" ht="15">
       <c r="A166" s="83" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="B166" s="83" t="s">
-        <v>814</v>
+        <v>812</v>
       </c>
       <c r="C166" s="83" t="s">
         <v>95</v>
@@ -28525,7 +28565,7 @@
       </c>
       <c r="O166" s="83"/>
       <c r="P166" s="83" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="Q166" s="83"/>
       <c r="R166" s="83"/>
@@ -28534,10 +28574,10 @@
     </row>
     <row r="167" spans="1:20" ht="15">
       <c r="A167" s="78" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="B167" s="78" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="C167" s="78" t="s">
         <v>95</v>
@@ -28571,7 +28611,7 @@
         <v>2220</v>
       </c>
       <c r="L167" s="78" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="M167" s="78"/>
       <c r="N167" s="78" t="s">
@@ -28579,7 +28619,7 @@
       </c>
       <c r="O167" s="78"/>
       <c r="P167" s="78" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="Q167" s="78"/>
       <c r="R167" s="78"/>
@@ -28588,10 +28628,10 @@
     </row>
     <row r="168" spans="1:20" ht="15">
       <c r="A168" s="83" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="B168" s="83" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
       <c r="C168" s="83" t="s">
         <v>95</v>
@@ -28631,7 +28671,7 @@
       </c>
       <c r="O168" s="83"/>
       <c r="P168" s="83" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="Q168" s="83"/>
       <c r="R168" s="83"/>
@@ -28640,10 +28680,10 @@
     </row>
     <row r="169" spans="1:20" ht="15">
       <c r="A169" s="78" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="B169" s="78" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="C169" s="78" t="s">
         <v>95</v>
@@ -28683,7 +28723,7 @@
       </c>
       <c r="O169" s="78"/>
       <c r="P169" s="78" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="Q169" s="78"/>
       <c r="R169" s="78"/>
@@ -28692,10 +28732,10 @@
     </row>
     <row r="170" spans="1:20" ht="30">
       <c r="A170" s="83" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
       <c r="B170" s="83" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
       <c r="C170" s="83" t="s">
         <v>95</v>
@@ -28735,7 +28775,7 @@
       </c>
       <c r="O170" s="83"/>
       <c r="P170" s="83" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
       <c r="Q170" s="83"/>
       <c r="R170" s="83"/>
@@ -28744,10 +28784,10 @@
     </row>
     <row r="171" spans="1:20" ht="15">
       <c r="A171" s="78" t="s">
-        <v>794</v>
+        <v>792</v>
       </c>
       <c r="B171" s="83" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="C171" s="78" t="s">
         <v>95</v>
@@ -28794,10 +28834,10 @@
     </row>
     <row r="172" spans="1:20" ht="15">
       <c r="A172" s="83" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
       <c r="B172" s="83" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
       <c r="C172" s="83" t="s">
         <v>95</v>
@@ -28844,10 +28884,10 @@
     </row>
     <row r="173" spans="1:20" ht="15">
       <c r="A173" s="78" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
       <c r="B173" s="78" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="C173" s="78" t="s">
         <v>95</v>
@@ -28894,10 +28934,10 @@
     </row>
     <row r="174" spans="1:20" ht="15">
       <c r="A174" s="83" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="B174" s="83" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="C174" s="83" t="s">
         <v>95</v>
@@ -28944,10 +28984,10 @@
     </row>
     <row r="175" spans="1:20" ht="90">
       <c r="A175" s="78" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
       <c r="B175" s="78" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="C175" s="78" t="s">
         <v>95</v>
@@ -28987,7 +29027,7 @@
       </c>
       <c r="O175" s="78"/>
       <c r="P175" s="78" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="Q175" s="78"/>
       <c r="R175" s="78"/>
@@ -36561,7 +36601,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1">
       <c r="A1" s="94" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="B1" s="94"/>
     </row>
@@ -36570,7 +36610,7 @@
         <v>42</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="13.5" customHeight="1">
@@ -36602,25 +36642,25 @@
         <v>42</v>
       </c>
       <c r="B7" s="72" t="s">
+        <v>722</v>
+      </c>
+      <c r="C7" s="72" t="s">
+        <v>723</v>
+      </c>
+      <c r="D7" s="72" t="s">
         <v>724</v>
       </c>
-      <c r="C7" s="72" t="s">
+      <c r="E7" s="72" t="s">
         <v>725</v>
       </c>
-      <c r="D7" s="72" t="s">
+      <c r="F7" s="72" t="s">
         <v>726</v>
       </c>
-      <c r="E7" s="72" t="s">
+      <c r="G7" s="72" t="s">
         <v>727</v>
       </c>
-      <c r="F7" s="72" t="s">
+      <c r="H7" s="72" t="s">
         <v>728</v>
-      </c>
-      <c r="G7" s="72" t="s">
-        <v>729</v>
-      </c>
-      <c r="H7" s="72" t="s">
-        <v>730</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="13.5" customHeight="1">
@@ -36724,7 +36764,7 @@
     </row>
     <row r="12" spans="1:8" s="74" customFormat="1" ht="15.75" customHeight="1">
       <c r="A12" s="95" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="B12" s="95"/>
       <c r="C12" s="95"/>
@@ -36737,13 +36777,13 @@
         <v>98</v>
       </c>
       <c r="B13" s="72" t="s">
+        <v>730</v>
+      </c>
+      <c r="C13" s="72" t="s">
+        <v>731</v>
+      </c>
+      <c r="D13" s="72" t="s">
         <v>732</v>
-      </c>
-      <c r="C13" s="72" t="s">
-        <v>733</v>
-      </c>
-      <c r="D13" s="72" t="s">
-        <v>734</v>
       </c>
       <c r="E13" s="72" t="s">
         <v>99</v>
@@ -36757,7 +36797,7 @@
         <v>45952</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>51</v>
@@ -36775,7 +36815,7 @@
         <v>45952</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>51</v>
@@ -36829,7 +36869,7 @@
         <v>45970</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>50</v>
@@ -36847,7 +36887,7 @@
         <v>45970</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>50</v>
@@ -36865,7 +36905,7 @@
         <v>45973</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>50</v>
@@ -36883,7 +36923,7 @@
         <v>45973</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>49</v>
@@ -36901,7 +36941,7 @@
         <v>46058</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>51</v>
@@ -36937,7 +36977,7 @@
         <v>46059</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>49</v>
@@ -36973,7 +37013,7 @@
         <v>46093</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>50</v>
@@ -36991,7 +37031,7 @@
         <v>46093</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>51</v>
@@ -37074,7 +37114,7 @@
     </row>
     <row r="58" spans="2:2" ht="13.5" customHeight="1">
       <c r="B58" s="6" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
     </row>
   </sheetData>
@@ -37104,7 +37144,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="13.5" customHeight="1">
       <c r="A1" s="77" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="73" customFormat="1" ht="13.5" customHeight="1">
@@ -37112,22 +37152,22 @@
         <v>42</v>
       </c>
       <c r="B3" s="72" t="s">
+        <v>736</v>
+      </c>
+      <c r="C3" s="72" t="s">
+        <v>721</v>
+      </c>
+      <c r="D3" s="72" t="s">
+        <v>737</v>
+      </c>
+      <c r="E3" s="72" t="s">
         <v>738</v>
       </c>
-      <c r="C3" s="72" t="s">
-        <v>723</v>
-      </c>
-      <c r="D3" s="72" t="s">
+      <c r="F3" s="72" t="s">
         <v>739</v>
       </c>
-      <c r="E3" s="72" t="s">
+      <c r="G3" s="72" t="s">
         <v>740</v>
-      </c>
-      <c r="F3" s="72" t="s">
-        <v>741</v>
-      </c>
-      <c r="G3" s="72" t="s">
-        <v>742</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="13.5" customHeight="1">
@@ -37136,7 +37176,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>245912</v>
+        <v>247012</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -37144,11 +37184,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>88971.457399999999</v>
+        <v>89338.19739999999</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>156940.54259999999</v>
+        <v>157673.8026</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -37156,7 +37196,7 @@
       </c>
       <c r="G4" s="16">
         <f>E4+F4</f>
-        <v>19630.516599999974</v>
+        <v>20363.776599999983</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -37173,11 +37213,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>88918.085200000001</v>
+        <v>89284.605200000005</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-80499.085200000001</v>
+        <v>-80865.605200000005</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -37185,7 +37225,7 @@
       </c>
       <c r="G5" s="18">
         <f>E5+F5</f>
-        <v>-8912.0432000000001</v>
+        <v>-9278.5632000000041</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -37202,11 +37242,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>88971.457399999999</v>
+        <v>89338.19739999999</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-76441.457399999999</v>
+        <v>-76808.19739999999</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -37214,7 +37254,7 @@
       </c>
       <c r="G6" s="16">
         <f>E6+F6</f>
-        <v>-10718.473399999988</v>
+        <v>-11085.213399999979</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">
@@ -37224,27 +37264,27 @@
     </row>
     <row r="10" spans="1:7" ht="13.5" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="13.5" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="13.5" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="13.5" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="13.5" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Latest sales and cash payments
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Apr26.xlsx
+++ b/docs/Chiraath-Summary-Apr26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC3D5BA-AC45-3A43-9A96-E56563B379FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A4E6F16-B8FD-A94B-A723-A9CE67661138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2123" uniqueCount="851">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2125" uniqueCount="851">
   <si>
     <t>Notes:</t>
   </si>
@@ -2528,9 +2528,6 @@
     <t>Banarasi Green Old design</t>
   </si>
   <si>
-    <t>Green Aanchal - XXL, Cream 2 piece aanchal - M,  Chikankari - XL, Blue Ajrakh Salwar - XXL</t>
-  </si>
-  <si>
     <t>Leena - Chikku Green, Prema - Chikku Maroon, Shini - Green</t>
   </si>
   <si>
@@ -2615,10 +2612,13 @@
     <t>Salwar maroon single piece M (CHR-78)</t>
   </si>
   <si>
-    <t>Ponnu - Red</t>
-  </si>
-  <si>
-    <t>Royal Blue/Peacock Teal, Maroon/Bottle Green</t>
+    <t>Green Aanchal - XXL, Cream 2 piece aanchal - M,  Chikankari - XL, Blue Ajrakh Salwar - XXL, Blue Banarasi new design</t>
+  </si>
+  <si>
+    <t>Maroon/Bottle Green</t>
+  </si>
+  <si>
+    <t>Ponnu - Red, Indu - Blue</t>
   </si>
 </sst>
 </file>
@@ -4289,7 +4289,7 @@
                   <c:v>22172</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>39538</c:v>
+                  <c:v>39598</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4449,7 +4449,7 @@
                   <c:v>16248</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>40759</c:v>
+                  <c:v>42139</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4889,7 +4889,7 @@
                   <c:v>-5924</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1221</c:v>
+                  <c:v>2541</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -6522,7 +6522,7 @@
     <col min="4" max="4" width="30.1640625" style="6" customWidth="1"/>
     <col min="5" max="5" width="22.1640625" style="6" customWidth="1"/>
     <col min="6" max="6" width="31.1640625" style="6" customWidth="1"/>
-    <col min="7" max="7" width="14.6640625" style="6" customWidth="1"/>
+    <col min="7" max="7" width="16.5" style="6" customWidth="1"/>
     <col min="8" max="16384" width="8.83203125" style="6"/>
   </cols>
   <sheetData>
@@ -6537,7 +6537,7 @@
       </c>
       <c r="B3" s="8">
         <f>SUM(Purchases!C:C)</f>
-        <v>318829</v>
+        <v>318889</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>42</v>
@@ -6552,7 +6552,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>270221</v>
+        <v>276101</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -6569,7 +6569,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>287571</v>
+        <v>288951</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -6586,7 +6586,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-48608</v>
+        <v>-42788</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -6621,7 +6621,7 @@
       </c>
       <c r="B10" s="13">
         <f>PartnerShares!H8</f>
-        <v>2216.3266666666714</v>
+        <v>2256.3266666666714</v>
       </c>
       <c r="C10" s="9"/>
     </row>
@@ -6631,7 +6631,7 @@
       </c>
       <c r="B11" s="14">
         <f>PartnerShares!H9</f>
-        <v>11517.33666666667</v>
+        <v>11497.33666666667</v>
       </c>
       <c r="C11" s="11"/>
     </row>
@@ -6641,7 +6641,7 @@
       </c>
       <c r="B12" s="13">
         <f>PartnerShares!H10</f>
-        <v>-13733.66333333333</v>
+        <v>-13753.66333333333</v>
       </c>
       <c r="C12" s="9"/>
     </row>
@@ -6680,15 +6680,15 @@
       </c>
       <c r="B18" s="10">
         <f>PartnerShares!B8</f>
-        <v>126796</v>
+        <v>126856</v>
       </c>
       <c r="C18" s="10">
         <f>PartnerShares!C8</f>
-        <v>106276.33333333333</v>
+        <v>106296.33333333333</v>
       </c>
       <c r="D18" s="10">
         <f>PartnerShares!D8</f>
-        <v>20519.666666666672</v>
+        <v>20559.666666666672</v>
       </c>
       <c r="E18" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -6696,11 +6696,11 @@
       </c>
       <c r="F18" s="13">
         <f>D18-E18</f>
-        <v>2216.3266666666714</v>
+        <v>2256.3266666666714</v>
       </c>
       <c r="G18" s="16" t="str">
         <f>IF(ROUND(F18,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F18),"#,##0"),IF(ROUND(F18,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F18),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹2,216</v>
+        <v>Receive ₹2,256</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1">
@@ -6714,11 +6714,11 @@
       </c>
       <c r="C19" s="12">
         <f>PartnerShares!C9</f>
-        <v>106276.33333333333</v>
+        <v>106296.33333333333</v>
       </c>
       <c r="D19" s="12">
         <f>PartnerShares!D9</f>
-        <v>53156.666666666672</v>
+        <v>53136.666666666672</v>
       </c>
       <c r="E19" s="12">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -6726,11 +6726,11 @@
       </c>
       <c r="F19" s="14">
         <f>D19-E19</f>
-        <v>11517.33666666667</v>
+        <v>11497.33666666667</v>
       </c>
       <c r="G19" s="17" t="str">
         <f>IF(ROUND(F19,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F19),"#,##0"),IF(ROUND(F19,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F19),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹11,517</v>
+        <v>Receive ₹11,497</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1">
@@ -6744,11 +6744,11 @@
       </c>
       <c r="C20" s="10">
         <f>PartnerShares!C10</f>
-        <v>106276.33333333333</v>
+        <v>106296.33333333333</v>
       </c>
       <c r="D20" s="10">
         <f>PartnerShares!D10</f>
-        <v>-73676.333333333328</v>
+        <v>-73696.333333333328</v>
       </c>
       <c r="E20" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -6756,11 +6756,11 @@
       </c>
       <c r="F20" s="13">
         <f>D20-E20</f>
-        <v>-13733.66333333333</v>
+        <v>-13753.66333333333</v>
       </c>
       <c r="G20" s="17" t="str">
         <f>IF(ROUND(F20,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F20),"#,##0"),IF(ROUND(F20,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F20),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹13,734</v>
+        <v>Pay ₹13,754</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1">
@@ -6798,15 +6798,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>249272</v>
+        <v>255152</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>90091.681399999987</v>
+        <v>92052.073399999994</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>159180.3186</v>
+        <v>163099.92660000001</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -6814,11 +6814,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>21870.292599999986</v>
+        <v>25789.900599999994</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹21,870</v>
+        <v>Pay ₹25,790</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -6832,11 +6832,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>90037.637199999997</v>
+        <v>91996.853199999998</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-81618.637199999997</v>
+        <v>-83577.853199999998</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -6844,11 +6844,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-10031.595199999996</v>
+        <v>-11990.811199999996</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹10,032</v>
+        <v>Receive ₹11,991</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -6862,11 +6862,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>90091.681399999987</v>
+        <v>92052.073399999994</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-77561.681399999987</v>
+        <v>-79522.073399999994</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -6874,11 +6874,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-11838.697399999975</v>
+        <v>-13799.089399999983</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹11,839</v>
+        <v>Receive ₹13,799</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -6990,7 +6990,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46135</v>
+        <v>46136</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -6999,14 +6999,14 @@
       </c>
       <c r="B5" s="21">
         <f>Summary!B3</f>
-        <v>318829</v>
+        <v>318889</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>69</v>
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>270221</v>
+        <v>276101</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -7015,7 +7015,7 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-48608</v>
+        <v>-42788</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
@@ -7124,15 +7124,15 @@
       </c>
       <c r="B13" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A13)*(YEAR(Purchases!$A$2:$A$998)=$B$7)*Purchases!$C$2:$C$998),0)</f>
-        <v>39538</v>
+        <v>39598</v>
       </c>
       <c r="C13" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$996,"MMM")=$A13)*(YEAR(Sales!$A$2:$A$996)=$B$7)*Sales!$C$2:$C$996),0)</f>
-        <v>40759</v>
+        <v>42139</v>
       </c>
       <c r="D13" s="27">
         <f t="shared" si="0"/>
-        <v>1221</v>
+        <v>2541</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1">
@@ -8338,10 +8338,18 @@
       </c>
     </row>
     <row r="66" spans="1:4" ht="15" customHeight="1">
-      <c r="A66" s="35"/>
-      <c r="B66" s="36"/>
-      <c r="C66" s="37"/>
-      <c r="D66" s="36"/>
+      <c r="A66" s="35">
+        <v>46134</v>
+      </c>
+      <c r="B66" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C66" s="37">
+        <v>60</v>
+      </c>
+      <c r="D66" s="36" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="67" spans="1:4" ht="15" customHeight="1">
       <c r="A67" s="38"/>
@@ -10656,6 +10664,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:I260"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
@@ -10665,7 +10674,7 @@
     <col min="4" max="4" width="18.1640625" style="90" customWidth="1"/>
     <col min="5" max="5" width="8.1640625" style="90" customWidth="1"/>
     <col min="6" max="6" width="7.1640625" style="93" customWidth="1"/>
-    <col min="7" max="7" width="8.1640625" style="90" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.83203125" style="90" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="35.1640625" style="90" customWidth="1"/>
     <col min="9" max="9" width="10.6640625" style="90" customWidth="1"/>
     <col min="10" max="16384" width="8.83203125" style="90"/>
@@ -10700,7 +10709,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" hidden="1">
       <c r="A2" s="75">
         <v>45900</v>
       </c>
@@ -10723,7 +10732,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" hidden="1">
       <c r="A3" s="79">
         <v>45900</v>
       </c>
@@ -10746,7 +10755,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" hidden="1">
       <c r="A4" s="75">
         <v>45900</v>
       </c>
@@ -10769,7 +10778,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" hidden="1">
       <c r="A5" s="79">
         <v>45900</v>
       </c>
@@ -10792,7 +10801,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" hidden="1">
       <c r="A6" s="75">
         <v>45900</v>
       </c>
@@ -10815,7 +10824,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" hidden="1">
       <c r="A7" s="79">
         <v>45900</v>
       </c>
@@ -10838,7 +10847,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" hidden="1">
       <c r="A8" s="75">
         <v>45900</v>
       </c>
@@ -10861,7 +10870,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" hidden="1">
       <c r="A9" s="79">
         <v>45901</v>
       </c>
@@ -10884,7 +10893,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" hidden="1">
       <c r="A10" s="75">
         <v>45902</v>
       </c>
@@ -10907,7 +10916,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" hidden="1">
       <c r="A11" s="79">
         <v>45903</v>
       </c>
@@ -10930,7 +10939,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" hidden="1">
       <c r="A12" s="75">
         <v>45904</v>
       </c>
@@ -10953,7 +10962,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" hidden="1">
       <c r="A13" s="79">
         <v>45905</v>
       </c>
@@ -10976,7 +10985,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" hidden="1">
       <c r="A14" s="75">
         <v>45906</v>
       </c>
@@ -10999,7 +11008,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" hidden="1">
       <c r="A15" s="79">
         <v>45907</v>
       </c>
@@ -11022,7 +11031,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" hidden="1">
       <c r="A16" s="75">
         <v>45908</v>
       </c>
@@ -11045,7 +11054,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" hidden="1">
       <c r="A17" s="79">
         <v>45909</v>
       </c>
@@ -11068,7 +11077,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" hidden="1">
       <c r="A18" s="75">
         <v>45910</v>
       </c>
@@ -11091,7 +11100,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" hidden="1">
       <c r="A19" s="79">
         <v>45911</v>
       </c>
@@ -11114,7 +11123,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" hidden="1">
       <c r="A20" s="75">
         <v>45912</v>
       </c>
@@ -11137,7 +11146,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" hidden="1">
       <c r="A21" s="79">
         <v>45913</v>
       </c>
@@ -11160,7 +11169,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" hidden="1">
       <c r="A22" s="75">
         <v>45914</v>
       </c>
@@ -11183,7 +11192,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" hidden="1">
       <c r="A23" s="79">
         <v>45915</v>
       </c>
@@ -11206,7 +11215,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" hidden="1">
       <c r="A24" s="75">
         <v>45916</v>
       </c>
@@ -11229,7 +11238,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" hidden="1">
       <c r="A25" s="79">
         <v>45917</v>
       </c>
@@ -11252,7 +11261,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:9" hidden="1">
       <c r="A26" s="75">
         <v>45917</v>
       </c>
@@ -11275,7 +11284,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" hidden="1">
       <c r="A27" s="79">
         <v>45918</v>
       </c>
@@ -11298,7 +11307,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" hidden="1">
       <c r="A28" s="75">
         <v>45919</v>
       </c>
@@ -11321,7 +11330,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="29" spans="1:9">
+    <row r="29" spans="1:9" hidden="1">
       <c r="A29" s="79">
         <v>45920</v>
       </c>
@@ -11344,7 +11353,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="30" spans="1:9">
+    <row r="30" spans="1:9" hidden="1">
       <c r="A30" s="75">
         <v>45921</v>
       </c>
@@ -11367,7 +11376,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="31" spans="1:9">
+    <row r="31" spans="1:9" hidden="1">
       <c r="A31" s="79">
         <v>45922</v>
       </c>
@@ -11390,7 +11399,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="32" spans="1:9">
+    <row r="32" spans="1:9" hidden="1">
       <c r="A32" s="75">
         <v>45924</v>
       </c>
@@ -11413,7 +11422,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="33" spans="1:9">
+    <row r="33" spans="1:9" hidden="1">
       <c r="A33" s="79">
         <v>45924</v>
       </c>
@@ -11436,7 +11445,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="34" spans="1:9">
+    <row r="34" spans="1:9" hidden="1">
       <c r="A34" s="75">
         <v>45930</v>
       </c>
@@ -11459,7 +11468,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="35" spans="1:9">
+    <row r="35" spans="1:9" hidden="1">
       <c r="A35" s="79">
         <v>45933.931944444397</v>
       </c>
@@ -11482,7 +11491,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="36" spans="1:9">
+    <row r="36" spans="1:9" hidden="1">
       <c r="A36" s="75">
         <v>45934.931944386597</v>
       </c>
@@ -11505,7 +11514,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="37" spans="1:9">
+    <row r="37" spans="1:9" hidden="1">
       <c r="A37" s="79">
         <v>45935.931944386597</v>
       </c>
@@ -11528,7 +11537,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="38" spans="1:9">
+    <row r="38" spans="1:9" hidden="1">
       <c r="A38" s="75">
         <v>45939.931944444397</v>
       </c>
@@ -11551,7 +11560,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="39" spans="1:9">
+    <row r="39" spans="1:9" hidden="1">
       <c r="A39" s="79">
         <v>45939.931944444397</v>
       </c>
@@ -11574,7 +11583,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="40" spans="1:9">
+    <row r="40" spans="1:9" hidden="1">
       <c r="A40" s="75">
         <v>45945</v>
       </c>
@@ -11597,7 +11606,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="41" spans="1:9">
+    <row r="41" spans="1:9" hidden="1">
       <c r="A41" s="79">
         <v>45946</v>
       </c>
@@ -11620,7 +11629,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="42" spans="1:9">
+    <row r="42" spans="1:9" hidden="1">
       <c r="A42" s="75">
         <v>45946</v>
       </c>
@@ -11643,7 +11652,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="43" spans="1:9">
+    <row r="43" spans="1:9" hidden="1">
       <c r="A43" s="79">
         <v>45947</v>
       </c>
@@ -11666,7 +11675,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="44" spans="1:9">
+    <row r="44" spans="1:9" hidden="1">
       <c r="A44" s="75">
         <v>45948</v>
       </c>
@@ -11689,7 +11698,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="45" spans="1:9">
+    <row r="45" spans="1:9" hidden="1">
       <c r="A45" s="79">
         <v>45949</v>
       </c>
@@ -11712,7 +11721,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="46" spans="1:9">
+    <row r="46" spans="1:9" hidden="1">
       <c r="A46" s="75">
         <v>45950</v>
       </c>
@@ -11735,7 +11744,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="47" spans="1:9">
+    <row r="47" spans="1:9" hidden="1">
       <c r="A47" s="79">
         <v>45951</v>
       </c>
@@ -11758,7 +11767,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="48" spans="1:9">
+    <row r="48" spans="1:9" hidden="1">
       <c r="A48" s="75">
         <v>45964</v>
       </c>
@@ -11781,7 +11790,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="49" spans="1:9">
+    <row r="49" spans="1:9" hidden="1">
       <c r="A49" s="79">
         <v>45963</v>
       </c>
@@ -11804,7 +11813,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="50" spans="1:9">
+    <row r="50" spans="1:9" hidden="1">
       <c r="A50" s="75">
         <v>45982</v>
       </c>
@@ -11827,7 +11836,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="51" spans="1:9">
+    <row r="51" spans="1:9" hidden="1">
       <c r="A51" s="79">
         <v>45983</v>
       </c>
@@ -11850,7 +11859,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="52" spans="1:9">
+    <row r="52" spans="1:9" hidden="1">
       <c r="A52" s="75">
         <v>45984</v>
       </c>
@@ -11873,7 +11882,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="53" spans="1:9">
+    <row r="53" spans="1:9" hidden="1">
       <c r="A53" s="79">
         <v>45985</v>
       </c>
@@ -11896,7 +11905,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="14">
+    <row r="54" spans="1:9" ht="14" hidden="1">
       <c r="A54" s="75">
         <v>45986</v>
       </c>
@@ -11921,7 +11930,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="15.75" customHeight="1">
+    <row r="55" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A55" s="79">
         <v>45992</v>
       </c>
@@ -11946,7 +11955,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="56" spans="1:9" ht="14">
+    <row r="56" spans="1:9" ht="14" hidden="1">
       <c r="A56" s="75">
         <v>45992</v>
       </c>
@@ -11971,7 +11980,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="57" spans="1:9" ht="15.75" customHeight="1">
+    <row r="57" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A57" s="79">
         <v>45996</v>
       </c>
@@ -11996,7 +12005,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="27.75" customHeight="1">
+    <row r="58" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A58" s="75">
         <v>45996</v>
       </c>
@@ -12021,7 +12030,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="15.75" customHeight="1">
+    <row r="59" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A59" s="79">
         <v>45996</v>
       </c>
@@ -12046,7 +12055,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="60" spans="1:9" ht="14">
+    <row r="60" spans="1:9" ht="14" hidden="1">
       <c r="A60" s="75">
         <v>46007</v>
       </c>
@@ -12071,7 +12080,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="61" spans="1:9" ht="15.75" customHeight="1">
+    <row r="61" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A61" s="79">
         <v>46008</v>
       </c>
@@ -12098,7 +12107,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="14">
+    <row r="62" spans="1:9" ht="14" hidden="1">
       <c r="A62" s="75">
         <v>46008</v>
       </c>
@@ -12123,7 +12132,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="63" spans="1:9" ht="15.75" customHeight="1">
+    <row r="63" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A63" s="79">
         <v>46008</v>
       </c>
@@ -12148,7 +12157,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="15.75" customHeight="1">
+    <row r="64" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A64" s="79">
         <v>46008</v>
       </c>
@@ -12173,7 +12182,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="14">
+    <row r="65" spans="1:9" ht="14" hidden="1">
       <c r="A65" s="75">
         <v>46009</v>
       </c>
@@ -12198,7 +12207,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="15.75" customHeight="1">
+    <row r="66" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A66" s="79">
         <v>46010</v>
       </c>
@@ -12223,7 +12232,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="67" spans="1:9" ht="14">
+    <row r="67" spans="1:9" ht="14" hidden="1">
       <c r="A67" s="75">
         <v>46010</v>
       </c>
@@ -12250,7 +12259,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="68" spans="1:9" ht="31.5" customHeight="1">
+    <row r="68" spans="1:9" ht="31.5" hidden="1" customHeight="1">
       <c r="A68" s="79">
         <v>46011</v>
       </c>
@@ -12275,7 +12284,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="69" spans="1:9" ht="14">
+    <row r="69" spans="1:9" ht="14" hidden="1">
       <c r="A69" s="75">
         <v>46011</v>
       </c>
@@ -12300,7 +12309,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="28">
+    <row r="70" spans="1:9" ht="28" hidden="1">
       <c r="A70" s="75">
         <v>46011</v>
       </c>
@@ -12325,7 +12334,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="71" spans="1:9" ht="15.75" customHeight="1">
+    <row r="71" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A71" s="79">
         <v>46011</v>
       </c>
@@ -12350,7 +12359,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="72" spans="1:9" ht="27.75" customHeight="1">
+    <row r="72" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A72" s="75">
         <v>46011</v>
       </c>
@@ -12375,7 +12384,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="73" spans="1:9" ht="31.5" customHeight="1">
+    <row r="73" spans="1:9" ht="31.5" hidden="1" customHeight="1">
       <c r="A73" s="79">
         <v>46011</v>
       </c>
@@ -12400,7 +12409,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="14">
+    <row r="74" spans="1:9" ht="14" hidden="1">
       <c r="A74" s="75">
         <v>46013</v>
       </c>
@@ -12427,7 +12436,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="15.75" customHeight="1">
+    <row r="75" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A75" s="79">
         <v>46013</v>
       </c>
@@ -12452,7 +12461,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="76" spans="1:9" ht="15.75" customHeight="1">
+    <row r="76" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A76" s="79">
         <v>46017</v>
       </c>
@@ -12477,7 +12486,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="14">
+    <row r="77" spans="1:9" ht="14" hidden="1">
       <c r="A77" s="75">
         <v>46017</v>
       </c>
@@ -12502,7 +12511,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="15.75" customHeight="1">
+    <row r="78" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A78" s="79">
         <v>46017</v>
       </c>
@@ -12527,7 +12536,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="79" spans="1:9" ht="14">
+    <row r="79" spans="1:9" ht="14" hidden="1">
       <c r="A79" s="75">
         <v>46017</v>
       </c>
@@ -12552,7 +12561,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="80" spans="1:9" ht="15.75" customHeight="1">
+    <row r="80" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A80" s="79">
         <v>46020</v>
       </c>
@@ -12577,7 +12586,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="81" spans="1:9" ht="14">
+    <row r="81" spans="1:9" ht="14" hidden="1">
       <c r="A81" s="75">
         <v>46024</v>
       </c>
@@ -12602,7 +12611,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="82" spans="1:9" ht="15.75" customHeight="1">
+    <row r="82" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A82" s="79">
         <v>46024</v>
       </c>
@@ -12627,7 +12636,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="83" spans="1:9" ht="14">
+    <row r="83" spans="1:9" ht="14" hidden="1">
       <c r="A83" s="75">
         <v>46024</v>
       </c>
@@ -12652,7 +12661,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="84" spans="1:9" ht="15.75" customHeight="1">
+    <row r="84" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A84" s="79">
         <v>46024</v>
       </c>
@@ -12677,7 +12686,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="85" spans="1:9" ht="14">
+    <row r="85" spans="1:9" ht="14" hidden="1">
       <c r="A85" s="75">
         <v>46027</v>
       </c>
@@ -12702,7 +12711,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="86" spans="1:9" ht="14">
+    <row r="86" spans="1:9" ht="14" hidden="1">
       <c r="A86" s="75">
         <v>46028</v>
       </c>
@@ -12727,7 +12736,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="87" spans="1:9" ht="15.75" customHeight="1">
+    <row r="87" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A87" s="79">
         <v>46029</v>
       </c>
@@ -12752,7 +12761,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="88" spans="1:9" ht="14">
+    <row r="88" spans="1:9" ht="14" hidden="1">
       <c r="A88" s="75">
         <v>46032</v>
       </c>
@@ -12777,7 +12786,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="89" spans="1:9" ht="15.75" customHeight="1">
+    <row r="89" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A89" s="79">
         <v>46033</v>
       </c>
@@ -12802,7 +12811,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="90" spans="1:9" ht="14">
+    <row r="90" spans="1:9" ht="14" hidden="1">
       <c r="A90" s="75">
         <v>46033</v>
       </c>
@@ -12827,7 +12836,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="91" spans="1:9" ht="15.75" customHeight="1">
+    <row r="91" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A91" s="79">
         <v>46034</v>
       </c>
@@ -12852,7 +12861,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="92" spans="1:9" ht="28">
+    <row r="92" spans="1:9" ht="28" hidden="1">
       <c r="A92" s="75">
         <v>46034</v>
       </c>
@@ -12877,7 +12886,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="93" spans="1:9" ht="15.75" customHeight="1">
+    <row r="93" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A93" s="79">
         <v>46035</v>
       </c>
@@ -12902,7 +12911,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="94" spans="1:9" ht="14">
+    <row r="94" spans="1:9" ht="14" hidden="1">
       <c r="A94" s="75">
         <v>46036</v>
       </c>
@@ -12927,7 +12936,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="95" spans="1:9" ht="15.75" customHeight="1">
+    <row r="95" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A95" s="79">
         <v>46038</v>
       </c>
@@ -12952,7 +12961,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="96" spans="1:9" ht="14">
+    <row r="96" spans="1:9" ht="14" hidden="1">
       <c r="A96" s="75">
         <v>46038</v>
       </c>
@@ -12977,7 +12986,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="97" spans="1:9" ht="15.75" customHeight="1">
+    <row r="97" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A97" s="79">
         <v>46039</v>
       </c>
@@ -13002,7 +13011,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="98" spans="1:9" ht="14">
+    <row r="98" spans="1:9" ht="14" hidden="1">
       <c r="A98" s="75">
         <v>46040</v>
       </c>
@@ -13027,7 +13036,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="15.75" customHeight="1">
+    <row r="99" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A99" s="79">
         <v>46041</v>
       </c>
@@ -13052,7 +13061,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="14">
+    <row r="100" spans="1:9" ht="14" hidden="1">
       <c r="A100" s="75">
         <v>46042</v>
       </c>
@@ -13077,7 +13086,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="101" spans="1:9" ht="15.75" customHeight="1">
+    <row r="101" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A101" s="79">
         <v>46043</v>
       </c>
@@ -13102,7 +13111,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="102" spans="1:9" ht="14">
+    <row r="102" spans="1:9" ht="14" hidden="1">
       <c r="A102" s="75">
         <v>46046</v>
       </c>
@@ -13127,7 +13136,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="103" spans="1:9" ht="14">
+    <row r="103" spans="1:9" ht="14" hidden="1">
       <c r="A103" s="79">
         <v>46048</v>
       </c>
@@ -13152,7 +13161,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="14">
+    <row r="104" spans="1:9" ht="14" hidden="1">
       <c r="A104" s="75">
         <v>46048</v>
       </c>
@@ -13177,7 +13186,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="105" spans="1:9" ht="15.75" customHeight="1">
+    <row r="105" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A105" s="79">
         <v>46049</v>
       </c>
@@ -13202,7 +13211,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="106" spans="1:9" ht="14">
+    <row r="106" spans="1:9" ht="14" hidden="1">
       <c r="A106" s="75">
         <v>46049</v>
       </c>
@@ -13227,7 +13236,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="107" spans="1:9" ht="15.75" customHeight="1">
+    <row r="107" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A107" s="79">
         <v>46049</v>
       </c>
@@ -13252,7 +13261,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="108" spans="1:9" ht="14">
+    <row r="108" spans="1:9" ht="14" hidden="1">
       <c r="A108" s="75">
         <v>46050</v>
       </c>
@@ -13277,7 +13286,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="109" spans="1:9" ht="15.75" customHeight="1">
+    <row r="109" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A109" s="79">
         <v>46051</v>
       </c>
@@ -13302,7 +13311,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="110" spans="1:9" ht="14">
+    <row r="110" spans="1:9" ht="14" hidden="1">
       <c r="A110" s="75">
         <v>46051</v>
       </c>
@@ -13327,7 +13336,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="111" spans="1:9" ht="15.75" customHeight="1">
+    <row r="111" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A111" s="79">
         <v>46051</v>
       </c>
@@ -13352,7 +13361,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="112" spans="1:9" ht="27.75" customHeight="1">
+    <row r="112" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A112" s="75">
         <v>46054</v>
       </c>
@@ -13377,7 +13386,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="113" spans="1:9" ht="15.75" customHeight="1">
+    <row r="113" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A113" s="79">
         <v>46054</v>
       </c>
@@ -13402,7 +13411,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="114" spans="1:9" ht="14">
+    <row r="114" spans="1:9" ht="14" hidden="1">
       <c r="A114" s="75">
         <v>46055</v>
       </c>
@@ -13427,7 +13436,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="115" spans="1:9" ht="15.75" customHeight="1">
+    <row r="115" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A115" s="79">
         <v>46055</v>
       </c>
@@ -13452,7 +13461,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="116" spans="1:9" ht="14">
+    <row r="116" spans="1:9" ht="14" hidden="1">
       <c r="A116" s="75">
         <v>46060</v>
       </c>
@@ -13477,7 +13486,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="117" spans="1:9" ht="15.75" customHeight="1">
+    <row r="117" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A117" s="79">
         <v>46062</v>
       </c>
@@ -13502,7 +13511,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="118" spans="1:9" ht="14">
+    <row r="118" spans="1:9" ht="14" hidden="1">
       <c r="A118" s="75">
         <v>46065</v>
       </c>
@@ -13527,7 +13536,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="119" spans="1:9" ht="15.75" customHeight="1">
+    <row r="119" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A119" s="79">
         <v>46055</v>
       </c>
@@ -13552,7 +13561,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="120" spans="1:9" ht="27.75" customHeight="1">
+    <row r="120" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A120" s="75">
         <v>46070</v>
       </c>
@@ -13577,7 +13586,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="121" spans="1:9" ht="15.75" customHeight="1">
+    <row r="121" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A121" s="79">
         <v>46073</v>
       </c>
@@ -13602,7 +13611,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="122" spans="1:9" ht="14">
+    <row r="122" spans="1:9" ht="14" hidden="1">
       <c r="A122" s="75">
         <v>46074</v>
       </c>
@@ -13627,7 +13636,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="15.75" customHeight="1">
+    <row r="123" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A123" s="79">
         <v>46075</v>
       </c>
@@ -13652,7 +13661,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="124" spans="1:9" ht="14">
+    <row r="124" spans="1:9" ht="14" hidden="1">
       <c r="A124" s="75">
         <v>46075</v>
       </c>
@@ -13677,7 +13686,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="125" spans="1:9" ht="31.5" customHeight="1">
+    <row r="125" spans="1:9" ht="31.5" hidden="1" customHeight="1">
       <c r="A125" s="79">
         <v>46079</v>
       </c>
@@ -13702,7 +13711,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="126" spans="1:9" ht="14">
+    <row r="126" spans="1:9" ht="14" hidden="1">
       <c r="A126" s="75">
         <v>46079</v>
       </c>
@@ -13727,7 +13736,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="127" spans="1:9" ht="14">
+    <row r="127" spans="1:9" ht="14" hidden="1">
       <c r="A127" s="79">
         <v>46090</v>
       </c>
@@ -13752,7 +13761,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="14">
+    <row r="128" spans="1:9" ht="14" hidden="1">
       <c r="A128" s="75">
         <v>46090</v>
       </c>
@@ -13777,7 +13786,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="129" spans="1:9" ht="14">
+    <row r="129" spans="1:9" ht="14" hidden="1">
       <c r="A129" s="75">
         <v>46090</v>
       </c>
@@ -13802,7 +13811,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="130" spans="1:9" ht="15.75" customHeight="1">
+    <row r="130" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A130" s="79">
         <v>46091</v>
       </c>
@@ -13827,7 +13836,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="131" spans="1:9" ht="14">
+    <row r="131" spans="1:9" ht="14" hidden="1">
       <c r="A131" s="75">
         <v>46092</v>
       </c>
@@ -13852,7 +13861,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="15.75" customHeight="1">
+    <row r="132" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A132" s="79">
         <v>46092</v>
       </c>
@@ -13877,7 +13886,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="133" spans="1:9" ht="27.75" customHeight="1">
+    <row r="133" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A133" s="75">
         <v>46093</v>
       </c>
@@ -13902,7 +13911,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="134" spans="1:9" ht="15.75" customHeight="1">
+    <row r="134" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A134" s="79">
         <v>46093</v>
       </c>
@@ -13927,7 +13936,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="135" spans="1:9" ht="14">
+    <row r="135" spans="1:9" ht="14" hidden="1">
       <c r="A135" s="75">
         <v>46097</v>
       </c>
@@ -13952,7 +13961,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="136" spans="1:9" ht="15.75" customHeight="1">
+    <row r="136" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A136" s="79">
         <v>46097</v>
       </c>
@@ -13977,7 +13986,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="137" spans="1:9" ht="14">
+    <row r="137" spans="1:9" ht="14" hidden="1">
       <c r="A137" s="75">
         <v>46100</v>
       </c>
@@ -14002,7 +14011,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="138" spans="1:9" ht="15.75" customHeight="1">
+    <row r="138" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A138" s="79">
         <v>46104</v>
       </c>
@@ -14027,7 +14036,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="139" spans="1:9" ht="27.75" customHeight="1">
+    <row r="139" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A139" s="75">
         <v>46105</v>
       </c>
@@ -14052,7 +14061,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="140" spans="1:9" ht="31.5" customHeight="1">
+    <row r="140" spans="1:9" ht="31.5" hidden="1" customHeight="1">
       <c r="A140" s="79">
         <v>46113</v>
       </c>
@@ -14077,7 +14086,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="141" spans="1:9" ht="14">
+    <row r="141" spans="1:9" ht="14" hidden="1">
       <c r="A141" s="75">
         <v>46118</v>
       </c>
@@ -14102,7 +14111,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="142" spans="1:9" ht="15.75" customHeight="1">
+    <row r="142" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A142" s="79">
         <v>46119</v>
       </c>
@@ -14127,7 +14136,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="143" spans="1:9" ht="14">
+    <row r="143" spans="1:9" ht="14" hidden="1">
       <c r="A143" s="75">
         <v>46120</v>
       </c>
@@ -14152,7 +14161,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="144" spans="1:9" ht="15.75" customHeight="1">
+    <row r="144" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A144" s="79">
         <v>46120</v>
       </c>
@@ -14177,7 +14186,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="145" spans="1:9" ht="14">
+    <row r="145" spans="1:9" ht="14" hidden="1">
       <c r="A145" s="75">
         <v>46120</v>
       </c>
@@ -14219,13 +14228,13 @@
       <c r="F146" s="91"/>
       <c r="G146" s="91"/>
       <c r="H146" s="92" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="I146" s="80" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="147" spans="1:9" ht="14">
+    <row r="147" spans="1:9" ht="14" hidden="1">
       <c r="A147" s="75">
         <v>46122</v>
       </c>
@@ -14250,7 +14259,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="148" spans="1:9" ht="15.75" customHeight="1">
+    <row r="148" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A148" s="79">
         <v>46122</v>
       </c>
@@ -14298,7 +14307,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="150" spans="1:9" ht="15.75" customHeight="1">
+    <row r="150" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A150" s="79">
         <v>46125</v>
       </c>
@@ -14323,7 +14332,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="151" spans="1:9" ht="14">
+    <row r="151" spans="1:9" ht="14" hidden="1">
       <c r="A151" s="75">
         <v>46125</v>
       </c>
@@ -14348,7 +14357,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="152" spans="1:9" ht="15.75" customHeight="1">
+    <row r="152" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A152" s="79">
         <v>46125</v>
       </c>
@@ -14373,7 +14382,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="153" spans="1:9" ht="14">
+    <row r="153" spans="1:9" ht="14" hidden="1">
       <c r="A153" s="75">
         <v>46125</v>
       </c>
@@ -14398,7 +14407,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="154" spans="1:9" ht="15.75" customHeight="1">
+    <row r="154" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A154" s="79">
         <v>46126</v>
       </c>
@@ -14423,7 +14432,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="155" spans="1:9" ht="14">
+    <row r="155" spans="1:9" ht="14" hidden="1">
       <c r="A155" s="75">
         <v>46127</v>
       </c>
@@ -14448,7 +14457,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="156" spans="1:9" ht="15.75" customHeight="1">
+    <row r="156" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A156" s="79">
         <v>46129</v>
       </c>
@@ -14473,7 +14482,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="157" spans="1:9" ht="14">
+    <row r="157" spans="1:9" ht="14" hidden="1">
       <c r="A157" s="75">
         <v>46129</v>
       </c>
@@ -14521,7 +14530,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="159" spans="1:9" ht="14">
+    <row r="159" spans="1:9" ht="14" hidden="1">
       <c r="A159" s="75">
         <v>46130</v>
       </c>
@@ -14569,12 +14578,12 @@
         <v>334</v>
       </c>
     </row>
-    <row r="161" spans="1:9" ht="14">
+    <row r="161" spans="1:9" ht="14" hidden="1">
       <c r="A161" s="75">
         <v>46132</v>
       </c>
       <c r="B161" s="76" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="C161" s="77">
         <v>1100</v>
@@ -14594,7 +14603,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="162" spans="1:9" ht="28">
+    <row r="162" spans="1:9" ht="42" hidden="1">
       <c r="A162" s="79">
         <v>46132</v>
       </c>
@@ -14602,7 +14611,7 @@
         <v>153</v>
       </c>
       <c r="C162" s="81">
-        <v>4500</v>
+        <v>5880</v>
       </c>
       <c r="D162" s="80"/>
       <c r="E162" s="80" t="s">
@@ -14611,10 +14620,10 @@
       <c r="F162" s="91"/>
       <c r="G162" s="91"/>
       <c r="H162" s="92" t="s">
-        <v>820</v>
+        <v>848</v>
       </c>
       <c r="I162" s="80" t="s">
-        <v>334</v>
+        <v>140</v>
       </c>
     </row>
     <row r="163" spans="1:9" ht="14">
@@ -14622,7 +14631,7 @@
         <v>46133</v>
       </c>
       <c r="B163" s="76" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C163" s="77">
         <v>1380</v>
@@ -14634,7 +14643,7 @@
       <c r="F163" s="76"/>
       <c r="G163" s="76"/>
       <c r="H163" s="78" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="I163" s="76" t="s">
         <v>334</v>
@@ -14657,7 +14666,7 @@
       <c r="F164" s="91"/>
       <c r="G164" s="91"/>
       <c r="H164" s="92" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="I164" s="80" t="s">
         <v>334</v>
@@ -14680,18 +14689,18 @@
       <c r="F165" s="76"/>
       <c r="G165" s="76"/>
       <c r="H165" s="78" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="I165" s="76" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="166" spans="1:9" ht="14">
+    <row r="166" spans="1:9" ht="14" hidden="1">
       <c r="A166" s="79">
         <v>46134</v>
       </c>
       <c r="B166" s="80" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="C166" s="81">
         <v>1280</v>
@@ -14705,7 +14714,7 @@
       <c r="F166" s="91"/>
       <c r="G166" s="91"/>
       <c r="H166" s="92" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="I166" s="80" t="s">
         <v>140</v>
@@ -14728,7 +14737,7 @@
       <c r="F167" s="76"/>
       <c r="G167" s="76"/>
       <c r="H167" s="78" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="I167" s="76" t="s">
         <v>334</v>
@@ -14751,7 +14760,7 @@
       <c r="F168" s="76"/>
       <c r="G168" s="76"/>
       <c r="H168" s="78" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="I168" s="76" t="s">
         <v>334</v>
@@ -14774,7 +14783,7 @@
       <c r="F169" s="91"/>
       <c r="G169" s="91"/>
       <c r="H169" s="92" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="I169" s="80" t="s">
         <v>334</v>
@@ -14785,7 +14794,7 @@
         <v>46134</v>
       </c>
       <c r="B170" s="76" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="C170" s="77">
         <v>650</v>
@@ -14797,7 +14806,7 @@
       <c r="F170" s="76"/>
       <c r="G170" s="76"/>
       <c r="H170" s="78" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="I170" s="76" t="s">
         <v>334</v>
@@ -15791,7 +15800,13 @@
       <c r="I260" s="84"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I170" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:I170" xr:uid="{00000000-0009-0000-0000-000004000000}">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="Pending"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1260" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"Ordered,Pending,Completed,Cancelled"</formula1>
@@ -22738,7 +22753,7 @@
         <v>0</v>
       </c>
       <c r="L65" s="42" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="M65" s="42"/>
       <c r="N65" s="42" t="s">
@@ -23480,7 +23495,7 @@
         <v>0</v>
       </c>
       <c r="L79" s="42" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="M79" s="42"/>
       <c r="N79" s="42" t="s">
@@ -23800,7 +23815,7 @@
         <v>895</v>
       </c>
       <c r="L85" s="42" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="M85" s="42"/>
       <c r="N85" s="42" t="s">
@@ -24220,14 +24235,14 @@
         <v>944</v>
       </c>
       <c r="L93" s="42" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="M93" s="42"/>
       <c r="N93" s="48" t="s">
         <v>451</v>
       </c>
       <c r="O93" s="42" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="P93" s="42"/>
       <c r="Q93" s="42"/>
@@ -25654,7 +25669,7 @@
         <v>2932.6733333333309</v>
       </c>
       <c r="L120" s="48" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="M120" s="48" t="s">
         <v>49</v>
@@ -25664,7 +25679,7 @@
       </c>
       <c r="O120" s="48"/>
       <c r="P120" s="48" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="Q120" s="48"/>
       <c r="R120" s="48"/>
@@ -27172,7 +27187,7 @@
         <v>0</v>
       </c>
       <c r="L136" s="48" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="M136" s="48"/>
       <c r="N136" s="48" t="s">
@@ -27278,7 +27293,7 @@
         <v>0</v>
       </c>
       <c r="L138" s="48" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="M138" s="48"/>
       <c r="N138" s="48" t="s">
@@ -27950,7 +27965,7 @@
         <v>645</v>
       </c>
       <c r="L151" s="42" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="M151" s="42"/>
       <c r="N151" s="42" t="s">
@@ -28326,14 +28341,14 @@
         <v>3356</v>
       </c>
       <c r="L158" s="48" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="M158" s="48"/>
       <c r="N158" s="48" t="s">
         <v>538</v>
       </c>
       <c r="O158" s="48" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="P158" s="48"/>
       <c r="Q158" s="48"/>
@@ -28380,14 +28395,14 @@
         <v>3356</v>
       </c>
       <c r="L159" s="42" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="M159" s="42"/>
       <c r="N159" s="42" t="s">
         <v>538</v>
       </c>
       <c r="O159" s="42" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="P159" s="42"/>
       <c r="Q159" s="42"/>
@@ -28954,7 +28969,7 @@
         <v>0</v>
       </c>
       <c r="L170" s="48" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="M170" s="48"/>
       <c r="N170" s="48" t="s">
@@ -29008,7 +29023,7 @@
         <v>1784</v>
       </c>
       <c r="L171" s="42" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="M171" s="42"/>
       <c r="N171" s="42" t="s">
@@ -29016,7 +29031,7 @@
       </c>
       <c r="O171" s="42"/>
       <c r="P171" s="42" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="Q171" s="42"/>
       <c r="R171" s="42"/>
@@ -33631,15 +33646,15 @@
       </c>
       <c r="B8" s="9">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A8,Purchases!$C:$C),0)</f>
-        <v>126796</v>
+        <v>126856</v>
       </c>
       <c r="C8" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>106276.33333333333</v>
+        <v>106296.33333333333</v>
       </c>
       <c r="D8" s="9">
         <f>B8-C8</f>
-        <v>20519.666666666672</v>
+        <v>20559.666666666672</v>
       </c>
       <c r="E8" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE()),0)</f>
@@ -33647,7 +33662,7 @@
       </c>
       <c r="F8" s="9">
         <f>D8+E8</f>
-        <v>20519.666666666672</v>
+        <v>20559.666666666672</v>
       </c>
       <c r="G8" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -33655,7 +33670,7 @@
       </c>
       <c r="H8" s="69">
         <f>F8-G8</f>
-        <v>2216.3266666666714</v>
+        <v>2256.3266666666714</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="13.5" customHeight="1">
@@ -33668,11 +33683,11 @@
       </c>
       <c r="C9" s="11">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>106276.33333333333</v>
+        <v>106296.33333333333</v>
       </c>
       <c r="D9" s="11">
         <f>B9-C9</f>
-        <v>53156.666666666672</v>
+        <v>53136.666666666672</v>
       </c>
       <c r="E9" s="11">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE()),0)</f>
@@ -33680,7 +33695,7 @@
       </c>
       <c r="F9" s="11">
         <f>D9+E9</f>
-        <v>53156.666666666672</v>
+        <v>53136.666666666672</v>
       </c>
       <c r="G9" s="11">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -33688,7 +33703,7 @@
       </c>
       <c r="H9" s="70">
         <f>F9-G9</f>
-        <v>11517.33666666667</v>
+        <v>11497.33666666667</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="13.5" customHeight="1">
@@ -33701,11 +33716,11 @@
       </c>
       <c r="C10" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>106276.33333333333</v>
+        <v>106296.33333333333</v>
       </c>
       <c r="D10" s="9">
         <f>B10-C10</f>
-        <v>-73676.333333333328</v>
+        <v>-73696.333333333328</v>
       </c>
       <c r="E10" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE()),0)</f>
@@ -33713,7 +33728,7 @@
       </c>
       <c r="F10" s="9">
         <f>D10+E10</f>
-        <v>-73676.333333333328</v>
+        <v>-73696.333333333328</v>
       </c>
       <c r="G10" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -33721,7 +33736,7 @@
       </c>
       <c r="H10" s="69">
         <f>F10-G10</f>
-        <v>-13733.66333333333</v>
+        <v>-13753.66333333333</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="71" customFormat="1" ht="15.75" customHeight="1">
@@ -34138,7 +34153,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>249272</v>
+        <v>255152</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -34146,11 +34161,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>90091.681399999987</v>
+        <v>92052.073399999994</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>159180.3186</v>
+        <v>163099.92660000001</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -34158,7 +34173,7 @@
       </c>
       <c r="G4" s="69">
         <f>E4+F4</f>
-        <v>21870.292599999986</v>
+        <v>25789.900599999994</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -34175,11 +34190,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>90037.637199999997</v>
+        <v>91996.853199999998</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-81618.637199999997</v>
+        <v>-83577.853199999998</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -34187,7 +34202,7 @@
       </c>
       <c r="G5" s="70">
         <f>E5+F5</f>
-        <v>-10031.595199999996</v>
+        <v>-11990.811199999996</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -34204,11 +34219,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>90091.681399999987</v>
+        <v>92052.073399999994</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-77561.681399999987</v>
+        <v>-79522.073399999994</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -34216,7 +34231,7 @@
       </c>
       <c r="G6" s="69">
         <f>E6+F6</f>
-        <v>-11838.697399999975</v>
+        <v>-13799.089399999983</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">

</xml_diff>

<commit_message>
Latest sales and purchases
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Apr26.xlsx
+++ b/docs/Chiraath-Summary-Apr26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{608839D9-4756-D54E-A812-A35FFB9A919B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E463C01-4F24-9042-BDD6-E0C3AAA8A2AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Purchases!$A$1:$D$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Sales!$A$1:$I$173</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Sales!$A$1:$I$180</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2164" uniqueCount="864">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2219" uniqueCount="894">
   <si>
     <t>Notes:</t>
   </si>
@@ -1782,9 +1782,6 @@
   </si>
   <si>
     <t>saree</t>
-  </si>
-  <si>
-    <t>Latha (500)</t>
   </si>
   <si>
     <t>CHR-91</t>
@@ -2203,14 +2200,6 @@
     <t>Matka Silk Saree collections - old design</t>
   </si>
   <si>
-    <t>Blue/bottle green - Saranya Hyd, Blue/red - Jothika, Mustard - Vineetha, Bottle Green/Golden Yellow - Swapna (Thrissur)-1200</t>
-  </si>
-  <si>
-    <t>Bottle Green/Golden Yellow - 2 
-Black/Golden Yellow - 2
-Navy Blue/Bottle Green - 2</t>
-  </si>
-  <si>
     <t>CHR-147</t>
   </si>
   <si>
@@ -2385,9 +2374,6 @@
     <t xml:space="preserve">Khadi Cotton Saree (Jar Border)  </t>
   </si>
   <si>
-    <t xml:space="preserve">Yellow, Dark Green, Violet  </t>
-  </si>
-  <si>
     <t>CHR-168</t>
   </si>
   <si>
@@ -2598,18 +2584,12 @@
     <t>Salwar maroon single piece M (CHR-78)</t>
   </si>
   <si>
-    <t>Blue</t>
-  </si>
-  <si>
     <t>Green Aanchal - XXL, Cream 2 piece aanchal - M,  Chikankari - XL, Blue Ajrakh Salwar - XXL, Maroon Banarasi new design</t>
   </si>
   <si>
     <t>CHR-119 - Chanderi Silk Blue</t>
   </si>
   <si>
-    <t>Ponnu - Red (1350), Indu - Maroon</t>
-  </si>
-  <si>
     <t>CHR-119 - Chanderi Silk Maroon</t>
   </si>
   <si>
@@ -2619,12 +2599,6 @@
     <t>Sherin Fathima (Thalassery)</t>
   </si>
   <si>
-    <t>matka</t>
-  </si>
-  <si>
-    <t>Maroon(1), Dark Green(1), Off white (1)</t>
-  </si>
-  <si>
     <t>Athira (Kollam)</t>
   </si>
   <si>
@@ -2640,23 +2614,142 @@
     <t>CHR-119 - Black?</t>
   </si>
   <si>
-    <t>Sherin - Maroon/navy blue</t>
+    <t>matka - Maroon/Navy Blue</t>
+  </si>
+  <si>
+    <t>Anju Shinoob</t>
+  </si>
+  <si>
+    <t>New Banarasi - Blue</t>
+  </si>
+  <si>
+    <t>Khadi Saree Violet and Rainbow saree</t>
+  </si>
+  <si>
+    <t>Ponnu - Red (1350), Indu - Maroon, Anju Shinoob - Blue</t>
+  </si>
+  <si>
+    <t>Latha (500), Baby Khadeeja</t>
+  </si>
+  <si>
+    <t>Baby Khadeeja - Violet</t>
+  </si>
+  <si>
+    <t>Yellow, Dark Green</t>
   </si>
   <si>
     <t>Peacok Blue/Maroon - 3
 Purple/Green - 1
-Navy Blue/Maroon - 3
+Navy Blue/Maroon - 2
 Lavender/Violet - 1
 Grey/Blue - 1</t>
   </si>
   <si>
-    <t>Aruna - violet, Resmi - navy blue, Malini - Rani Pink, Dona - Black, Dona - Blue, Jayalakshmi - Pink, Jyothimol - Blue, Amrutha - Maroon, Athira - Black, Jini - Maroon, off while - booked, Dark green - booked</t>
-  </si>
-  <si>
-    <t>CHR-119 - off white (booked)</t>
-  </si>
-  <si>
-    <t>CHR-199 - Dark green (booked)</t>
+    <t>Sherin - Maroon/navy blue(1099)</t>
+  </si>
+  <si>
+    <t>Blue/bottle green - Saranya Hyd, Blue/red - Jothika, Mustard - Vineetha, Bottle Green/Golden Yellow - Swapna (Thrissur)-1200, Black/Golden yellow - Kavya(Kasargod) - 1200</t>
+  </si>
+  <si>
+    <t>Bottle Green/Golden Yellow - 2 
+Black/Golden Yellow - 1
+Navy Blue/Bottle Green - 2</t>
+  </si>
+  <si>
+    <t>Kavya (Kasargod)</t>
+  </si>
+  <si>
+    <t>Matka Black with Golden Yellow</t>
+  </si>
+  <si>
+    <t>Old batch: Maroon(1), Dark Green(1), Off white (1) 
+New batch: Blue (2), mustard yellow (2), navy blue (3), Green (2), Rani pink (2), Maroon (3), offwhite (3), Orange (2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First Set: Aruna - violet, Resmi - navy blue, Malini - Rani Pink
+Second Set: Dona - Black, Dona - Blue, Jayalakshmi - Pink, Jyothimol - Blue, Amrutha - Maroon, Athira - Black, Jini - Maroon
+Third Set: </t>
+  </si>
+  <si>
+    <t>Matka Green/Yellow &amp; Bengal Cotton (Adv:100)</t>
+  </si>
+  <si>
+    <t>Silpa Kannur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saree Fanna (Tusser Silk) </t>
+  </si>
+  <si>
+    <t>violet, black, navy blue, maroon</t>
+  </si>
+  <si>
+    <t>CHR-175</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sarees TSR R/P GALA (Tusser Silk) </t>
+  </si>
+  <si>
+    <t>burned orange, Grey, wine, violet/grape, onion peal</t>
+  </si>
+  <si>
+    <t>CHR-176</t>
+  </si>
+  <si>
+    <t>CHR-177</t>
+  </si>
+  <si>
+    <t>CHR-178</t>
+  </si>
+  <si>
+    <t>CHR-179</t>
+  </si>
+  <si>
+    <t>CHR-180</t>
+  </si>
+  <si>
+    <t>CHR-181</t>
+  </si>
+  <si>
+    <t>CHR-182</t>
+  </si>
+  <si>
+    <t>CHR-183</t>
+  </si>
+  <si>
+    <t>CHR-184</t>
+  </si>
+  <si>
+    <t>CHR-185</t>
+  </si>
+  <si>
+    <t>CHR-186</t>
+  </si>
+  <si>
+    <t>CHR-187</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sarees TSR C/P BUTI (Silk) </t>
+  </si>
+  <si>
+    <t>Light brown, Pista green</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sarees katan li sapa (Chanderi) </t>
+  </si>
+  <si>
+    <t>black/pink, orange/black, black/parrot green</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sarees matka siky (Matka Silk) </t>
+  </si>
+  <si>
+    <t>Sky blue/pink, red/parrot green, deep red/bottle green</t>
+  </si>
+  <si>
+    <t>Sarees d mix (Organsa Sarees)</t>
+  </si>
+  <si>
+    <t>aby pink, baby orange, baby yellow, baby blue, light grey</t>
   </si>
 </sst>
 </file>
@@ -2668,7 +2761,7 @@
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="166" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2884,6 +2977,12 @@
       <sz val="10"/>
       <name val="Trebuchet MS"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="9">
@@ -3567,7 +3666,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>150</c:v>
+                  <c:v>155</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>81</c:v>
@@ -3670,7 +3769,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>69</c:v>
+                  <c:v>105</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>64</c:v>
@@ -4003,7 +4102,7 @@
                   <c:v>66578</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>50878.32</c:v>
+                  <c:v>75871.18333333332</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1829</c:v>
@@ -4327,7 +4426,7 @@
                   <c:v>22172</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>39660</c:v>
+                  <c:v>64842</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4487,7 +4586,7 @@
                   <c:v>16248</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>47998</c:v>
+                  <c:v>52577</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4927,7 +5026,7 @@
                   <c:v>-5924</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8338</c:v>
+                  <c:v>-12265</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -5400,10 +5499,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>233</c:v>
+                  <c:v>238</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>138</c:v>
+                  <c:v>174</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6575,7 +6674,7 @@
       </c>
       <c r="B3" s="8">
         <f>SUM(Purchases!C:C)</f>
-        <v>318951</v>
+        <v>344133</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>42</v>
@@ -6590,7 +6689,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>281960</v>
+        <v>286020</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -6607,7 +6706,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>294810</v>
+        <v>299389</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -6624,7 +6723,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-36991</v>
+        <v>-58113</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -6659,7 +6758,7 @@
       </c>
       <c r="B10" s="13">
         <f>PartnerShares!H8</f>
-        <v>2297.66</v>
+        <v>19085.66</v>
       </c>
       <c r="C10" s="9"/>
     </row>
@@ -6669,7 +6768,7 @@
       </c>
       <c r="B11" s="14">
         <f>PartnerShares!H9</f>
-        <v>11476.669999999998</v>
+        <v>3082.6699999999983</v>
       </c>
       <c r="C11" s="11"/>
     </row>
@@ -6679,7 +6778,7 @@
       </c>
       <c r="B12" s="13">
         <f>PartnerShares!H10</f>
-        <v>-13774.330000000002</v>
+        <v>-22168.33</v>
       </c>
       <c r="C12" s="9"/>
     </row>
@@ -6718,15 +6817,15 @@
       </c>
       <c r="B18" s="10">
         <f>PartnerShares!B8</f>
-        <v>126918</v>
+        <v>152100</v>
       </c>
       <c r="C18" s="10">
         <f>PartnerShares!C8</f>
-        <v>106317</v>
+        <v>114711</v>
       </c>
       <c r="D18" s="10">
         <f>PartnerShares!D8</f>
-        <v>20601</v>
+        <v>37389</v>
       </c>
       <c r="E18" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -6734,11 +6833,11 @@
       </c>
       <c r="F18" s="13">
         <f>D18-E18</f>
-        <v>2297.66</v>
+        <v>19085.66</v>
       </c>
       <c r="G18" s="16" t="str">
         <f>IF(ROUND(F18,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F18),"#,##0"),IF(ROUND(F18,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F18),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹2,298</v>
+        <v>Receive ₹19,086</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1">
@@ -6752,11 +6851,11 @@
       </c>
       <c r="C19" s="12">
         <f>PartnerShares!C9</f>
-        <v>106317</v>
+        <v>114711</v>
       </c>
       <c r="D19" s="12">
         <f>PartnerShares!D9</f>
-        <v>53116</v>
+        <v>44722</v>
       </c>
       <c r="E19" s="12">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -6764,11 +6863,11 @@
       </c>
       <c r="F19" s="14">
         <f>D19-E19</f>
-        <v>11476.669999999998</v>
+        <v>3082.6699999999983</v>
       </c>
       <c r="G19" s="17" t="str">
         <f>IF(ROUND(F19,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F19),"#,##0"),IF(ROUND(F19,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F19),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹11,477</v>
+        <v>Receive ₹3,083</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1">
@@ -6782,11 +6881,11 @@
       </c>
       <c r="C20" s="10">
         <f>PartnerShares!C10</f>
-        <v>106317</v>
+        <v>114711</v>
       </c>
       <c r="D20" s="10">
         <f>PartnerShares!D10</f>
-        <v>-73717</v>
+        <v>-82111</v>
       </c>
       <c r="E20" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -6794,11 +6893,11 @@
       </c>
       <c r="F20" s="13">
         <f>D20-E20</f>
-        <v>-13774.330000000002</v>
+        <v>-22168.33</v>
       </c>
       <c r="G20" s="17" t="str">
         <f>IF(ROUND(F20,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F20),"#,##0"),IF(ROUND(F20,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F20),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹13,774</v>
+        <v>Pay ₹22,168</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1">
@@ -6836,15 +6935,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>261011</v>
+        <v>265071</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>94005.463999999993</v>
+        <v>95359.067999999999</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>167005.53600000002</v>
+        <v>169711.932</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -6852,11 +6951,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>29695.510000000009</v>
+        <v>32401.905999999988</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹29,696</v>
+        <v>Pay ₹32,402</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -6870,11 +6969,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>93949.072</v>
+        <v>95301.864000000001</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-85530.072</v>
+        <v>-86882.864000000001</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -6882,11 +6981,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-13943.029999999999</v>
+        <v>-15295.822</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹13,943</v>
+        <v>Receive ₹15,296</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -6900,11 +6999,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>94005.463999999993</v>
+        <v>95359.067999999999</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-81475.463999999993</v>
+        <v>-82829.067999999999</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -6912,11 +7011,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-15752.479999999981</v>
+        <v>-17106.083999999988</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹15,752</v>
+        <v>Receive ₹17,106</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -7028,7 +7127,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -7037,14 +7136,14 @@
       </c>
       <c r="B5" s="21">
         <f>Summary!B3</f>
-        <v>318951</v>
+        <v>344133</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>69</v>
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>281960</v>
+        <v>286020</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -7053,14 +7152,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-36991</v>
+        <v>-58113</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>115214.51999999999</v>
+        <v>140207.3833333333</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -7112,7 +7211,7 @@
       </c>
       <c r="G10" s="21">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>233</v>
+        <v>238</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -7136,7 +7235,7 @@
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>138</v>
+        <v>174</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -7162,15 +7261,15 @@
       </c>
       <c r="B13" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A13)*(YEAR(Purchases!$A$2:$A$998)=$B$7)*Purchases!$C$2:$C$998),0)</f>
-        <v>39660</v>
+        <v>64842</v>
       </c>
       <c r="C13" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$996,"MMM")=$A13)*(YEAR(Sales!$A$2:$A$996)=$B$7)*Sales!$C$2:$C$996),0)</f>
-        <v>47998</v>
+        <v>52577</v>
       </c>
       <c r="D13" s="27">
         <f t="shared" si="0"/>
-        <v>8338</v>
+        <v>-12265</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1">
@@ -7332,11 +7431,11 @@
       </c>
       <c r="G47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>69</v>
+        <v>105</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
@@ -7363,7 +7462,7 @@
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>50878.32</v>
+        <v>75871.18333333332</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -8358,7 +8457,7 @@
         <v>100</v>
       </c>
       <c r="D64" s="36" t="s">
-        <v>817</v>
+        <v>813</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="15" customHeight="1">
@@ -8404,16 +8503,32 @@
       </c>
     </row>
     <row r="68" spans="1:4" ht="15" customHeight="1">
-      <c r="A68" s="35"/>
-      <c r="B68" s="36"/>
-      <c r="C68" s="37"/>
-      <c r="D68" s="36"/>
+      <c r="A68" s="35">
+        <v>46140</v>
+      </c>
+      <c r="B68" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C68" s="37">
+        <v>42</v>
+      </c>
+      <c r="D68" s="36" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="69" spans="1:4" ht="15" customHeight="1">
-      <c r="A69" s="38"/>
-      <c r="B69" s="39"/>
-      <c r="C69" s="40"/>
-      <c r="D69" s="39"/>
+      <c r="A69" s="38">
+        <v>46140</v>
+      </c>
+      <c r="B69" s="39" t="s">
+        <v>49</v>
+      </c>
+      <c r="C69" s="40">
+        <v>25140</v>
+      </c>
+      <c r="D69" s="39" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="70" spans="1:4" ht="15" customHeight="1">
       <c r="A70" s="35"/>
@@ -14273,7 +14388,7 @@
       <c r="F146" s="91"/>
       <c r="G146" s="91"/>
       <c r="H146" s="92" t="s">
-        <v>843</v>
+        <v>839</v>
       </c>
       <c r="I146" s="80" t="s">
         <v>334</v>
@@ -14617,7 +14732,7 @@
       <c r="F160" s="91"/>
       <c r="G160" s="91"/>
       <c r="H160" s="92" t="s">
-        <v>818</v>
+        <v>814</v>
       </c>
       <c r="I160" s="80" t="s">
         <v>334</v>
@@ -14628,7 +14743,7 @@
         <v>46132</v>
       </c>
       <c r="B161" s="76" t="s">
-        <v>832</v>
+        <v>828</v>
       </c>
       <c r="C161" s="77">
         <v>1100</v>
@@ -14665,7 +14780,7 @@
       <c r="F162" s="91"/>
       <c r="G162" s="91"/>
       <c r="H162" s="92" t="s">
-        <v>846</v>
+        <v>841</v>
       </c>
       <c r="I162" s="80" t="s">
         <v>140</v>
@@ -14676,7 +14791,7 @@
         <v>46133</v>
       </c>
       <c r="B163" s="76" t="s">
-        <v>822</v>
+        <v>818</v>
       </c>
       <c r="C163" s="77">
         <v>1350</v>
@@ -14688,7 +14803,7 @@
       <c r="F163" s="76"/>
       <c r="G163" s="76"/>
       <c r="H163" s="78" t="s">
-        <v>823</v>
+        <v>819</v>
       </c>
       <c r="I163" s="76" t="s">
         <v>140</v>
@@ -14711,7 +14826,7 @@
       <c r="F164" s="91"/>
       <c r="G164" s="91"/>
       <c r="H164" s="92" t="s">
-        <v>824</v>
+        <v>820</v>
       </c>
       <c r="I164" s="80" t="s">
         <v>334</v>
@@ -14734,7 +14849,7 @@
       <c r="F165" s="76"/>
       <c r="G165" s="76"/>
       <c r="H165" s="78" t="s">
-        <v>825</v>
+        <v>821</v>
       </c>
       <c r="I165" s="76" t="s">
         <v>334</v>
@@ -14745,7 +14860,7 @@
         <v>46134</v>
       </c>
       <c r="B166" s="80" t="s">
-        <v>837</v>
+        <v>833</v>
       </c>
       <c r="C166" s="81">
         <v>1280</v>
@@ -14759,7 +14874,7 @@
       <c r="F166" s="91"/>
       <c r="G166" s="91"/>
       <c r="H166" s="92" t="s">
-        <v>839</v>
+        <v>835</v>
       </c>
       <c r="I166" s="80" t="s">
         <v>140</v>
@@ -14782,7 +14897,7 @@
       <c r="F167" s="76"/>
       <c r="G167" s="76"/>
       <c r="H167" s="78" t="s">
-        <v>835</v>
+        <v>831</v>
       </c>
       <c r="I167" s="76" t="s">
         <v>334</v>
@@ -14805,7 +14920,7 @@
       <c r="F168" s="76"/>
       <c r="G168" s="76"/>
       <c r="H168" s="78" t="s">
-        <v>844</v>
+        <v>840</v>
       </c>
       <c r="I168" s="76" t="s">
         <v>334</v>
@@ -14828,7 +14943,7 @@
       <c r="F169" s="91"/>
       <c r="G169" s="91"/>
       <c r="H169" s="92" t="s">
-        <v>841</v>
+        <v>837</v>
       </c>
       <c r="I169" s="80" t="s">
         <v>334</v>
@@ -14839,7 +14954,7 @@
         <v>46134</v>
       </c>
       <c r="B170" s="76" t="s">
-        <v>836</v>
+        <v>832</v>
       </c>
       <c r="C170" s="77">
         <v>650</v>
@@ -14853,7 +14968,7 @@
       <c r="F170" s="76"/>
       <c r="G170" s="76"/>
       <c r="H170" s="78" t="s">
-        <v>842</v>
+        <v>838</v>
       </c>
       <c r="I170" s="76" t="s">
         <v>140</v>
@@ -14876,7 +14991,7 @@
       <c r="F171" s="91"/>
       <c r="G171" s="91"/>
       <c r="H171" s="92" t="s">
-        <v>847</v>
+        <v>842</v>
       </c>
       <c r="I171" s="80" t="s">
         <v>334</v>
@@ -14887,19 +15002,21 @@
         <v>46138</v>
       </c>
       <c r="B172" s="76" t="s">
-        <v>850</v>
+        <v>844</v>
       </c>
       <c r="C172" s="77">
         <v>690</v>
       </c>
-      <c r="D172" s="76"/>
+      <c r="D172" s="76" t="s">
+        <v>154</v>
+      </c>
       <c r="E172" s="76" t="s">
         <v>49</v>
       </c>
       <c r="F172" s="76"/>
       <c r="G172" s="76"/>
       <c r="H172" s="78" t="s">
-        <v>849</v>
+        <v>843</v>
       </c>
       <c r="I172" s="76" t="s">
         <v>140</v>
@@ -14910,19 +15027,21 @@
         <v>46138</v>
       </c>
       <c r="B173" s="80" t="s">
-        <v>851</v>
+        <v>845</v>
       </c>
       <c r="C173" s="81">
         <v>1099</v>
       </c>
-      <c r="D173" s="80"/>
+      <c r="D173" s="80" t="s">
+        <v>154</v>
+      </c>
       <c r="E173" s="80" t="s">
         <v>49</v>
       </c>
       <c r="F173" s="91"/>
       <c r="G173" s="91"/>
       <c r="H173" s="92" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="I173" s="80" t="s">
         <v>140</v>
@@ -14933,7 +15052,7 @@
         <v>46139</v>
       </c>
       <c r="B174" s="76" t="s">
-        <v>854</v>
+        <v>846</v>
       </c>
       <c r="C174" s="77">
         <v>690</v>
@@ -14947,7 +15066,7 @@
       <c r="F174" s="76"/>
       <c r="G174" s="76"/>
       <c r="H174" s="78" t="s">
-        <v>855</v>
+        <v>847</v>
       </c>
       <c r="I174" s="76" t="s">
         <v>140</v>
@@ -14958,7 +15077,7 @@
         <v>46139</v>
       </c>
       <c r="B175" s="80" t="s">
-        <v>856</v>
+        <v>848</v>
       </c>
       <c r="C175" s="81">
         <v>690</v>
@@ -14972,7 +15091,7 @@
       <c r="F175" s="91"/>
       <c r="G175" s="91"/>
       <c r="H175" s="92" t="s">
-        <v>849</v>
+        <v>843</v>
       </c>
       <c r="I175" s="80" t="s">
         <v>140</v>
@@ -14983,7 +15102,7 @@
         <v>46139</v>
       </c>
       <c r="B176" s="76" t="s">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="C176" s="77">
         <v>690</v>
@@ -14997,7 +15116,7 @@
       <c r="F176" s="76"/>
       <c r="G176" s="76"/>
       <c r="H176" s="78" t="s">
-        <v>858</v>
+        <v>850</v>
       </c>
       <c r="I176" s="76" t="s">
         <v>140</v>
@@ -15007,9 +15126,11 @@
       <c r="A177" s="79">
         <v>46140</v>
       </c>
-      <c r="B177" s="80"/>
+      <c r="B177" s="80" t="s">
+        <v>852</v>
+      </c>
       <c r="C177" s="81">
-        <v>690</v>
+        <v>1380</v>
       </c>
       <c r="D177" s="80" t="s">
         <v>154</v>
@@ -15020,22 +15141,24 @@
       <c r="F177" s="91"/>
       <c r="G177" s="91"/>
       <c r="H177" s="92" t="s">
-        <v>862</v>
+        <v>853</v>
       </c>
       <c r="I177" s="80" t="s">
-        <v>334</v>
+        <v>140</v>
       </c>
     </row>
     <row r="178" spans="1:9" ht="14">
       <c r="A178" s="75">
         <v>46140</v>
       </c>
-      <c r="B178" s="76"/>
+      <c r="B178" s="76" t="s">
+        <v>178</v>
+      </c>
       <c r="C178" s="77">
-        <v>690</v>
+        <v>1480</v>
       </c>
       <c r="D178" s="76" t="s">
-        <v>293</v>
+        <v>154</v>
       </c>
       <c r="E178" s="76" t="s">
         <v>49</v>
@@ -15043,33 +15166,61 @@
       <c r="F178" s="76"/>
       <c r="G178" s="76"/>
       <c r="H178" s="78" t="s">
+        <v>854</v>
+      </c>
+      <c r="I178" s="76" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="179" spans="1:9" ht="14">
+      <c r="A179" s="79">
+        <v>46140</v>
+      </c>
+      <c r="B179" s="80" t="s">
         <v>863</v>
       </c>
-      <c r="I178" s="76" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="179" spans="1:9">
-      <c r="A179" s="79"/>
-      <c r="B179" s="80"/>
-      <c r="C179" s="81"/>
-      <c r="D179" s="80"/>
-      <c r="E179" s="80"/>
+      <c r="C179" s="81">
+        <v>1200</v>
+      </c>
+      <c r="D179" s="80" t="s">
+        <v>154</v>
+      </c>
+      <c r="E179" s="80" t="s">
+        <v>49</v>
+      </c>
       <c r="F179" s="91"/>
       <c r="G179" s="91"/>
-      <c r="H179" s="92"/>
-      <c r="I179" s="80"/>
-    </row>
-    <row r="180" spans="1:9">
-      <c r="A180" s="75"/>
-      <c r="B180" s="76"/>
-      <c r="C180" s="77"/>
-      <c r="D180" s="76"/>
-      <c r="E180" s="76"/>
+      <c r="H179" s="92" t="s">
+        <v>864</v>
+      </c>
+      <c r="I179" s="80" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="180" spans="1:9" ht="28">
+      <c r="A180" s="75">
+        <v>46140</v>
+      </c>
+      <c r="B180" s="76" t="s">
+        <v>868</v>
+      </c>
+      <c r="C180" s="77">
+        <v>1899</v>
+      </c>
+      <c r="D180" s="76" t="s">
+        <v>154</v>
+      </c>
+      <c r="E180" s="76" t="s">
+        <v>49</v>
+      </c>
       <c r="F180" s="76"/>
       <c r="G180" s="76"/>
-      <c r="H180" s="78"/>
-      <c r="I180" s="76"/>
+      <c r="H180" s="78" t="s">
+        <v>867</v>
+      </c>
+      <c r="I180" s="76" t="s">
+        <v>334</v>
+      </c>
     </row>
     <row r="181" spans="1:9">
       <c r="A181" s="79"/>
@@ -15949,7 +16100,7 @@
       <c r="I260" s="84"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I173" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:I180" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1260" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"Ordered,Pending,Completed,Cancelled"</formula1>
@@ -15969,7 +16120,7 @@
     <col min="1" max="1" width="10" style="43" customWidth="1"/>
     <col min="2" max="2" width="94.33203125" style="43" customWidth="1"/>
     <col min="3" max="3" width="13.83203125" style="43" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" style="43" customWidth="1"/>
+    <col min="4" max="4" width="17.5" style="43" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.33203125" style="43" customWidth="1"/>
     <col min="6" max="6" width="8.1640625" style="43" customWidth="1"/>
     <col min="7" max="7" width="11.1640625" style="43" customWidth="1"/>
@@ -22896,7 +23047,7 @@
         <v>0</v>
       </c>
       <c r="L65" s="42" t="s">
-        <v>838</v>
+        <v>834</v>
       </c>
       <c r="M65" s="42"/>
       <c r="N65" s="42" t="s">
@@ -23638,7 +23789,7 @@
         <v>0</v>
       </c>
       <c r="L79" s="42" t="s">
-        <v>840</v>
+        <v>836</v>
       </c>
       <c r="M79" s="42"/>
       <c r="N79" s="42" t="s">
@@ -23958,7 +24109,7 @@
         <v>895</v>
       </c>
       <c r="L85" s="42" t="s">
-        <v>831</v>
+        <v>827</v>
       </c>
       <c r="M85" s="42"/>
       <c r="N85" s="42" t="s">
@@ -24252,10 +24403,10 @@
         <v>689</v>
       </c>
       <c r="F91" s="51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G91" s="51">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H91" s="42">
         <f t="shared" si="6"/>
@@ -24267,18 +24418,18 @@
       </c>
       <c r="J91" s="42">
         <f t="shared" si="7"/>
-        <v>389</v>
+        <v>778</v>
       </c>
       <c r="K91" s="42">
         <f t="shared" si="8"/>
-        <v>389</v>
+        <v>0</v>
       </c>
       <c r="L91" s="42" t="s">
-        <v>578</v>
+        <v>856</v>
       </c>
       <c r="M91" s="42"/>
       <c r="N91" s="42" t="s">
-        <v>538</v>
+        <v>366</v>
       </c>
       <c r="O91" s="42"/>
       <c r="P91" s="42"/>
@@ -24289,10 +24440,10 @@
     </row>
     <row r="92" spans="1:20" ht="15" customHeight="1">
       <c r="A92" s="48" t="s">
+        <v>578</v>
+      </c>
+      <c r="B92" s="48" t="s">
         <v>579</v>
-      </c>
-      <c r="B92" s="48" t="s">
-        <v>580</v>
       </c>
       <c r="C92" s="48" t="s">
         <v>577</v>
@@ -24326,7 +24477,7 @@
         <v>0</v>
       </c>
       <c r="L92" s="48" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="M92" s="48"/>
       <c r="N92" s="48" t="s">
@@ -24341,10 +24492,10 @@
     </row>
     <row r="93" spans="1:20" ht="15" customHeight="1">
       <c r="A93" s="42" t="s">
+        <v>581</v>
+      </c>
+      <c r="B93" s="42" t="s">
         <v>582</v>
-      </c>
-      <c r="B93" s="42" t="s">
-        <v>583</v>
       </c>
       <c r="C93" s="42" t="s">
         <v>97</v>
@@ -24378,14 +24529,14 @@
         <v>944</v>
       </c>
       <c r="L93" s="42" t="s">
-        <v>820</v>
+        <v>816</v>
       </c>
       <c r="M93" s="42"/>
       <c r="N93" s="48" t="s">
         <v>451</v>
       </c>
       <c r="O93" s="42" t="s">
-        <v>821</v>
+        <v>817</v>
       </c>
       <c r="P93" s="42"/>
       <c r="Q93" s="42"/>
@@ -24395,10 +24546,10 @@
     </row>
     <row r="94" spans="1:20" ht="15" customHeight="1">
       <c r="A94" s="48" t="s">
+        <v>583</v>
+      </c>
+      <c r="B94" s="48" t="s">
         <v>584</v>
-      </c>
-      <c r="B94" s="48" t="s">
-        <v>585</v>
       </c>
       <c r="C94" s="48" t="s">
         <v>95</v>
@@ -24447,10 +24598,10 @@
     </row>
     <row r="95" spans="1:20" ht="15" customHeight="1">
       <c r="A95" s="42" t="s">
+        <v>585</v>
+      </c>
+      <c r="B95" s="42" t="s">
         <v>586</v>
-      </c>
-      <c r="B95" s="42" t="s">
-        <v>587</v>
       </c>
       <c r="C95" s="42" t="s">
         <v>95</v>
@@ -24484,7 +24635,7 @@
         <v>0</v>
       </c>
       <c r="L95" s="42" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="M95" s="42"/>
       <c r="N95" s="42" t="s">
@@ -24499,10 +24650,10 @@
     </row>
     <row r="96" spans="1:20" ht="15" customHeight="1">
       <c r="A96" s="48" t="s">
+        <v>588</v>
+      </c>
+      <c r="B96" s="48" t="s">
         <v>589</v>
-      </c>
-      <c r="B96" s="48" t="s">
-        <v>590</v>
       </c>
       <c r="C96" s="48" t="s">
         <v>95</v>
@@ -24549,10 +24700,10 @@
     </row>
     <row r="97" spans="1:20" ht="15" customHeight="1">
       <c r="A97" s="42" t="s">
+        <v>590</v>
+      </c>
+      <c r="B97" s="42" t="s">
         <v>591</v>
-      </c>
-      <c r="B97" s="42" t="s">
-        <v>592</v>
       </c>
       <c r="C97" s="42" t="s">
         <v>95</v>
@@ -24601,10 +24752,10 @@
     </row>
     <row r="98" spans="1:20" ht="15" customHeight="1">
       <c r="A98" s="48" t="s">
+        <v>592</v>
+      </c>
+      <c r="B98" s="48" t="s">
         <v>593</v>
-      </c>
-      <c r="B98" s="48" t="s">
-        <v>594</v>
       </c>
       <c r="C98" s="48" t="s">
         <v>96</v>
@@ -24655,10 +24806,10 @@
     </row>
     <row r="99" spans="1:20" ht="15" customHeight="1">
       <c r="A99" s="42" t="s">
+        <v>594</v>
+      </c>
+      <c r="B99" s="42" t="s">
         <v>595</v>
-      </c>
-      <c r="B99" s="42" t="s">
-        <v>596</v>
       </c>
       <c r="C99" s="42" t="s">
         <v>96</v>
@@ -24709,10 +24860,10 @@
     </row>
     <row r="100" spans="1:20" ht="15" customHeight="1">
       <c r="A100" s="48" t="s">
+        <v>596</v>
+      </c>
+      <c r="B100" s="48" t="s">
         <v>597</v>
-      </c>
-      <c r="B100" s="48" t="s">
-        <v>598</v>
       </c>
       <c r="C100" s="48" t="s">
         <v>96</v>
@@ -24763,10 +24914,10 @@
     </row>
     <row r="101" spans="1:20" ht="15" customHeight="1">
       <c r="A101" s="42" t="s">
+        <v>598</v>
+      </c>
+      <c r="B101" s="42" t="s">
         <v>599</v>
-      </c>
-      <c r="B101" s="42" t="s">
-        <v>600</v>
       </c>
       <c r="C101" s="42" t="s">
         <v>96</v>
@@ -24817,10 +24968,10 @@
     </row>
     <row r="102" spans="1:20" ht="15" customHeight="1">
       <c r="A102" s="48" t="s">
+        <v>600</v>
+      </c>
+      <c r="B102" s="48" t="s">
         <v>601</v>
-      </c>
-      <c r="B102" s="48" t="s">
-        <v>602</v>
       </c>
       <c r="C102" s="48" t="s">
         <v>96</v>
@@ -24871,10 +25022,10 @@
     </row>
     <row r="103" spans="1:20" ht="15" customHeight="1">
       <c r="A103" s="42" t="s">
+        <v>602</v>
+      </c>
+      <c r="B103" s="42" t="s">
         <v>603</v>
-      </c>
-      <c r="B103" s="42" t="s">
-        <v>604</v>
       </c>
       <c r="C103" s="42" t="s">
         <v>96</v>
@@ -24925,10 +25076,10 @@
     </row>
     <row r="104" spans="1:20" ht="15" customHeight="1">
       <c r="A104" s="48" t="s">
+        <v>604</v>
+      </c>
+      <c r="B104" s="48" t="s">
         <v>605</v>
-      </c>
-      <c r="B104" s="48" t="s">
-        <v>606</v>
       </c>
       <c r="C104" s="48" t="s">
         <v>96</v>
@@ -24979,10 +25130,10 @@
     </row>
     <row r="105" spans="1:20" ht="15" customHeight="1">
       <c r="A105" s="42" t="s">
+        <v>606</v>
+      </c>
+      <c r="B105" s="42" t="s">
         <v>607</v>
-      </c>
-      <c r="B105" s="42" t="s">
-        <v>608</v>
       </c>
       <c r="C105" s="42" t="s">
         <v>96</v>
@@ -25033,10 +25184,10 @@
     </row>
     <row r="106" spans="1:20" ht="15" customHeight="1">
       <c r="A106" s="48" t="s">
+        <v>608</v>
+      </c>
+      <c r="B106" s="48" t="s">
         <v>609</v>
-      </c>
-      <c r="B106" s="48" t="s">
-        <v>610</v>
       </c>
       <c r="C106" s="48" t="s">
         <v>96</v>
@@ -25085,10 +25236,10 @@
     </row>
     <row r="107" spans="1:20" ht="15" customHeight="1">
       <c r="A107" s="42" t="s">
+        <v>610</v>
+      </c>
+      <c r="B107" s="42" t="s">
         <v>611</v>
-      </c>
-      <c r="B107" s="42" t="s">
-        <v>612</v>
       </c>
       <c r="C107" s="42" t="s">
         <v>96</v>
@@ -25139,10 +25290,10 @@
     </row>
     <row r="108" spans="1:20" ht="15" customHeight="1">
       <c r="A108" s="48" t="s">
+        <v>612</v>
+      </c>
+      <c r="B108" s="48" t="s">
         <v>613</v>
-      </c>
-      <c r="B108" s="48" t="s">
-        <v>614</v>
       </c>
       <c r="C108" s="48" t="s">
         <v>96</v>
@@ -25193,10 +25344,10 @@
     </row>
     <row r="109" spans="1:20" ht="15" customHeight="1">
       <c r="A109" s="42" t="s">
+        <v>614</v>
+      </c>
+      <c r="B109" s="42" t="s">
         <v>615</v>
-      </c>
-      <c r="B109" s="42" t="s">
-        <v>616</v>
       </c>
       <c r="C109" s="42" t="s">
         <v>96</v>
@@ -25247,10 +25398,10 @@
     </row>
     <row r="110" spans="1:20" ht="15" customHeight="1">
       <c r="A110" s="48" t="s">
+        <v>616</v>
+      </c>
+      <c r="B110" s="48" t="s">
         <v>617</v>
-      </c>
-      <c r="B110" s="48" t="s">
-        <v>618</v>
       </c>
       <c r="C110" s="48" t="s">
         <v>96</v>
@@ -25301,10 +25452,10 @@
     </row>
     <row r="111" spans="1:20" ht="15" customHeight="1">
       <c r="A111" s="42" t="s">
+        <v>618</v>
+      </c>
+      <c r="B111" s="42" t="s">
         <v>619</v>
-      </c>
-      <c r="B111" s="42" t="s">
-        <v>620</v>
       </c>
       <c r="C111" s="42" t="s">
         <v>96</v>
@@ -25355,10 +25506,10 @@
     </row>
     <row r="112" spans="1:20" ht="15" customHeight="1">
       <c r="A112" s="48" t="s">
+        <v>620</v>
+      </c>
+      <c r="B112" s="48" t="s">
         <v>621</v>
-      </c>
-      <c r="B112" s="48" t="s">
-        <v>622</v>
       </c>
       <c r="C112" s="48" t="s">
         <v>96</v>
@@ -25407,10 +25558,10 @@
     </row>
     <row r="113" spans="1:246" ht="15" customHeight="1">
       <c r="A113" s="42" t="s">
+        <v>622</v>
+      </c>
+      <c r="B113" s="42" t="s">
         <v>623</v>
-      </c>
-      <c r="B113" s="42" t="s">
-        <v>624</v>
       </c>
       <c r="C113" s="42" t="s">
         <v>96</v>
@@ -25461,10 +25612,10 @@
     </row>
     <row r="114" spans="1:246" ht="15" customHeight="1">
       <c r="A114" s="48" t="s">
+        <v>624</v>
+      </c>
+      <c r="B114" s="48" t="s">
         <v>625</v>
-      </c>
-      <c r="B114" s="48" t="s">
-        <v>626</v>
       </c>
       <c r="C114" s="48" t="s">
         <v>95</v>
@@ -25513,10 +25664,10 @@
     </row>
     <row r="115" spans="1:246" ht="30" customHeight="1">
       <c r="A115" s="42" t="s">
+        <v>626</v>
+      </c>
+      <c r="B115" s="42" t="s">
         <v>627</v>
-      </c>
-      <c r="B115" s="42" t="s">
-        <v>628</v>
       </c>
       <c r="C115" s="42" t="s">
         <v>95</v>
@@ -25550,7 +25701,7 @@
         <v>0</v>
       </c>
       <c r="L115" s="42" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M115" s="42"/>
       <c r="N115" s="42" t="s">
@@ -25565,10 +25716,10 @@
     </row>
     <row r="116" spans="1:246" ht="150" customHeight="1">
       <c r="A116" s="48" t="s">
+        <v>629</v>
+      </c>
+      <c r="B116" s="48" t="s">
         <v>630</v>
-      </c>
-      <c r="B116" s="48" t="s">
-        <v>631</v>
       </c>
       <c r="C116" s="48" t="s">
         <v>95</v>
@@ -25602,7 +25753,7 @@
         <v>0</v>
       </c>
       <c r="L116" s="48" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="M116" s="48"/>
       <c r="N116" s="48" t="s">
@@ -25617,10 +25768,10 @@
     </row>
     <row r="117" spans="1:246" ht="15" customHeight="1">
       <c r="A117" s="42" t="s">
+        <v>632</v>
+      </c>
+      <c r="B117" s="42" t="s">
         <v>633</v>
-      </c>
-      <c r="B117" s="42" t="s">
-        <v>634</v>
       </c>
       <c r="C117" s="42" t="s">
         <v>95</v>
@@ -25669,10 +25820,10 @@
     </row>
     <row r="118" spans="1:246" ht="15" customHeight="1">
       <c r="A118" s="48" t="s">
+        <v>634</v>
+      </c>
+      <c r="B118" s="48" t="s">
         <v>635</v>
-      </c>
-      <c r="B118" s="48" t="s">
-        <v>636</v>
       </c>
       <c r="C118" s="48" t="s">
         <v>95</v>
@@ -25706,7 +25857,7 @@
         <v>2095.8000000000002</v>
       </c>
       <c r="L118" s="48" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="M118" s="48"/>
       <c r="N118" s="48" t="s">
@@ -25714,7 +25865,7 @@
       </c>
       <c r="O118" s="48"/>
       <c r="P118" s="48" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="Q118" s="48"/>
       <c r="R118" s="48"/>
@@ -25723,10 +25874,10 @@
     </row>
     <row r="119" spans="1:246" ht="15" customHeight="1">
       <c r="A119" s="42" t="s">
+        <v>638</v>
+      </c>
+      <c r="B119" s="42" t="s">
         <v>639</v>
-      </c>
-      <c r="B119" s="42" t="s">
-        <v>640</v>
       </c>
       <c r="C119" s="42" t="s">
         <v>95</v>
@@ -25775,10 +25926,10 @@
     </row>
     <row r="120" spans="1:246" ht="83" customHeight="1">
       <c r="A120" s="48" t="s">
+        <v>640</v>
+      </c>
+      <c r="B120" s="48" t="s">
         <v>641</v>
-      </c>
-      <c r="B120" s="48" t="s">
-        <v>642</v>
       </c>
       <c r="C120" s="48" t="s">
         <v>95</v>
@@ -25793,11 +25944,11 @@
         <v>10</v>
       </c>
       <c r="G120" s="49">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="H120" s="48">
         <f t="shared" si="9"/>
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="I120" s="48">
         <f>IF(D120&lt;&gt;"",D120,IFERROR(E120/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -25809,10 +25960,10 @@
       </c>
       <c r="K120" s="48">
         <f t="shared" si="11"/>
-        <v>1256.859999999999</v>
+        <v>9216.9733333333261</v>
       </c>
       <c r="L120" s="48" t="s">
-        <v>861</v>
+        <v>866</v>
       </c>
       <c r="M120" s="48" t="s">
         <v>49</v>
@@ -25822,7 +25973,7 @@
       </c>
       <c r="O120" s="48"/>
       <c r="P120" s="48" t="s">
-        <v>853</v>
+        <v>865</v>
       </c>
       <c r="Q120" s="48"/>
       <c r="R120" s="48"/>
@@ -25831,10 +25982,10 @@
     </row>
     <row r="121" spans="1:246" ht="15" customHeight="1">
       <c r="A121" s="42" t="s">
+        <v>642</v>
+      </c>
+      <c r="B121" s="42" t="s">
         <v>643</v>
-      </c>
-      <c r="B121" s="42" t="s">
-        <v>644</v>
       </c>
       <c r="C121" s="42" t="s">
         <v>95</v>
@@ -25868,7 +26019,7 @@
         <v>0</v>
       </c>
       <c r="L121" s="42" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="M121" s="42"/>
       <c r="N121" s="42" t="s">
@@ -25876,7 +26027,7 @@
       </c>
       <c r="O121" s="42"/>
       <c r="P121" s="42" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="Q121" s="42"/>
       <c r="R121" s="42"/>
@@ -25885,10 +26036,10 @@
     </row>
     <row r="122" spans="1:246" ht="15" customHeight="1">
       <c r="A122" s="48" t="s">
+        <v>646</v>
+      </c>
+      <c r="B122" s="48" t="s">
         <v>647</v>
-      </c>
-      <c r="B122" s="48" t="s">
-        <v>648</v>
       </c>
       <c r="C122" s="48" t="s">
         <v>96</v>
@@ -25922,14 +26073,14 @@
         <v>3525</v>
       </c>
       <c r="L122" s="48" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="M122" s="48"/>
       <c r="N122" s="48" t="s">
         <v>451</v>
       </c>
       <c r="O122" s="48" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="P122" s="48"/>
       <c r="Q122" s="48"/>
@@ -25939,10 +26090,10 @@
     </row>
     <row r="123" spans="1:246" s="53" customFormat="1" ht="75" customHeight="1">
       <c r="A123" s="59" t="s">
+        <v>650</v>
+      </c>
+      <c r="B123" s="59" t="s">
         <v>651</v>
-      </c>
-      <c r="B123" s="59" t="s">
-        <v>652</v>
       </c>
       <c r="C123" s="59" t="s">
         <v>95</v>
@@ -25976,7 +26127,7 @@
         <v>891.44</v>
       </c>
       <c r="L123" s="59" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="M123" s="59"/>
       <c r="N123" s="59" t="s">
@@ -26217,10 +26368,10 @@
     </row>
     <row r="124" spans="1:246" s="64" customFormat="1" ht="30" customHeight="1">
       <c r="A124" s="61" t="s">
+        <v>653</v>
+      </c>
+      <c r="B124" s="61" t="s">
         <v>654</v>
-      </c>
-      <c r="B124" s="61" t="s">
-        <v>655</v>
       </c>
       <c r="C124" s="61" t="s">
         <v>95</v>
@@ -26254,7 +26405,7 @@
         <v>0</v>
       </c>
       <c r="L124" s="61" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="M124" s="61"/>
       <c r="N124" s="61" t="s">
@@ -26497,10 +26648,10 @@
     </row>
     <row r="125" spans="1:246" s="53" customFormat="1" ht="15" customHeight="1">
       <c r="A125" s="59" t="s">
+        <v>656</v>
+      </c>
+      <c r="B125" s="59" t="s">
         <v>657</v>
-      </c>
-      <c r="B125" s="59" t="s">
-        <v>658</v>
       </c>
       <c r="C125" s="59" t="s">
         <v>95</v>
@@ -26534,7 +26685,7 @@
         <v>0</v>
       </c>
       <c r="L125" s="59" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="M125" s="59"/>
       <c r="N125" s="59" t="s">
@@ -26542,7 +26693,7 @@
       </c>
       <c r="O125" s="59"/>
       <c r="P125" s="59" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="Q125" s="59"/>
       <c r="R125" s="59"/>
@@ -26777,10 +26928,10 @@
     </row>
     <row r="126" spans="1:246" ht="15" customHeight="1">
       <c r="A126" s="61" t="s">
+        <v>660</v>
+      </c>
+      <c r="B126" s="48" t="s">
         <v>661</v>
-      </c>
-      <c r="B126" s="48" t="s">
-        <v>662</v>
       </c>
       <c r="C126" s="48" t="s">
         <v>96</v>
@@ -26814,14 +26965,14 @@
         <v>0</v>
       </c>
       <c r="L126" s="48" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="M126" s="48"/>
       <c r="N126" s="48" t="s">
         <v>366</v>
       </c>
       <c r="O126" s="48" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="P126" s="48"/>
       <c r="Q126" s="48"/>
@@ -26831,10 +26982,10 @@
     </row>
     <row r="127" spans="1:246" ht="15" customHeight="1">
       <c r="A127" s="59" t="s">
+        <v>664</v>
+      </c>
+      <c r="B127" s="42" t="s">
         <v>665</v>
-      </c>
-      <c r="B127" s="42" t="s">
-        <v>666</v>
       </c>
       <c r="C127" s="42" t="s">
         <v>96</v>
@@ -26885,10 +27036,10 @@
     </row>
     <row r="128" spans="1:246" ht="15" customHeight="1">
       <c r="A128" s="61" t="s">
+        <v>666</v>
+      </c>
+      <c r="B128" s="48" t="s">
         <v>667</v>
-      </c>
-      <c r="B128" s="48" t="s">
-        <v>668</v>
       </c>
       <c r="C128" s="48" t="s">
         <v>95</v>
@@ -26935,10 +27086,10 @@
     </row>
     <row r="129" spans="1:20" ht="15" customHeight="1">
       <c r="A129" s="59" t="s">
+        <v>668</v>
+      </c>
+      <c r="B129" s="42" t="s">
         <v>669</v>
-      </c>
-      <c r="B129" s="42" t="s">
-        <v>670</v>
       </c>
       <c r="C129" s="42" t="s">
         <v>95</v>
@@ -26972,7 +27123,7 @@
         <v>0</v>
       </c>
       <c r="L129" s="42" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="M129" s="42"/>
       <c r="N129" s="42" t="s">
@@ -26987,10 +27138,10 @@
     </row>
     <row r="130" spans="1:20" ht="15" customHeight="1">
       <c r="A130" s="61" t="s">
+        <v>671</v>
+      </c>
+      <c r="B130" s="48" t="s">
         <v>672</v>
-      </c>
-      <c r="B130" s="48" t="s">
-        <v>673</v>
       </c>
       <c r="C130" s="48" t="s">
         <v>95</v>
@@ -27024,7 +27175,7 @@
         <v>0</v>
       </c>
       <c r="L130" s="48" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="M130" s="48"/>
       <c r="N130" s="48" t="s">
@@ -27039,10 +27190,10 @@
     </row>
     <row r="131" spans="1:20" ht="15" customHeight="1">
       <c r="A131" s="59" t="s">
+        <v>674</v>
+      </c>
+      <c r="B131" s="42" t="s">
         <v>675</v>
-      </c>
-      <c r="B131" s="42" t="s">
-        <v>676</v>
       </c>
       <c r="C131" s="42" t="s">
         <v>95</v>
@@ -27089,10 +27240,10 @@
     </row>
     <row r="132" spans="1:20" ht="15" customHeight="1">
       <c r="A132" s="61" t="s">
+        <v>676</v>
+      </c>
+      <c r="B132" s="48" t="s">
         <v>677</v>
-      </c>
-      <c r="B132" s="48" t="s">
-        <v>678</v>
       </c>
       <c r="C132" s="48" t="s">
         <v>95</v>
@@ -27126,7 +27277,7 @@
         <v>0</v>
       </c>
       <c r="L132" s="48" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="M132" s="48"/>
       <c r="N132" s="48" t="s">
@@ -27141,10 +27292,10 @@
     </row>
     <row r="133" spans="1:20" ht="15" customHeight="1">
       <c r="A133" s="59" t="s">
+        <v>679</v>
+      </c>
+      <c r="B133" s="42" t="s">
         <v>680</v>
-      </c>
-      <c r="B133" s="42" t="s">
-        <v>681</v>
       </c>
       <c r="C133" s="42" t="s">
         <v>95</v>
@@ -27191,10 +27342,10 @@
     </row>
     <row r="134" spans="1:20" ht="15" customHeight="1">
       <c r="A134" s="61" t="s">
+        <v>681</v>
+      </c>
+      <c r="B134" s="48" t="s">
         <v>682</v>
-      </c>
-      <c r="B134" s="48" t="s">
-        <v>683</v>
       </c>
       <c r="C134" s="48" t="s">
         <v>95</v>
@@ -27241,10 +27392,10 @@
     </row>
     <row r="135" spans="1:20" ht="15" customHeight="1">
       <c r="A135" s="59" t="s">
+        <v>683</v>
+      </c>
+      <c r="B135" s="42" t="s">
         <v>684</v>
-      </c>
-      <c r="B135" s="42" t="s">
-        <v>685</v>
       </c>
       <c r="C135" s="42" t="s">
         <v>95</v>
@@ -27278,7 +27429,7 @@
         <v>0</v>
       </c>
       <c r="L135" s="42" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="M135" s="42"/>
       <c r="N135" s="42" t="s">
@@ -27293,10 +27444,10 @@
     </row>
     <row r="136" spans="1:20" ht="15" customHeight="1">
       <c r="A136" s="61" t="s">
+        <v>686</v>
+      </c>
+      <c r="B136" s="48" t="s">
         <v>687</v>
-      </c>
-      <c r="B136" s="48" t="s">
-        <v>688</v>
       </c>
       <c r="C136" s="48" t="s">
         <v>95</v>
@@ -27330,7 +27481,7 @@
         <v>0</v>
       </c>
       <c r="L136" s="48" t="s">
-        <v>834</v>
+        <v>830</v>
       </c>
       <c r="M136" s="48"/>
       <c r="N136" s="48" t="s">
@@ -27338,7 +27489,7 @@
       </c>
       <c r="O136" s="48"/>
       <c r="P136" s="48" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="Q136" s="48"/>
       <c r="R136" s="48"/>
@@ -27347,10 +27498,10 @@
     </row>
     <row r="137" spans="1:20" ht="15" customHeight="1">
       <c r="A137" s="59" t="s">
+        <v>689</v>
+      </c>
+      <c r="B137" s="42" t="s">
         <v>690</v>
-      </c>
-      <c r="B137" s="42" t="s">
-        <v>691</v>
       </c>
       <c r="C137" s="42" t="s">
         <v>95</v>
@@ -27399,10 +27550,10 @@
     </row>
     <row r="138" spans="1:20" ht="15" customHeight="1">
       <c r="A138" s="61" t="s">
+        <v>691</v>
+      </c>
+      <c r="B138" s="48" t="s">
         <v>692</v>
-      </c>
-      <c r="B138" s="48" t="s">
-        <v>693</v>
       </c>
       <c r="C138" s="48" t="s">
         <v>95</v>
@@ -27436,7 +27587,7 @@
         <v>0</v>
       </c>
       <c r="L138" s="48" t="s">
-        <v>833</v>
+        <v>829</v>
       </c>
       <c r="M138" s="48"/>
       <c r="N138" s="48" t="s">
@@ -27451,10 +27602,10 @@
     </row>
     <row r="139" spans="1:20" ht="15" customHeight="1">
       <c r="A139" s="59" t="s">
+        <v>693</v>
+      </c>
+      <c r="B139" s="42" t="s">
         <v>694</v>
-      </c>
-      <c r="B139" s="42" t="s">
-        <v>695</v>
       </c>
       <c r="C139" s="42" t="s">
         <v>95</v>
@@ -27503,10 +27654,10 @@
     </row>
     <row r="140" spans="1:20" ht="15" customHeight="1">
       <c r="A140" s="61" t="s">
+        <v>695</v>
+      </c>
+      <c r="B140" s="48" t="s">
         <v>696</v>
-      </c>
-      <c r="B140" s="48" t="s">
-        <v>697</v>
       </c>
       <c r="C140" s="48" t="s">
         <v>95</v>
@@ -27540,7 +27691,7 @@
         <v>699</v>
       </c>
       <c r="L140" s="48" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="M140" s="48"/>
       <c r="N140" s="48" t="s">
@@ -27555,10 +27706,10 @@
     </row>
     <row r="141" spans="1:20" ht="15" customHeight="1">
       <c r="A141" s="59" t="s">
+        <v>698</v>
+      </c>
+      <c r="B141" s="42" t="s">
         <v>699</v>
-      </c>
-      <c r="B141" s="42" t="s">
-        <v>700</v>
       </c>
       <c r="C141" s="42" t="s">
         <v>95</v>
@@ -27605,10 +27756,10 @@
     </row>
     <row r="142" spans="1:20" ht="15" customHeight="1">
       <c r="A142" s="48" t="s">
+        <v>700</v>
+      </c>
+      <c r="B142" s="48" t="s">
         <v>701</v>
-      </c>
-      <c r="B142" s="48" t="s">
-        <v>702</v>
       </c>
       <c r="C142" s="48" t="s">
         <v>95</v>
@@ -27642,7 +27793,7 @@
         <v>600</v>
       </c>
       <c r="L142" s="48" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="M142" s="48"/>
       <c r="N142" s="48" t="s">
@@ -27659,10 +27810,10 @@
     </row>
     <row r="143" spans="1:20" ht="15" customHeight="1">
       <c r="A143" s="42" t="s">
+        <v>703</v>
+      </c>
+      <c r="B143" s="42" t="s">
         <v>704</v>
-      </c>
-      <c r="B143" s="42" t="s">
-        <v>705</v>
       </c>
       <c r="C143" s="42" t="s">
         <v>95</v>
@@ -27709,10 +27860,10 @@
     </row>
     <row r="144" spans="1:20" ht="15" customHeight="1">
       <c r="A144" s="48" t="s">
+        <v>705</v>
+      </c>
+      <c r="B144" s="48" t="s">
         <v>706</v>
-      </c>
-      <c r="B144" s="48" t="s">
-        <v>707</v>
       </c>
       <c r="C144" s="48" t="s">
         <v>95</v>
@@ -27759,7 +27910,7 @@
     </row>
     <row r="145" spans="1:20" ht="15" customHeight="1">
       <c r="A145" s="42" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B145" s="42" t="s">
         <v>294</v>
@@ -27811,10 +27962,10 @@
     </row>
     <row r="146" spans="1:20" ht="15" customHeight="1">
       <c r="A146" s="48" t="s">
+        <v>708</v>
+      </c>
+      <c r="B146" s="48" t="s">
         <v>709</v>
-      </c>
-      <c r="B146" s="48" t="s">
-        <v>710</v>
       </c>
       <c r="C146" s="48" t="s">
         <v>95</v>
@@ -27848,7 +27999,7 @@
         <v>1522</v>
       </c>
       <c r="L146" s="48" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="M146" s="48"/>
       <c r="N146" s="48" t="s">
@@ -27863,10 +28014,10 @@
     </row>
     <row r="147" spans="1:20" ht="45" customHeight="1">
       <c r="A147" s="42" t="s">
+        <v>711</v>
+      </c>
+      <c r="B147" s="42" t="s">
         <v>712</v>
-      </c>
-      <c r="B147" s="42" t="s">
-        <v>713</v>
       </c>
       <c r="C147" s="42" t="s">
         <v>95</v>
@@ -27900,7 +28051,7 @@
         <v>5033</v>
       </c>
       <c r="L147" s="42" t="s">
-        <v>714</v>
+        <v>861</v>
       </c>
       <c r="M147" s="42"/>
       <c r="N147" s="42" t="s">
@@ -27908,7 +28059,7 @@
       </c>
       <c r="O147" s="42"/>
       <c r="P147" s="42" t="s">
-        <v>715</v>
+        <v>862</v>
       </c>
       <c r="Q147" s="42"/>
       <c r="R147" s="42"/>
@@ -27917,10 +28068,10 @@
     </row>
     <row r="148" spans="1:20" ht="15" customHeight="1">
       <c r="A148" s="48" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="B148" s="48" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="C148" s="48" t="s">
         <v>95</v>
@@ -27954,7 +28105,7 @@
         <v>502</v>
       </c>
       <c r="L148" s="48" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="M148" s="48"/>
       <c r="N148" s="48" t="s">
@@ -27969,10 +28120,10 @@
     </row>
     <row r="149" spans="1:20" ht="15" customHeight="1">
       <c r="A149" s="42" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
       <c r="B149" s="42" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="C149" s="42" t="s">
         <v>95</v>
@@ -28006,7 +28157,7 @@
         <v>1024</v>
       </c>
       <c r="L149" s="42" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
       <c r="M149" s="42"/>
       <c r="N149" s="42" t="s">
@@ -28021,10 +28172,10 @@
     </row>
     <row r="150" spans="1:20" ht="15" customHeight="1">
       <c r="A150" s="48" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
       <c r="B150" s="48" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="C150" s="48" t="s">
         <v>95</v>
@@ -28071,10 +28222,10 @@
     </row>
     <row r="151" spans="1:20" ht="15" customHeight="1">
       <c r="A151" s="42" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
       <c r="B151" s="42" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="C151" s="42" t="s">
         <v>96</v>
@@ -28108,7 +28259,7 @@
         <v>645</v>
       </c>
       <c r="L151" s="42" t="s">
-        <v>826</v>
+        <v>822</v>
       </c>
       <c r="M151" s="42"/>
       <c r="N151" s="42" t="s">
@@ -28118,7 +28269,7 @@
         <v>208</v>
       </c>
       <c r="P151" s="42" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="Q151" s="42"/>
       <c r="R151" s="42"/>
@@ -28127,10 +28278,10 @@
     </row>
     <row r="152" spans="1:20" ht="15" customHeight="1">
       <c r="A152" s="48" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="B152" s="48" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="C152" s="48" t="s">
         <v>97</v>
@@ -28164,17 +28315,17 @@
         <v>885</v>
       </c>
       <c r="L152" s="48" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="M152" s="48"/>
       <c r="N152" s="48" t="s">
         <v>451</v>
       </c>
       <c r="O152" s="48" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
       <c r="P152" s="48" t="s">
-        <v>731</v>
+        <v>728</v>
       </c>
       <c r="Q152" s="48"/>
       <c r="R152" s="48"/>
@@ -28183,10 +28334,10 @@
     </row>
     <row r="153" spans="1:20" ht="15" customHeight="1">
       <c r="A153" s="42" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
       <c r="B153" s="42" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="C153" s="42" t="s">
         <v>95</v>
@@ -28220,7 +28371,7 @@
         <v>891.5</v>
       </c>
       <c r="L153" s="42" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="M153" s="42"/>
       <c r="N153" s="42" t="s">
@@ -28228,7 +28379,7 @@
       </c>
       <c r="O153" s="42"/>
       <c r="P153" s="42" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
       <c r="Q153" s="42"/>
       <c r="R153" s="42"/>
@@ -28237,10 +28388,10 @@
     </row>
     <row r="154" spans="1:20" ht="15" customHeight="1">
       <c r="A154" s="48" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
       <c r="B154" s="48" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
       <c r="C154" s="48" t="s">
         <v>96</v>
@@ -28279,7 +28430,7 @@
         <v>538</v>
       </c>
       <c r="O154" s="48" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
       <c r="P154" s="48"/>
       <c r="Q154" s="48"/>
@@ -28289,10 +28440,10 @@
     </row>
     <row r="155" spans="1:20" ht="15" customHeight="1">
       <c r="A155" s="42" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
       <c r="B155" s="42" t="s">
-        <v>740</v>
+        <v>737</v>
       </c>
       <c r="C155" s="42" t="s">
         <v>96</v>
@@ -28331,7 +28482,7 @@
         <v>538</v>
       </c>
       <c r="O155" s="42" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
       <c r="P155" s="42"/>
       <c r="Q155" s="42"/>
@@ -28341,10 +28492,10 @@
     </row>
     <row r="156" spans="1:20" ht="15" customHeight="1">
       <c r="A156" s="48" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
       <c r="B156" s="48" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
       <c r="C156" s="48" t="s">
         <v>96</v>
@@ -28383,7 +28534,7 @@
         <v>538</v>
       </c>
       <c r="O156" s="48" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
       <c r="P156" s="48"/>
       <c r="Q156" s="48"/>
@@ -28393,10 +28544,10 @@
     </row>
     <row r="157" spans="1:20" ht="15" customHeight="1">
       <c r="A157" s="42" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
       <c r="B157" s="42" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="C157" s="42" t="s">
         <v>96</v>
@@ -28430,14 +28581,14 @@
         <v>1575</v>
       </c>
       <c r="L157" s="42" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
       <c r="M157" s="42"/>
       <c r="N157" s="42" t="s">
         <v>451</v>
       </c>
       <c r="O157" s="42" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="P157" s="42"/>
       <c r="Q157" s="42"/>
@@ -28447,10 +28598,10 @@
     </row>
     <row r="158" spans="1:20" ht="15" customHeight="1">
       <c r="A158" s="48" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="B158" s="48" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
       <c r="C158" s="48" t="s">
         <v>96</v>
@@ -28484,14 +28635,14 @@
         <v>3356</v>
       </c>
       <c r="L158" s="48" t="s">
-        <v>829</v>
+        <v>825</v>
       </c>
       <c r="M158" s="48"/>
       <c r="N158" s="48" t="s">
         <v>538</v>
       </c>
       <c r="O158" s="48" t="s">
-        <v>830</v>
+        <v>826</v>
       </c>
       <c r="P158" s="48"/>
       <c r="Q158" s="48"/>
@@ -28501,10 +28652,10 @@
     </row>
     <row r="159" spans="1:20" ht="15" customHeight="1">
       <c r="A159" s="42" t="s">
-        <v>749</v>
+        <v>746</v>
       </c>
       <c r="B159" s="42" t="s">
-        <v>750</v>
+        <v>747</v>
       </c>
       <c r="C159" s="42" t="s">
         <v>96</v>
@@ -28538,14 +28689,14 @@
         <v>3356</v>
       </c>
       <c r="L159" s="42" t="s">
-        <v>827</v>
+        <v>823</v>
       </c>
       <c r="M159" s="42"/>
       <c r="N159" s="42" t="s">
         <v>538</v>
       </c>
       <c r="O159" s="42" t="s">
-        <v>828</v>
+        <v>824</v>
       </c>
       <c r="P159" s="42"/>
       <c r="Q159" s="42"/>
@@ -28555,10 +28706,10 @@
     </row>
     <row r="160" spans="1:20" ht="15" customHeight="1">
       <c r="A160" s="48" t="s">
-        <v>751</v>
+        <v>748</v>
       </c>
       <c r="B160" s="48" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
       <c r="C160" s="48" t="s">
         <v>95</v>
@@ -28607,10 +28758,10 @@
     </row>
     <row r="161" spans="1:20" ht="15" customHeight="1">
       <c r="A161" s="42" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
       <c r="B161" s="42" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="C161" s="42" t="s">
         <v>95</v>
@@ -28659,10 +28810,10 @@
     </row>
     <row r="162" spans="1:20" ht="15" customHeight="1">
       <c r="A162" s="48" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="B162" s="48" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="C162" s="48" t="s">
         <v>95</v>
@@ -28709,10 +28860,10 @@
     </row>
     <row r="163" spans="1:20" ht="15" customHeight="1">
       <c r="A163" s="42" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="B163" s="42" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
       <c r="C163" s="42" t="s">
         <v>95</v>
@@ -28759,10 +28910,10 @@
     </row>
     <row r="164" spans="1:20" ht="60" customHeight="1">
       <c r="A164" s="48" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="B164" s="48" t="s">
-        <v>760</v>
+        <v>757</v>
       </c>
       <c r="C164" s="48" t="s">
         <v>95</v>
@@ -28802,7 +28953,7 @@
       </c>
       <c r="O164" s="48"/>
       <c r="P164" s="48" t="s">
-        <v>761</v>
+        <v>758</v>
       </c>
       <c r="Q164" s="48"/>
       <c r="R164" s="48"/>
@@ -28811,10 +28962,10 @@
     </row>
     <row r="165" spans="1:20" ht="15" customHeight="1">
       <c r="A165" s="42" t="s">
-        <v>762</v>
+        <v>759</v>
       </c>
       <c r="B165" s="42" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
       <c r="C165" s="42" t="s">
         <v>95</v>
@@ -28856,7 +29007,7 @@
       </c>
       <c r="O165" s="42"/>
       <c r="P165" s="42" t="s">
-        <v>764</v>
+        <v>761</v>
       </c>
       <c r="Q165" s="42"/>
       <c r="R165" s="42"/>
@@ -28865,10 +29016,10 @@
     </row>
     <row r="166" spans="1:20" ht="15" customHeight="1">
       <c r="A166" s="48" t="s">
-        <v>765</v>
+        <v>762</v>
       </c>
       <c r="B166" s="48" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
       <c r="C166" s="48" t="s">
         <v>95</v>
@@ -28908,7 +29059,7 @@
       </c>
       <c r="O166" s="48"/>
       <c r="P166" s="48" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
       <c r="Q166" s="48"/>
       <c r="R166" s="48"/>
@@ -28917,10 +29068,10 @@
     </row>
     <row r="167" spans="1:20" ht="15" customHeight="1">
       <c r="A167" s="42" t="s">
-        <v>768</v>
+        <v>765</v>
       </c>
       <c r="B167" s="42" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
       <c r="C167" s="42" t="s">
         <v>95</v>
@@ -28954,7 +29105,7 @@
         <v>2220</v>
       </c>
       <c r="L167" s="42" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
       <c r="M167" s="42"/>
       <c r="N167" s="42" t="s">
@@ -28962,7 +29113,7 @@
       </c>
       <c r="O167" s="42"/>
       <c r="P167" s="42" t="s">
-        <v>771</v>
+        <v>768</v>
       </c>
       <c r="Q167" s="42"/>
       <c r="R167" s="42"/>
@@ -28971,10 +29122,10 @@
     </row>
     <row r="168" spans="1:20" ht="15" customHeight="1">
       <c r="A168" s="48" t="s">
-        <v>772</v>
+        <v>769</v>
       </c>
       <c r="B168" s="48" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="C168" s="48" t="s">
         <v>95</v>
@@ -28983,13 +29134,13 @@
         <v>608</v>
       </c>
       <c r="E168" s="49">
-        <v>950</v>
+        <v>980</v>
       </c>
       <c r="F168" s="62">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G168" s="62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H168" s="61">
         <f t="shared" si="15"/>
@@ -29001,20 +29152,22 @@
       </c>
       <c r="J168" s="61">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>608</v>
       </c>
       <c r="K168" s="61">
         <f t="shared" si="17"/>
-        <v>1824</v>
-      </c>
-      <c r="L168" s="48"/>
+        <v>1216</v>
+      </c>
+      <c r="L168" s="48" t="s">
+        <v>857</v>
+      </c>
       <c r="M168" s="48"/>
       <c r="N168" s="48" t="s">
-        <v>538</v>
+        <v>451</v>
       </c>
       <c r="O168" s="48"/>
       <c r="P168" s="48" t="s">
-        <v>774</v>
+        <v>858</v>
       </c>
       <c r="Q168" s="48"/>
       <c r="R168" s="48"/>
@@ -29023,10 +29176,10 @@
     </row>
     <row r="169" spans="1:20" ht="15" customHeight="1">
       <c r="A169" s="42" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
       <c r="B169" s="42" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="C169" s="42" t="s">
         <v>95</v>
@@ -29066,7 +29219,7 @@
       </c>
       <c r="O169" s="42"/>
       <c r="P169" s="42" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="Q169" s="42"/>
       <c r="R169" s="42"/>
@@ -29075,10 +29228,10 @@
     </row>
     <row r="170" spans="1:20" ht="30" customHeight="1">
       <c r="A170" s="48" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="B170" s="48" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="C170" s="48" t="s">
         <v>95</v>
@@ -29112,7 +29265,7 @@
         <v>0</v>
       </c>
       <c r="L170" s="48" t="s">
-        <v>819</v>
+        <v>815</v>
       </c>
       <c r="M170" s="48"/>
       <c r="N170" s="48" t="s">
@@ -29120,7 +29273,7 @@
       </c>
       <c r="O170" s="48"/>
       <c r="P170" s="48" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="Q170" s="48"/>
       <c r="R170" s="48"/>
@@ -29129,10 +29282,10 @@
     </row>
     <row r="171" spans="1:20" ht="32" customHeight="1">
       <c r="A171" s="42" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="B171" s="48" t="s">
-        <v>782</v>
+        <v>778</v>
       </c>
       <c r="C171" s="42" t="s">
         <v>95</v>
@@ -29144,10 +29297,10 @@
         <v>1380</v>
       </c>
       <c r="F171" s="60">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G171" s="60">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H171" s="59">
         <f t="shared" si="15"/>
@@ -29159,23 +29312,21 @@
       </c>
       <c r="J171" s="59">
         <f t="shared" si="16"/>
-        <v>892</v>
+        <v>2676</v>
       </c>
       <c r="K171" s="59">
         <f t="shared" si="17"/>
-        <v>1784</v>
+        <v>0</v>
       </c>
       <c r="L171" s="42" t="s">
-        <v>848</v>
+        <v>855</v>
       </c>
       <c r="M171" s="42"/>
       <c r="N171" s="42" t="s">
-        <v>451</v>
+        <v>366</v>
       </c>
       <c r="O171" s="42"/>
-      <c r="P171" s="42" t="s">
-        <v>845</v>
-      </c>
+      <c r="P171" s="42"/>
       <c r="Q171" s="42"/>
       <c r="R171" s="42"/>
       <c r="S171" s="42"/>
@@ -29183,10 +29334,10 @@
     </row>
     <row r="172" spans="1:20" ht="15" customHeight="1">
       <c r="A172" s="48" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="B172" s="48" t="s">
-        <v>784</v>
+        <v>780</v>
       </c>
       <c r="C172" s="48" t="s">
         <v>95</v>
@@ -29233,10 +29384,10 @@
     </row>
     <row r="173" spans="1:20" ht="15" customHeight="1">
       <c r="A173" s="42" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
       <c r="B173" s="42" t="s">
-        <v>786</v>
+        <v>782</v>
       </c>
       <c r="C173" s="42" t="s">
         <v>95</v>
@@ -29283,10 +29434,10 @@
     </row>
     <row r="174" spans="1:20" ht="15" customHeight="1">
       <c r="A174" s="48" t="s">
-        <v>787</v>
+        <v>783</v>
       </c>
       <c r="B174" s="48" t="s">
-        <v>788</v>
+        <v>784</v>
       </c>
       <c r="C174" s="48" t="s">
         <v>95</v>
@@ -29333,10 +29484,10 @@
     </row>
     <row r="175" spans="1:20" ht="90" customHeight="1">
       <c r="A175" s="42" t="s">
-        <v>789</v>
+        <v>785</v>
       </c>
       <c r="B175" s="42" t="s">
-        <v>790</v>
+        <v>786</v>
       </c>
       <c r="C175" s="42" t="s">
         <v>95</v>
@@ -29348,10 +29499,10 @@
         <v>1250</v>
       </c>
       <c r="F175" s="60">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G175" s="60">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H175" s="59">
         <f t="shared" si="15"/>
@@ -29363,14 +29514,14 @@
       </c>
       <c r="J175" s="59">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>698.25</v>
       </c>
       <c r="K175" s="59">
         <f t="shared" si="17"/>
-        <v>6982.5</v>
+        <v>6284.25</v>
       </c>
       <c r="L175" s="42" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="M175" s="42"/>
       <c r="N175" s="42" t="s">
@@ -29378,147 +29529,329 @@
       </c>
       <c r="O175" s="42"/>
       <c r="P175" s="42" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="Q175" s="42"/>
       <c r="R175" s="42"/>
       <c r="S175" s="42"/>
       <c r="T175" s="42"/>
     </row>
-    <row r="176" spans="1:20">
-      <c r="A176" s="48"/>
-      <c r="B176" s="48"/>
-      <c r="C176" s="48"/>
-      <c r="D176" s="49"/>
-      <c r="E176" s="49"/>
-      <c r="F176" s="62"/>
-      <c r="G176" s="62"/>
-      <c r="H176" s="61"/>
-      <c r="I176" s="61"/>
-      <c r="J176" s="61"/>
-      <c r="K176" s="61"/>
+    <row r="176" spans="1:20" ht="15">
+      <c r="A176" s="48" t="s">
+        <v>871</v>
+      </c>
+      <c r="B176" s="48" t="s">
+        <v>869</v>
+      </c>
+      <c r="C176" s="48" t="s">
+        <v>95</v>
+      </c>
+      <c r="D176" s="49">
+        <v>908</v>
+      </c>
+      <c r="E176" s="49">
+        <v>1350</v>
+      </c>
+      <c r="F176" s="62">
+        <v>0</v>
+      </c>
+      <c r="G176" s="62">
+        <v>4</v>
+      </c>
+      <c r="H176" s="61">
+        <f t="shared" ref="H176:H188" si="18">F176+IF(LEN(G176)=0,0,G176)</f>
+        <v>4</v>
+      </c>
+      <c r="I176" s="61">
+        <f>IF(D176&lt;&gt;"",D176,IFERROR(E176/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
+        <v>908</v>
+      </c>
+      <c r="J176" s="61">
+        <f t="shared" ref="J176:J188" si="19">F176*I176</f>
+        <v>0</v>
+      </c>
+      <c r="K176" s="61">
+        <f t="shared" ref="K176:K188" si="20">IF(LEN(G176)=0,0,G176)*I176</f>
+        <v>3632</v>
+      </c>
       <c r="L176" s="48"/>
       <c r="M176" s="48"/>
-      <c r="N176" s="48"/>
+      <c r="N176" s="48" t="s">
+        <v>538</v>
+      </c>
       <c r="O176" s="48"/>
-      <c r="P176" s="48"/>
+      <c r="P176" s="48" t="s">
+        <v>870</v>
+      </c>
       <c r="Q176" s="48"/>
       <c r="R176" s="48"/>
       <c r="S176" s="48"/>
       <c r="T176" s="48"/>
     </row>
-    <row r="177" spans="1:20">
-      <c r="A177" s="42"/>
-      <c r="B177" s="42"/>
-      <c r="C177" s="42"/>
-      <c r="D177" s="51"/>
-      <c r="E177" s="51"/>
-      <c r="F177" s="60"/>
-      <c r="G177" s="60"/>
-      <c r="H177" s="59"/>
-      <c r="I177" s="59"/>
-      <c r="J177" s="59"/>
-      <c r="K177" s="59"/>
+    <row r="177" spans="1:20" ht="30">
+      <c r="A177" s="42" t="s">
+        <v>874</v>
+      </c>
+      <c r="B177" s="42" t="s">
+        <v>872</v>
+      </c>
+      <c r="C177" s="42" t="s">
+        <v>95</v>
+      </c>
+      <c r="D177" s="51">
+        <v>906</v>
+      </c>
+      <c r="E177" s="51">
+        <v>1350</v>
+      </c>
+      <c r="F177" s="60">
+        <v>0</v>
+      </c>
+      <c r="G177" s="60">
+        <v>5</v>
+      </c>
+      <c r="H177" s="59">
+        <f t="shared" si="18"/>
+        <v>5</v>
+      </c>
+      <c r="I177" s="59">
+        <f>IF(D177&lt;&gt;"",D177,IFERROR(E177/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
+        <v>906</v>
+      </c>
+      <c r="J177" s="59">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="K177" s="59">
+        <f t="shared" si="20"/>
+        <v>4530</v>
+      </c>
       <c r="L177" s="42"/>
       <c r="M177" s="42"/>
-      <c r="N177" s="42"/>
+      <c r="N177" s="42" t="s">
+        <v>538</v>
+      </c>
       <c r="O177" s="42"/>
-      <c r="P177" s="42"/>
+      <c r="P177" s="42" t="s">
+        <v>873</v>
+      </c>
       <c r="Q177" s="42"/>
       <c r="R177" s="42"/>
       <c r="S177" s="42"/>
       <c r="T177" s="42"/>
     </row>
-    <row r="178" spans="1:20">
-      <c r="A178" s="48"/>
-      <c r="B178" s="48"/>
-      <c r="C178" s="48"/>
-      <c r="D178" s="49"/>
-      <c r="E178" s="49"/>
-      <c r="F178" s="62"/>
-      <c r="G178" s="62"/>
-      <c r="H178" s="61"/>
-      <c r="I178" s="61"/>
-      <c r="J178" s="61"/>
-      <c r="K178" s="61"/>
+    <row r="178" spans="1:20" ht="15">
+      <c r="A178" s="48" t="s">
+        <v>875</v>
+      </c>
+      <c r="B178" s="48" t="s">
+        <v>886</v>
+      </c>
+      <c r="C178" s="48" t="s">
+        <v>95</v>
+      </c>
+      <c r="D178" s="49">
+        <v>938</v>
+      </c>
+      <c r="E178" s="49">
+        <v>1400</v>
+      </c>
+      <c r="F178" s="62">
+        <v>0</v>
+      </c>
+      <c r="G178" s="62">
+        <v>2</v>
+      </c>
+      <c r="H178" s="61">
+        <f t="shared" si="18"/>
+        <v>2</v>
+      </c>
+      <c r="I178" s="61">
+        <f>IF(D178&lt;&gt;"",D178,IFERROR(E178/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
+        <v>938</v>
+      </c>
+      <c r="J178" s="61">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="K178" s="61">
+        <f t="shared" si="20"/>
+        <v>1876</v>
+      </c>
       <c r="L178" s="48"/>
       <c r="M178" s="48"/>
-      <c r="N178" s="48"/>
+      <c r="N178" s="48" t="s">
+        <v>538</v>
+      </c>
       <c r="O178" s="48"/>
-      <c r="P178" s="48"/>
+      <c r="P178" s="48" t="s">
+        <v>887</v>
+      </c>
       <c r="Q178" s="48"/>
       <c r="R178" s="48"/>
       <c r="S178" s="48"/>
       <c r="T178" s="48"/>
     </row>
-    <row r="179" spans="1:20">
-      <c r="A179" s="42"/>
-      <c r="B179" s="42"/>
-      <c r="C179" s="42"/>
-      <c r="D179" s="51"/>
-      <c r="E179" s="51"/>
-      <c r="F179" s="60"/>
-      <c r="G179" s="60"/>
-      <c r="H179" s="59"/>
-      <c r="I179" s="59"/>
-      <c r="J179" s="59"/>
-      <c r="K179" s="59"/>
+    <row r="179" spans="1:20" ht="15">
+      <c r="A179" s="42" t="s">
+        <v>876</v>
+      </c>
+      <c r="B179" s="42" t="s">
+        <v>888</v>
+      </c>
+      <c r="C179" s="42" t="s">
+        <v>95</v>
+      </c>
+      <c r="D179" s="51">
+        <v>919</v>
+      </c>
+      <c r="E179" s="51">
+        <v>1350</v>
+      </c>
+      <c r="F179" s="60">
+        <v>0</v>
+      </c>
+      <c r="G179" s="60">
+        <v>3</v>
+      </c>
+      <c r="H179" s="59">
+        <f t="shared" si="18"/>
+        <v>3</v>
+      </c>
+      <c r="I179" s="59">
+        <f>IF(D179&lt;&gt;"",D179,IFERROR(E179/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
+        <v>919</v>
+      </c>
+      <c r="J179" s="59">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="K179" s="59">
+        <f t="shared" si="20"/>
+        <v>2757</v>
+      </c>
       <c r="L179" s="42"/>
       <c r="M179" s="42"/>
-      <c r="N179" s="42"/>
+      <c r="N179" s="42" t="s">
+        <v>538</v>
+      </c>
       <c r="O179" s="42"/>
-      <c r="P179" s="42"/>
+      <c r="P179" s="42" t="s">
+        <v>889</v>
+      </c>
       <c r="Q179" s="42"/>
       <c r="R179" s="42"/>
       <c r="S179" s="42"/>
       <c r="T179" s="42"/>
     </row>
-    <row r="180" spans="1:20">
-      <c r="A180" s="48"/>
-      <c r="B180" s="48"/>
-      <c r="C180" s="48"/>
-      <c r="D180" s="49"/>
-      <c r="E180" s="49"/>
-      <c r="F180" s="62"/>
-      <c r="G180" s="62"/>
-      <c r="H180" s="61"/>
-      <c r="I180" s="61"/>
-      <c r="J180" s="61"/>
-      <c r="K180" s="61"/>
+    <row r="180" spans="1:20" ht="30">
+      <c r="A180" s="48" t="s">
+        <v>877</v>
+      </c>
+      <c r="B180" s="48" t="s">
+        <v>890</v>
+      </c>
+      <c r="C180" s="48" t="s">
+        <v>95</v>
+      </c>
+      <c r="D180" s="49">
+        <v>919</v>
+      </c>
+      <c r="E180" s="49">
+        <v>1380</v>
+      </c>
+      <c r="F180" s="62">
+        <v>0</v>
+      </c>
+      <c r="G180" s="62">
+        <v>3</v>
+      </c>
+      <c r="H180" s="61">
+        <f t="shared" si="18"/>
+        <v>3</v>
+      </c>
+      <c r="I180" s="61">
+        <f>IF(D180&lt;&gt;"",D180,IFERROR(E180/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
+        <v>919</v>
+      </c>
+      <c r="J180" s="61">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="K180" s="61">
+        <f t="shared" si="20"/>
+        <v>2757</v>
+      </c>
       <c r="L180" s="48"/>
       <c r="M180" s="48"/>
-      <c r="N180" s="48"/>
+      <c r="N180" s="48" t="s">
+        <v>538</v>
+      </c>
       <c r="O180" s="48"/>
-      <c r="P180" s="48"/>
+      <c r="P180" s="48" t="s">
+        <v>891</v>
+      </c>
       <c r="Q180" s="48"/>
       <c r="R180" s="48"/>
       <c r="S180" s="48"/>
       <c r="T180" s="48"/>
     </row>
-    <row r="181" spans="1:20">
-      <c r="A181" s="42"/>
-      <c r="B181" s="42"/>
-      <c r="C181" s="42"/>
-      <c r="D181" s="51"/>
-      <c r="E181" s="51"/>
-      <c r="F181" s="60"/>
-      <c r="G181" s="60"/>
-      <c r="H181" s="59"/>
-      <c r="I181" s="59"/>
-      <c r="J181" s="59"/>
-      <c r="K181" s="59"/>
+    <row r="181" spans="1:20" ht="30">
+      <c r="A181" s="42" t="s">
+        <v>878</v>
+      </c>
+      <c r="B181" s="42" t="s">
+        <v>892</v>
+      </c>
+      <c r="C181" s="42" t="s">
+        <v>95</v>
+      </c>
+      <c r="D181" s="51">
+        <v>992</v>
+      </c>
+      <c r="E181" s="51">
+        <v>1450</v>
+      </c>
+      <c r="F181" s="60">
+        <v>0</v>
+      </c>
+      <c r="G181" s="60">
+        <v>5</v>
+      </c>
+      <c r="H181" s="59">
+        <f t="shared" si="18"/>
+        <v>5</v>
+      </c>
+      <c r="I181" s="59">
+        <f>IF(D181&lt;&gt;"",D181,IFERROR(E181/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
+        <v>992</v>
+      </c>
+      <c r="J181" s="59">
+        <f t="shared" ref="J181" si="21">F181*I181</f>
+        <v>0</v>
+      </c>
+      <c r="K181" s="59">
+        <f t="shared" ref="K181" si="22">IF(LEN(G181)=0,0,G181)*I181</f>
+        <v>4960</v>
+      </c>
       <c r="L181" s="42"/>
       <c r="M181" s="42"/>
-      <c r="N181" s="42"/>
+      <c r="N181" s="42" t="s">
+        <v>538</v>
+      </c>
       <c r="O181" s="42"/>
-      <c r="P181" s="42"/>
+      <c r="P181" s="42" t="s">
+        <v>893</v>
+      </c>
       <c r="Q181" s="42"/>
       <c r="R181" s="42"/>
       <c r="S181" s="42"/>
       <c r="T181" s="42"/>
     </row>
-    <row r="182" spans="1:20">
-      <c r="A182" s="48"/>
+    <row r="182" spans="1:20" ht="15">
+      <c r="A182" s="48" t="s">
+        <v>879</v>
+      </c>
       <c r="B182" s="48"/>
       <c r="C182" s="48"/>
       <c r="D182" s="49"/>
@@ -29539,8 +29872,10 @@
       <c r="S182" s="48"/>
       <c r="T182" s="48"/>
     </row>
-    <row r="183" spans="1:20">
-      <c r="A183" s="42"/>
+    <row r="183" spans="1:20" ht="15">
+      <c r="A183" s="42" t="s">
+        <v>880</v>
+      </c>
       <c r="B183" s="42"/>
       <c r="C183" s="42"/>
       <c r="D183" s="51"/>
@@ -29561,8 +29896,10 @@
       <c r="S183" s="42"/>
       <c r="T183" s="42"/>
     </row>
-    <row r="184" spans="1:20">
-      <c r="A184" s="48"/>
+    <row r="184" spans="1:20" ht="15">
+      <c r="A184" s="48" t="s">
+        <v>881</v>
+      </c>
       <c r="B184" s="48"/>
       <c r="C184" s="48"/>
       <c r="D184" s="49"/>
@@ -29583,8 +29920,10 @@
       <c r="S184" s="48"/>
       <c r="T184" s="48"/>
     </row>
-    <row r="185" spans="1:20">
-      <c r="A185" s="42"/>
+    <row r="185" spans="1:20" ht="15">
+      <c r="A185" s="42" t="s">
+        <v>882</v>
+      </c>
       <c r="B185" s="42"/>
       <c r="C185" s="42"/>
       <c r="D185" s="51"/>
@@ -29605,8 +29944,10 @@
       <c r="S185" s="42"/>
       <c r="T185" s="42"/>
     </row>
-    <row r="186" spans="1:20">
-      <c r="A186" s="48"/>
+    <row r="186" spans="1:20" ht="15">
+      <c r="A186" s="48" t="s">
+        <v>883</v>
+      </c>
       <c r="B186" s="48"/>
       <c r="C186" s="48"/>
       <c r="D186" s="49"/>
@@ -29627,8 +29968,10 @@
       <c r="S186" s="48"/>
       <c r="T186" s="48"/>
     </row>
-    <row r="187" spans="1:20">
-      <c r="A187" s="42"/>
+    <row r="187" spans="1:20" ht="15">
+      <c r="A187" s="42" t="s">
+        <v>884</v>
+      </c>
       <c r="B187" s="42"/>
       <c r="C187" s="42"/>
       <c r="D187" s="51"/>
@@ -29649,8 +29992,10 @@
       <c r="S187" s="42"/>
       <c r="T187" s="42"/>
     </row>
-    <row r="188" spans="1:20">
-      <c r="A188" s="48"/>
+    <row r="188" spans="1:20" ht="15">
+      <c r="A188" s="48" t="s">
+        <v>885</v>
+      </c>
       <c r="B188" s="48"/>
       <c r="C188" s="48"/>
       <c r="D188" s="49"/>
@@ -33694,6 +34039,7 @@
       <c r="T1189" s="43"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N988" xr:uid="{00000000-0002-0000-0500-000000000000}">
       <formula1>"Pending,Partially Sold,Sold Out,New,Reserved"</formula1>
@@ -33723,7 +34069,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1">
       <c r="A1" s="95" t="s">
-        <v>791</v>
+        <v>787</v>
       </c>
       <c r="B1" s="95"/>
     </row>
@@ -33732,7 +34078,7 @@
         <v>42</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>792</v>
+        <v>788</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="13.5" customHeight="1">
@@ -33764,25 +34110,25 @@
         <v>42</v>
       </c>
       <c r="B7" s="67" t="s">
+        <v>789</v>
+      </c>
+      <c r="C7" s="67" t="s">
+        <v>790</v>
+      </c>
+      <c r="D7" s="67" t="s">
+        <v>791</v>
+      </c>
+      <c r="E7" s="67" t="s">
+        <v>792</v>
+      </c>
+      <c r="F7" s="67" t="s">
         <v>793</v>
       </c>
-      <c r="C7" s="67" t="s">
+      <c r="G7" s="67" t="s">
         <v>794</v>
       </c>
-      <c r="D7" s="67" t="s">
+      <c r="H7" s="67" t="s">
         <v>795</v>
-      </c>
-      <c r="E7" s="67" t="s">
-        <v>796</v>
-      </c>
-      <c r="F7" s="67" t="s">
-        <v>797</v>
-      </c>
-      <c r="G7" s="67" t="s">
-        <v>798</v>
-      </c>
-      <c r="H7" s="67" t="s">
-        <v>799</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="13.5" customHeight="1">
@@ -33791,15 +34137,15 @@
       </c>
       <c r="B8" s="9">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A8,Purchases!$C:$C),0)</f>
-        <v>126918</v>
+        <v>152100</v>
       </c>
       <c r="C8" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>106317</v>
+        <v>114711</v>
       </c>
       <c r="D8" s="9">
         <f>B8-C8</f>
-        <v>20601</v>
+        <v>37389</v>
       </c>
       <c r="E8" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE()),0)</f>
@@ -33807,7 +34153,7 @@
       </c>
       <c r="F8" s="9">
         <f>D8+E8</f>
-        <v>20601</v>
+        <v>37389</v>
       </c>
       <c r="G8" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -33815,7 +34161,7 @@
       </c>
       <c r="H8" s="69">
         <f>F8-G8</f>
-        <v>2297.66</v>
+        <v>19085.66</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="13.5" customHeight="1">
@@ -33828,11 +34174,11 @@
       </c>
       <c r="C9" s="11">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>106317</v>
+        <v>114711</v>
       </c>
       <c r="D9" s="11">
         <f>B9-C9</f>
-        <v>53116</v>
+        <v>44722</v>
       </c>
       <c r="E9" s="11">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE()),0)</f>
@@ -33840,7 +34186,7 @@
       </c>
       <c r="F9" s="11">
         <f>D9+E9</f>
-        <v>53116</v>
+        <v>44722</v>
       </c>
       <c r="G9" s="11">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -33848,7 +34194,7 @@
       </c>
       <c r="H9" s="70">
         <f>F9-G9</f>
-        <v>11476.669999999998</v>
+        <v>3082.6699999999983</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="13.5" customHeight="1">
@@ -33861,11 +34207,11 @@
       </c>
       <c r="C10" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>106317</v>
+        <v>114711</v>
       </c>
       <c r="D10" s="9">
         <f>B10-C10</f>
-        <v>-73717</v>
+        <v>-82111</v>
       </c>
       <c r="E10" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE()),0)</f>
@@ -33873,7 +34219,7 @@
       </c>
       <c r="F10" s="9">
         <f>D10+E10</f>
-        <v>-73717</v>
+        <v>-82111</v>
       </c>
       <c r="G10" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -33881,12 +34227,12 @@
       </c>
       <c r="H10" s="69">
         <f>F10-G10</f>
-        <v>-13774.330000000002</v>
+        <v>-22168.33</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="71" customFormat="1" ht="15.75" customHeight="1">
       <c r="A12" s="96" t="s">
-        <v>800</v>
+        <v>796</v>
       </c>
       <c r="B12" s="96"/>
       <c r="C12" s="96"/>
@@ -33899,13 +34245,13 @@
         <v>98</v>
       </c>
       <c r="B13" s="67" t="s">
-        <v>801</v>
+        <v>797</v>
       </c>
       <c r="C13" s="67" t="s">
-        <v>802</v>
+        <v>798</v>
       </c>
       <c r="D13" s="67" t="s">
-        <v>803</v>
+        <v>799</v>
       </c>
       <c r="E13" s="67" t="s">
         <v>99</v>
@@ -33919,7 +34265,7 @@
         <v>45952</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>804</v>
+        <v>800</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>51</v>
@@ -33937,7 +34283,7 @@
         <v>45952</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>804</v>
+        <v>800</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>51</v>
@@ -33991,7 +34337,7 @@
         <v>45970</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>804</v>
+        <v>800</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>50</v>
@@ -34009,7 +34355,7 @@
         <v>45970</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>804</v>
+        <v>800</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>50</v>
@@ -34027,7 +34373,7 @@
         <v>45973</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>804</v>
+        <v>800</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>50</v>
@@ -34045,7 +34391,7 @@
         <v>45973</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>804</v>
+        <v>800</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>49</v>
@@ -34063,7 +34409,7 @@
         <v>46058</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>804</v>
+        <v>800</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>51</v>
@@ -34099,7 +34445,7 @@
         <v>46059</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>804</v>
+        <v>800</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>49</v>
@@ -34135,7 +34481,7 @@
         <v>46093</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>804</v>
+        <v>800</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>50</v>
@@ -34153,7 +34499,7 @@
         <v>46093</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>804</v>
+        <v>800</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>51</v>
@@ -34236,7 +34582,7 @@
     </row>
     <row r="58" spans="2:2" ht="13.5" customHeight="1">
       <c r="B58" s="6" t="s">
-        <v>805</v>
+        <v>801</v>
       </c>
     </row>
   </sheetData>
@@ -34266,7 +34612,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="13.5" customHeight="1">
       <c r="A1" s="74" t="s">
-        <v>806</v>
+        <v>802</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="68" customFormat="1" ht="13.5" customHeight="1">
@@ -34274,22 +34620,22 @@
         <v>42</v>
       </c>
       <c r="B3" s="67" t="s">
+        <v>803</v>
+      </c>
+      <c r="C3" s="67" t="s">
+        <v>788</v>
+      </c>
+      <c r="D3" s="67" t="s">
+        <v>804</v>
+      </c>
+      <c r="E3" s="67" t="s">
+        <v>805</v>
+      </c>
+      <c r="F3" s="67" t="s">
+        <v>806</v>
+      </c>
+      <c r="G3" s="67" t="s">
         <v>807</v>
-      </c>
-      <c r="C3" s="67" t="s">
-        <v>792</v>
-      </c>
-      <c r="D3" s="67" t="s">
-        <v>808</v>
-      </c>
-      <c r="E3" s="67" t="s">
-        <v>809</v>
-      </c>
-      <c r="F3" s="67" t="s">
-        <v>810</v>
-      </c>
-      <c r="G3" s="67" t="s">
-        <v>811</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="13.5" customHeight="1">
@@ -34298,7 +34644,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>261011</v>
+        <v>265071</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -34306,11 +34652,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>94005.463999999993</v>
+        <v>95359.067999999999</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>167005.53600000002</v>
+        <v>169711.932</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -34318,7 +34664,7 @@
       </c>
       <c r="G4" s="69">
         <f>E4+F4</f>
-        <v>29695.510000000009</v>
+        <v>32401.905999999988</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -34335,11 +34681,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>93949.072</v>
+        <v>95301.864000000001</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-85530.072</v>
+        <v>-86882.864000000001</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -34347,7 +34693,7 @@
       </c>
       <c r="G5" s="70">
         <f>E5+F5</f>
-        <v>-13943.029999999999</v>
+        <v>-15295.822</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -34364,11 +34710,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>94005.463999999993</v>
+        <v>95359.067999999999</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-81475.463999999993</v>
+        <v>-82829.067999999999</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -34376,7 +34722,7 @@
       </c>
       <c r="G6" s="69">
         <f>E6+F6</f>
-        <v>-15752.479999999981</v>
+        <v>-17106.083999999988</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">
@@ -34386,27 +34732,27 @@
     </row>
     <row r="10" spans="1:7" ht="13.5" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>812</v>
+        <v>808</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="13.5" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>813</v>
+        <v>809</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="13.5" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="13.5" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>815</v>
+        <v>811</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="13.5" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>816</v>
+        <v>812</v>
       </c>
     </row>
   </sheetData>

</xml_diff>